<commit_message>
표 업뎃, job queue
</commit_message>
<xml_diff>
--- a/results/converted_results.xlsx
+++ b/results/converted_results.xlsx
@@ -296,6 +296,13 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="P53" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Gopher, seed 6010
+STORM-1/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
     <comment ref="T53" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9999
@@ -310,6 +317,13 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="P54" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Gopher, seed 6010
+STORM-1/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
     <comment ref="T54" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9999
@@ -320,6 +334,13 @@
     <comment ref="O55" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 6000
+STORM-1/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="P55" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Gopher, seed 6010
 STORM-1/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
@@ -3212,7 +3233,7 @@
           <t>2486.00</t>
         </is>
       </c>
-      <c r="P53" s="8" t="inlineStr">
+      <c r="P53" s="12" t="inlineStr">
         <is>
           <t>1250.00</t>
         </is>
@@ -3256,7 +3277,7 @@
       <c r="M54" s="8" t="inlineStr"/>
       <c r="N54" s="8" t="inlineStr"/>
       <c r="O54" s="12" t="inlineStr"/>
-      <c r="P54" s="8" t="inlineStr"/>
+      <c r="P54" s="12" t="inlineStr"/>
       <c r="Q54" s="8" t="inlineStr"/>
       <c r="R54" s="13" t="inlineStr">
         <is>
@@ -3302,7 +3323,7 @@
           <t>1024.00</t>
         </is>
       </c>
-      <c r="P55" s="8" t="inlineStr">
+      <c r="P55" s="12" t="inlineStr">
         <is>
           <t>927.00</t>
         </is>

</xml_diff>

<commit_message>
job queue와 schedule_experimemts 수정
</commit_message>
<xml_diff>
--- a/results/converted_results.xlsx
+++ b/results/converted_results.xlsx
@@ -175,10 +175,10 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -283,6 +283,111 @@
 모든 평균은 EXCLUDED_SEEDS를 제외한 공통 시드 기준이며 HNS 차이는 부호를 유지합니다. 백분율이 아닙니다.</t>
       </text>
     </comment>
+    <comment ref="N3" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Alien, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N4" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Alien, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N5" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Alien, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N6" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Alien, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N7" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Alien, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N9" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Amidar, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N10" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Amidar, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N11" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Amidar, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N12" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Amidar, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="N13" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Amidar, seed 5090
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="L15" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Assault, seed 2010
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="L16" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Assault, seed 2010
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="L17" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Assault, seed 2010
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="L18" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Assault, seed 2010
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="L19" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: Assault, seed 2010
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
     <comment ref="Q27" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: BankHeist, seed 6020
@@ -354,6 +459,13 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="K33" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: BattleZone, seed 2000
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
     <comment ref="P33" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: BattleZone, seed 6010
@@ -361,6 +473,13 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="K34" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: BattleZone, seed 2000
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
     <comment ref="P34" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: BattleZone, seed 6010
@@ -368,6 +487,13 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="K35" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: BattleZone, seed 2000
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
     <comment ref="P35" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: BattleZone, seed 6010
@@ -375,9 +501,23 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="K36" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: BattleZone, seed 2000
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
     <comment ref="P36" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: BattleZone, seed 6010
+STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
+취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="K37" authorId="0" shapeId="0">
+      <text>
+        <t>EXCLUDED_SEEDS: BattleZone, seed 2000
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
@@ -1382,10 +1522,10 @@
       <c r="Y2" s="4" t="inlineStr"/>
       <c r="Z2" s="5" t="inlineStr"/>
       <c r="AA2" s="6" t="n">
-        <v>57.79999999999995</v>
+        <v>107.625</v>
       </c>
       <c r="AB2" s="7" t="n">
-        <v>0.008376932999028966</v>
+        <v>0.01559805214568327</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
@@ -1418,7 +1558,7 @@
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr"/>
-      <c r="N3" s="8" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>842.50</t>
         </is>
@@ -1442,11 +1582,11 @@
       <c r="W3" s="8" t="inlineStr"/>
       <c r="X3" s="8" t="inlineStr"/>
       <c r="Y3" s="8" t="inlineStr"/>
-      <c r="Z3" s="9" t="n">
-        <v>1041.8</v>
-      </c>
-      <c r="AA3" s="10" t="inlineStr"/>
-      <c r="AB3" s="11" t="inlineStr"/>
+      <c r="Z3" s="10" t="n">
+        <v>1091.625</v>
+      </c>
+      <c r="AA3" s="11" t="inlineStr"/>
+      <c r="AB3" s="12" t="inlineStr"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="1" t="n"/>
@@ -1474,7 +1614,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr"/>
       <c r="M4" s="8" t="inlineStr"/>
-      <c r="N4" s="8" t="inlineStr"/>
+      <c r="N4" s="9" t="inlineStr"/>
       <c r="O4" s="8" t="inlineStr">
         <is>
           <t>1303.50</t>
@@ -1494,9 +1634,9 @@
       <c r="W4" s="8" t="inlineStr"/>
       <c r="X4" s="8" t="inlineStr"/>
       <c r="Y4" s="8" t="inlineStr"/>
-      <c r="Z4" s="9" t="inlineStr"/>
-      <c r="AA4" s="10" t="inlineStr"/>
-      <c r="AB4" s="11" t="inlineStr"/>
+      <c r="Z4" s="10" t="inlineStr"/>
+      <c r="AA4" s="11" t="inlineStr"/>
+      <c r="AB4" s="12" t="inlineStr"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="1" t="n"/>
@@ -1524,7 +1664,7 @@
       </c>
       <c r="L5" s="8" t="inlineStr"/>
       <c r="M5" s="8" t="inlineStr"/>
-      <c r="N5" s="8" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
         <is>
           <t>864.00</t>
         </is>
@@ -1548,14 +1688,14 @@
       <c r="W5" s="8" t="inlineStr"/>
       <c r="X5" s="8" t="inlineStr"/>
       <c r="Y5" s="8" t="inlineStr"/>
-      <c r="Z5" s="9" t="n">
-        <v>1091.1</v>
-      </c>
-      <c r="AA5" s="9" t="n">
-        <v>49.29999999999995</v>
-      </c>
-      <c r="AB5" s="11" t="n">
-        <v>0.007145031087407058</v>
+      <c r="Z5" s="10" t="n">
+        <v>1147.875</v>
+      </c>
+      <c r="AA5" s="10" t="n">
+        <v>56.25</v>
+      </c>
+      <c r="AB5" s="12" t="n">
+        <v>0.0081522920622038</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
@@ -1580,7 +1720,7 @@
       </c>
       <c r="L6" s="8" t="inlineStr"/>
       <c r="M6" s="8" t="inlineStr"/>
-      <c r="N6" s="8" t="inlineStr"/>
+      <c r="N6" s="9" t="inlineStr"/>
       <c r="O6" s="8" t="inlineStr"/>
       <c r="P6" s="8" t="inlineStr"/>
       <c r="Q6" s="8" t="inlineStr"/>
@@ -1592,9 +1732,9 @@
       <c r="W6" s="8" t="inlineStr"/>
       <c r="X6" s="8" t="inlineStr"/>
       <c r="Y6" s="8" t="inlineStr"/>
-      <c r="Z6" s="9" t="inlineStr"/>
-      <c r="AA6" s="10" t="inlineStr"/>
-      <c r="AB6" s="11" t="inlineStr"/>
+      <c r="Z6" s="10" t="inlineStr"/>
+      <c r="AA6" s="11" t="inlineStr"/>
+      <c r="AB6" s="12" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="1" t="n"/>
@@ -1618,7 +1758,7 @@
       </c>
       <c r="L7" s="8" t="inlineStr"/>
       <c r="M7" s="8" t="inlineStr"/>
-      <c r="N7" s="8" t="inlineStr"/>
+      <c r="N7" s="9" t="inlineStr"/>
       <c r="O7" s="8" t="inlineStr"/>
       <c r="P7" s="8" t="inlineStr"/>
       <c r="Q7" s="8" t="inlineStr"/>
@@ -1630,9 +1770,9 @@
       <c r="W7" s="8" t="inlineStr"/>
       <c r="X7" s="8" t="inlineStr"/>
       <c r="Y7" s="8" t="inlineStr"/>
-      <c r="Z7" s="9" t="inlineStr"/>
-      <c r="AA7" s="10" t="inlineStr"/>
-      <c r="AB7" s="11" t="inlineStr"/>
+      <c r="Z7" s="10" t="inlineStr"/>
+      <c r="AA7" s="11" t="inlineStr"/>
+      <c r="AB7" s="12" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1672,10 +1812,10 @@
       <c r="Y8" s="4" t="inlineStr"/>
       <c r="Z8" s="5" t="inlineStr"/>
       <c r="AA8" s="6" t="n">
-        <v>2.849999999999994</v>
+        <v>3.599999999999994</v>
       </c>
       <c r="AB8" s="7" t="n">
-        <v>0.001663068214973446</v>
+        <v>0.002100717745229617</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -1704,7 +1844,7 @@
       </c>
       <c r="L9" s="8" t="inlineStr"/>
       <c r="M9" s="8" t="inlineStr"/>
-      <c r="N9" s="8" t="inlineStr">
+      <c r="N9" s="9" t="inlineStr">
         <is>
           <t>204.85</t>
         </is>
@@ -1732,11 +1872,11 @@
       <c r="W9" s="8" t="inlineStr"/>
       <c r="X9" s="8" t="inlineStr"/>
       <c r="Y9" s="8" t="inlineStr"/>
-      <c r="Z9" s="9" t="n">
-        <v>207.85</v>
-      </c>
-      <c r="AA9" s="10" t="inlineStr"/>
-      <c r="AB9" s="11" t="inlineStr"/>
+      <c r="Z9" s="10" t="n">
+        <v>208.6</v>
+      </c>
+      <c r="AA9" s="11" t="inlineStr"/>
+      <c r="AB9" s="12" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -1760,7 +1900,7 @@
       <c r="K10" s="8" t="inlineStr"/>
       <c r="L10" s="8" t="inlineStr"/>
       <c r="M10" s="8" t="inlineStr"/>
-      <c r="N10" s="8" t="inlineStr"/>
+      <c r="N10" s="9" t="inlineStr"/>
       <c r="O10" s="8" t="inlineStr">
         <is>
           <t>211.70</t>
@@ -1784,9 +1924,9 @@
       <c r="W10" s="8" t="inlineStr"/>
       <c r="X10" s="8" t="inlineStr"/>
       <c r="Y10" s="8" t="inlineStr"/>
-      <c r="Z10" s="9" t="inlineStr"/>
-      <c r="AA10" s="10" t="inlineStr"/>
-      <c r="AB10" s="11" t="inlineStr"/>
+      <c r="Z10" s="10" t="inlineStr"/>
+      <c r="AA10" s="11" t="inlineStr"/>
+      <c r="AB10" s="12" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="1" t="n"/>
@@ -1814,7 +1954,7 @@
       </c>
       <c r="L11" s="8" t="inlineStr"/>
       <c r="M11" s="8" t="inlineStr"/>
-      <c r="N11" s="8" t="inlineStr">
+      <c r="N11" s="9" t="inlineStr">
         <is>
           <t>147.80</t>
         </is>
@@ -1838,14 +1978,14 @@
       <c r="W11" s="8" t="inlineStr"/>
       <c r="X11" s="8" t="inlineStr"/>
       <c r="Y11" s="8" t="inlineStr"/>
-      <c r="Z11" s="9" t="n">
-        <v>164.88</v>
-      </c>
-      <c r="AA11" s="9" t="n">
-        <v>42.96999999999997</v>
-      </c>
-      <c r="AB11" s="11" t="n">
-        <v>-0.02507440042014353</v>
+      <c r="Z11" s="10" t="n">
+        <v>169.15</v>
+      </c>
+      <c r="AA11" s="10" t="n">
+        <v>39.44999999999999</v>
+      </c>
+      <c r="AB11" s="12" t="n">
+        <v>-0.02302036529147458</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -1866,7 +2006,7 @@
       <c r="K12" s="8" t="inlineStr"/>
       <c r="L12" s="8" t="inlineStr"/>
       <c r="M12" s="8" t="inlineStr"/>
-      <c r="N12" s="8" t="inlineStr"/>
+      <c r="N12" s="9" t="inlineStr"/>
       <c r="O12" s="8" t="inlineStr"/>
       <c r="P12" s="8" t="inlineStr"/>
       <c r="Q12" s="8" t="inlineStr">
@@ -1882,9 +2022,9 @@
       <c r="W12" s="8" t="inlineStr"/>
       <c r="X12" s="8" t="inlineStr"/>
       <c r="Y12" s="8" t="inlineStr"/>
-      <c r="Z12" s="9" t="inlineStr"/>
-      <c r="AA12" s="10" t="inlineStr"/>
-      <c r="AB12" s="11" t="inlineStr"/>
+      <c r="Z12" s="10" t="inlineStr"/>
+      <c r="AA12" s="11" t="inlineStr"/>
+      <c r="AB12" s="12" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="1" t="n"/>
@@ -1904,7 +2044,7 @@
       <c r="K13" s="8" t="inlineStr"/>
       <c r="L13" s="8" t="inlineStr"/>
       <c r="M13" s="8" t="inlineStr"/>
-      <c r="N13" s="8" t="inlineStr"/>
+      <c r="N13" s="9" t="inlineStr"/>
       <c r="O13" s="8" t="inlineStr"/>
       <c r="P13" s="8" t="inlineStr"/>
       <c r="Q13" s="8" t="inlineStr">
@@ -1920,9 +2060,9 @@
       <c r="W13" s="8" t="inlineStr"/>
       <c r="X13" s="8" t="inlineStr"/>
       <c r="Y13" s="8" t="inlineStr"/>
-      <c r="Z13" s="9" t="inlineStr"/>
-      <c r="AA13" s="10" t="inlineStr"/>
-      <c r="AB13" s="11" t="inlineStr"/>
+      <c r="Z13" s="10" t="inlineStr"/>
+      <c r="AA13" s="11" t="inlineStr"/>
+      <c r="AB13" s="12" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1962,10 +2102,10 @@
       <c r="Y14" s="4" t="inlineStr"/>
       <c r="Z14" s="5" t="inlineStr"/>
       <c r="AA14" s="6" t="n">
-        <v>-22.95000000000005</v>
+        <v>20.11249999999995</v>
       </c>
       <c r="AB14" s="7" t="n">
-        <v>-0.04416859122401856</v>
+        <v>0.03870765973826011</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
@@ -1992,7 +2132,7 @@
           <t>620.40</t>
         </is>
       </c>
-      <c r="L15" s="8" t="inlineStr">
+      <c r="L15" s="9" t="inlineStr">
         <is>
           <t>605.80</t>
         </is>
@@ -2022,11 +2162,11 @@
       <c r="W15" s="8" t="inlineStr"/>
       <c r="X15" s="8" t="inlineStr"/>
       <c r="Y15" s="8" t="inlineStr"/>
-      <c r="Z15" s="9" t="n">
-        <v>778.05</v>
-      </c>
-      <c r="AA15" s="10" t="inlineStr"/>
-      <c r="AB15" s="11" t="inlineStr"/>
+      <c r="Z15" s="10" t="n">
+        <v>821.1125</v>
+      </c>
+      <c r="AA15" s="11" t="inlineStr"/>
+      <c r="AB15" s="12" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="1" t="n"/>
@@ -2052,7 +2192,7 @@
           <t>693.30</t>
         </is>
       </c>
-      <c r="L16" s="8" t="inlineStr"/>
+      <c r="L16" s="9" t="inlineStr"/>
       <c r="M16" s="8" t="inlineStr"/>
       <c r="N16" s="8" t="inlineStr"/>
       <c r="O16" s="8" t="inlineStr">
@@ -2074,9 +2214,9 @@
       <c r="W16" s="8" t="inlineStr"/>
       <c r="X16" s="8" t="inlineStr"/>
       <c r="Y16" s="8" t="inlineStr"/>
-      <c r="Z16" s="9" t="inlineStr"/>
-      <c r="AA16" s="10" t="inlineStr"/>
-      <c r="AB16" s="11" t="inlineStr"/>
+      <c r="Z16" s="10" t="inlineStr"/>
+      <c r="AA16" s="11" t="inlineStr"/>
+      <c r="AB16" s="12" t="inlineStr"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="1" t="n"/>
@@ -2114,7 +2254,7 @@
           <t>666.55</t>
         </is>
       </c>
-      <c r="L17" s="8" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
         <is>
           <t>633.05</t>
         </is>
@@ -2140,14 +2280,14 @@
       <c r="W17" s="8" t="inlineStr"/>
       <c r="X17" s="8" t="inlineStr"/>
       <c r="Y17" s="8" t="inlineStr"/>
-      <c r="Z17" s="9" t="n">
-        <v>705.5400000000001</v>
-      </c>
-      <c r="AA17" s="9" t="n">
-        <v>72.50999999999988</v>
-      </c>
-      <c r="AB17" s="11" t="n">
-        <v>-0.1395496535796764</v>
+      <c r="Z17" s="10" t="n">
+        <v>723.6625</v>
+      </c>
+      <c r="AA17" s="10" t="n">
+        <v>97.44999999999993</v>
+      </c>
+      <c r="AB17" s="12" t="n">
+        <v>-0.1875481139337951</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
@@ -2166,7 +2306,7 @@
       <c r="I18" s="8" t="inlineStr"/>
       <c r="J18" s="8" t="inlineStr"/>
       <c r="K18" s="8" t="inlineStr"/>
-      <c r="L18" s="8" t="inlineStr"/>
+      <c r="L18" s="9" t="inlineStr"/>
       <c r="M18" s="8" t="inlineStr"/>
       <c r="N18" s="8" t="inlineStr"/>
       <c r="O18" s="8" t="inlineStr"/>
@@ -2184,9 +2324,9 @@
       <c r="W18" s="8" t="inlineStr"/>
       <c r="X18" s="8" t="inlineStr"/>
       <c r="Y18" s="8" t="inlineStr"/>
-      <c r="Z18" s="9" t="inlineStr"/>
-      <c r="AA18" s="10" t="inlineStr"/>
-      <c r="AB18" s="11" t="inlineStr"/>
+      <c r="Z18" s="10" t="inlineStr"/>
+      <c r="AA18" s="11" t="inlineStr"/>
+      <c r="AB18" s="12" t="inlineStr"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="1" t="n"/>
@@ -2204,7 +2344,7 @@
       <c r="I19" s="8" t="inlineStr"/>
       <c r="J19" s="8" t="inlineStr"/>
       <c r="K19" s="8" t="inlineStr"/>
-      <c r="L19" s="8" t="inlineStr"/>
+      <c r="L19" s="9" t="inlineStr"/>
       <c r="M19" s="8" t="inlineStr"/>
       <c r="N19" s="8" t="inlineStr"/>
       <c r="O19" s="8" t="inlineStr"/>
@@ -2222,9 +2362,9 @@
       <c r="W19" s="8" t="inlineStr"/>
       <c r="X19" s="8" t="inlineStr"/>
       <c r="Y19" s="8" t="inlineStr"/>
-      <c r="Z19" s="9" t="inlineStr"/>
-      <c r="AA19" s="10" t="inlineStr"/>
-      <c r="AB19" s="11" t="inlineStr"/>
+      <c r="Z19" s="10" t="inlineStr"/>
+      <c r="AA19" s="11" t="inlineStr"/>
+      <c r="AB19" s="12" t="inlineStr"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2320,11 +2460,11 @@
       <c r="W21" s="8" t="inlineStr"/>
       <c r="X21" s="8" t="inlineStr"/>
       <c r="Y21" s="8" t="inlineStr"/>
-      <c r="Z21" s="9" t="n">
+      <c r="Z21" s="10" t="n">
         <v>677.5</v>
       </c>
-      <c r="AA21" s="10" t="inlineStr"/>
-      <c r="AB21" s="11" t="inlineStr"/>
+      <c r="AA21" s="11" t="inlineStr"/>
+      <c r="AB21" s="12" t="inlineStr"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="1" t="n"/>
@@ -2368,9 +2508,9 @@
       <c r="W22" s="8" t="inlineStr"/>
       <c r="X22" s="8" t="inlineStr"/>
       <c r="Y22" s="8" t="inlineStr"/>
-      <c r="Z22" s="9" t="inlineStr"/>
-      <c r="AA22" s="10" t="inlineStr"/>
-      <c r="AB22" s="11" t="inlineStr"/>
+      <c r="Z22" s="10" t="inlineStr"/>
+      <c r="AA22" s="11" t="inlineStr"/>
+      <c r="AB22" s="12" t="inlineStr"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="1" t="n"/>
@@ -2418,13 +2558,13 @@
       <c r="W23" s="8" t="inlineStr"/>
       <c r="X23" s="8" t="inlineStr"/>
       <c r="Y23" s="8" t="inlineStr"/>
-      <c r="Z23" s="9" t="n">
+      <c r="Z23" s="10" t="n">
         <v>759.375</v>
       </c>
-      <c r="AA23" s="9" t="n">
+      <c r="AA23" s="10" t="n">
         <v>81.875</v>
       </c>
-      <c r="AB23" s="11" t="n">
+      <c r="AB23" s="12" t="n">
         <v>0.009872427139980468</v>
       </c>
     </row>
@@ -2462,9 +2602,9 @@
       <c r="W24" s="8" t="inlineStr"/>
       <c r="X24" s="8" t="inlineStr"/>
       <c r="Y24" s="8" t="inlineStr"/>
-      <c r="Z24" s="9" t="inlineStr"/>
-      <c r="AA24" s="10" t="inlineStr"/>
-      <c r="AB24" s="11" t="inlineStr"/>
+      <c r="Z24" s="10" t="inlineStr"/>
+      <c r="AA24" s="11" t="inlineStr"/>
+      <c r="AB24" s="12" t="inlineStr"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="1" t="n"/>
@@ -2500,9 +2640,9 @@
       <c r="W25" s="8" t="inlineStr"/>
       <c r="X25" s="8" t="inlineStr"/>
       <c r="Y25" s="8" t="inlineStr"/>
-      <c r="Z25" s="9" t="inlineStr"/>
-      <c r="AA25" s="10" t="inlineStr"/>
-      <c r="AB25" s="11" t="inlineStr"/>
+      <c r="Z25" s="10" t="inlineStr"/>
+      <c r="AA25" s="11" t="inlineStr"/>
+      <c r="AB25" s="12" t="inlineStr"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2589,12 +2729,12 @@
           <t>170.00</t>
         </is>
       </c>
-      <c r="Q27" s="12" t="inlineStr">
+      <c r="Q27" s="9" t="inlineStr">
         <is>
           <t>677.00</t>
         </is>
       </c>
-      <c r="R27" s="12" t="inlineStr"/>
+      <c r="R27" s="9" t="inlineStr"/>
       <c r="S27" s="8" t="inlineStr"/>
       <c r="T27" s="8" t="inlineStr"/>
       <c r="U27" s="8" t="inlineStr"/>
@@ -2610,11 +2750,11 @@
         </is>
       </c>
       <c r="Y27" s="8" t="inlineStr"/>
-      <c r="Z27" s="9" t="n">
+      <c r="Z27" s="10" t="n">
         <v>556.25</v>
       </c>
-      <c r="AA27" s="10" t="inlineStr"/>
-      <c r="AB27" s="11" t="inlineStr"/>
+      <c r="AA27" s="11" t="inlineStr"/>
+      <c r="AB27" s="12" t="inlineStr"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="1" t="n"/>
@@ -2637,8 +2777,8 @@
       <c r="N28" s="8" t="inlineStr"/>
       <c r="O28" s="8" t="inlineStr"/>
       <c r="P28" s="8" t="inlineStr"/>
-      <c r="Q28" s="12" t="inlineStr"/>
-      <c r="R28" s="12" t="inlineStr"/>
+      <c r="Q28" s="9" t="inlineStr"/>
+      <c r="R28" s="9" t="inlineStr"/>
       <c r="S28" s="8" t="inlineStr"/>
       <c r="T28" s="8" t="inlineStr"/>
       <c r="U28" s="8" t="inlineStr"/>
@@ -2650,9 +2790,9 @@
         </is>
       </c>
       <c r="Y28" s="8" t="inlineStr"/>
-      <c r="Z28" s="9" t="inlineStr"/>
-      <c r="AA28" s="10" t="inlineStr"/>
-      <c r="AB28" s="11" t="inlineStr"/>
+      <c r="Z28" s="10" t="inlineStr"/>
+      <c r="AA28" s="11" t="inlineStr"/>
+      <c r="AB28" s="12" t="inlineStr"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="1" t="n"/>
@@ -2683,7 +2823,7 @@
       <c r="N29" s="8" t="inlineStr"/>
       <c r="O29" s="8" t="inlineStr"/>
       <c r="P29" s="8" t="inlineStr"/>
-      <c r="Q29" s="12" t="inlineStr">
+      <c r="Q29" s="9" t="inlineStr">
         <is>
           <t>114.00</t>
         </is>
@@ -2708,13 +2848,13 @@
         </is>
       </c>
       <c r="Y29" s="8" t="inlineStr"/>
-      <c r="Z29" s="9" t="n">
+      <c r="Z29" s="10" t="n">
         <v>483.5</v>
       </c>
-      <c r="AA29" s="9" t="n">
+      <c r="AA29" s="10" t="n">
         <v>72.75</v>
       </c>
-      <c r="AB29" s="11" t="n">
+      <c r="AB29" s="12" t="n">
         <v>-0.09845716605765327</v>
       </c>
     </row>
@@ -2739,8 +2879,8 @@
       <c r="N30" s="8" t="inlineStr"/>
       <c r="O30" s="8" t="inlineStr"/>
       <c r="P30" s="8" t="inlineStr"/>
-      <c r="Q30" s="12" t="inlineStr"/>
-      <c r="R30" s="12" t="inlineStr"/>
+      <c r="Q30" s="9" t="inlineStr"/>
+      <c r="R30" s="9" t="inlineStr"/>
       <c r="S30" s="8" t="inlineStr"/>
       <c r="T30" s="8" t="inlineStr"/>
       <c r="U30" s="8" t="inlineStr"/>
@@ -2752,9 +2892,9 @@
         </is>
       </c>
       <c r="Y30" s="8" t="inlineStr"/>
-      <c r="Z30" s="9" t="inlineStr"/>
-      <c r="AA30" s="10" t="inlineStr"/>
-      <c r="AB30" s="11" t="inlineStr"/>
+      <c r="Z30" s="10" t="inlineStr"/>
+      <c r="AA30" s="11" t="inlineStr"/>
+      <c r="AB30" s="12" t="inlineStr"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="1" t="n"/>
@@ -2777,8 +2917,8 @@
       <c r="N31" s="8" t="inlineStr"/>
       <c r="O31" s="8" t="inlineStr"/>
       <c r="P31" s="8" t="inlineStr"/>
-      <c r="Q31" s="12" t="inlineStr"/>
-      <c r="R31" s="12" t="inlineStr"/>
+      <c r="Q31" s="9" t="inlineStr"/>
+      <c r="R31" s="9" t="inlineStr"/>
       <c r="S31" s="8" t="inlineStr"/>
       <c r="T31" s="8" t="inlineStr"/>
       <c r="U31" s="8" t="inlineStr"/>
@@ -2790,9 +2930,9 @@
         </is>
       </c>
       <c r="Y31" s="8" t="inlineStr"/>
-      <c r="Z31" s="9" t="inlineStr"/>
-      <c r="AA31" s="10" t="inlineStr"/>
-      <c r="AB31" s="11" t="inlineStr"/>
+      <c r="Z31" s="10" t="inlineStr"/>
+      <c r="AA31" s="11" t="inlineStr"/>
+      <c r="AB31" s="12" t="inlineStr"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -2832,10 +2972,10 @@
       <c r="Y32" s="4" t="inlineStr"/>
       <c r="Z32" s="5" t="inlineStr"/>
       <c r="AA32" s="6" t="n">
-        <v>-2710</v>
+        <v>-1327.5</v>
       </c>
       <c r="AB32" s="7" t="n">
-        <v>-0.07781207379226186</v>
+        <v>-0.03811643098126481</v>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
@@ -2853,7 +2993,7 @@
       <c r="H33" s="8" t="inlineStr"/>
       <c r="I33" s="8" t="inlineStr"/>
       <c r="J33" s="8" t="inlineStr"/>
-      <c r="K33" s="8" t="inlineStr">
+      <c r="K33" s="9" t="inlineStr">
         <is>
           <t>5300.00</t>
         </is>
@@ -2874,7 +3014,7 @@
           <t>15100.00, 16150.00, 14200.00, 14800.00</t>
         </is>
       </c>
-      <c r="P33" s="12" t="inlineStr">
+      <c r="P33" s="9" t="inlineStr">
         <is>
           <t>9300.00, 8850.00, 8250.00, 9250.00</t>
         </is>
@@ -2892,11 +3032,11 @@
       <c r="W33" s="8" t="inlineStr"/>
       <c r="X33" s="8" t="inlineStr"/>
       <c r="Y33" s="8" t="inlineStr"/>
-      <c r="Z33" s="9" t="n">
-        <v>10830</v>
-      </c>
-      <c r="AA33" s="10" t="inlineStr"/>
-      <c r="AB33" s="11" t="inlineStr"/>
+      <c r="Z33" s="10" t="n">
+        <v>12212.5</v>
+      </c>
+      <c r="AA33" s="11" t="inlineStr"/>
+      <c r="AB33" s="12" t="inlineStr"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="1" t="n"/>
@@ -2913,7 +3053,7 @@
       <c r="H34" s="8" t="inlineStr"/>
       <c r="I34" s="8" t="inlineStr"/>
       <c r="J34" s="8" t="inlineStr"/>
-      <c r="K34" s="8" t="inlineStr">
+      <c r="K34" s="9" t="inlineStr">
         <is>
           <t>5550.00</t>
         </is>
@@ -2930,7 +3070,7 @@
           <t>10950.00</t>
         </is>
       </c>
-      <c r="P34" s="12" t="inlineStr">
+      <c r="P34" s="9" t="inlineStr">
         <is>
           <t>5900.00</t>
         </is>
@@ -2948,9 +3088,9 @@
       <c r="W34" s="8" t="inlineStr"/>
       <c r="X34" s="8" t="inlineStr"/>
       <c r="Y34" s="8" t="inlineStr"/>
-      <c r="Z34" s="9" t="inlineStr"/>
-      <c r="AA34" s="10" t="inlineStr"/>
-      <c r="AB34" s="11" t="inlineStr"/>
+      <c r="Z34" s="10" t="inlineStr"/>
+      <c r="AA34" s="11" t="inlineStr"/>
+      <c r="AB34" s="12" t="inlineStr"/>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="1" t="n"/>
@@ -2967,7 +3107,7 @@
       <c r="H35" s="8" t="inlineStr"/>
       <c r="I35" s="8" t="inlineStr"/>
       <c r="J35" s="8" t="inlineStr"/>
-      <c r="K35" s="8" t="inlineStr">
+      <c r="K35" s="9" t="inlineStr">
         <is>
           <t>5500.00</t>
         </is>
@@ -2988,7 +3128,7 @@
           <t>14350.00</t>
         </is>
       </c>
-      <c r="P35" s="12" t="inlineStr">
+      <c r="P35" s="9" t="inlineStr">
         <is>
           <t>5650.00</t>
         </is>
@@ -3006,14 +3146,14 @@
       <c r="W35" s="8" t="inlineStr"/>
       <c r="X35" s="8" t="inlineStr"/>
       <c r="Y35" s="8" t="inlineStr"/>
-      <c r="Z35" s="9" t="n">
-        <v>11600</v>
-      </c>
-      <c r="AA35" s="9" t="n">
-        <v>770</v>
-      </c>
-      <c r="AB35" s="11" t="n">
-        <v>0.02210896561625153</v>
+      <c r="Z35" s="10" t="n">
+        <v>13125</v>
+      </c>
+      <c r="AA35" s="10" t="n">
+        <v>912.5</v>
+      </c>
+      <c r="AB35" s="12" t="n">
+        <v>0.026200559902376</v>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1">
@@ -3031,7 +3171,7 @@
       <c r="H36" s="8" t="inlineStr"/>
       <c r="I36" s="8" t="inlineStr"/>
       <c r="J36" s="8" t="inlineStr"/>
-      <c r="K36" s="8" t="inlineStr"/>
+      <c r="K36" s="9" t="inlineStr"/>
       <c r="L36" s="8" t="inlineStr"/>
       <c r="M36" s="8" t="inlineStr"/>
       <c r="N36" s="8" t="inlineStr"/>
@@ -3040,7 +3180,7 @@
           <t>18350.00</t>
         </is>
       </c>
-      <c r="P36" s="12" t="inlineStr"/>
+      <c r="P36" s="9" t="inlineStr"/>
       <c r="Q36" s="14" t="inlineStr">
         <is>
           <t>RUNNING</t>
@@ -3054,9 +3194,9 @@
       <c r="W36" s="8" t="inlineStr"/>
       <c r="X36" s="8" t="inlineStr"/>
       <c r="Y36" s="8" t="inlineStr"/>
-      <c r="Z36" s="9" t="inlineStr"/>
-      <c r="AA36" s="10" t="inlineStr"/>
-      <c r="AB36" s="11" t="inlineStr"/>
+      <c r="Z36" s="10" t="inlineStr"/>
+      <c r="AA36" s="11" t="inlineStr"/>
+      <c r="AB36" s="12" t="inlineStr"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="1" t="n"/>
@@ -3073,7 +3213,7 @@
       <c r="H37" s="8" t="inlineStr"/>
       <c r="I37" s="8" t="inlineStr"/>
       <c r="J37" s="8" t="inlineStr"/>
-      <c r="K37" s="8" t="inlineStr"/>
+      <c r="K37" s="9" t="inlineStr"/>
       <c r="L37" s="8" t="inlineStr"/>
       <c r="M37" s="8" t="inlineStr"/>
       <c r="N37" s="8" t="inlineStr"/>
@@ -3082,7 +3222,7 @@
           <t>19850.00</t>
         </is>
       </c>
-      <c r="P37" s="12" t="inlineStr"/>
+      <c r="P37" s="9" t="inlineStr"/>
       <c r="Q37" s="14" t="inlineStr">
         <is>
           <t>RUNNING</t>
@@ -3096,9 +3236,9 @@
       <c r="W37" s="8" t="inlineStr"/>
       <c r="X37" s="8" t="inlineStr"/>
       <c r="Y37" s="8" t="inlineStr"/>
-      <c r="Z37" s="9" t="inlineStr"/>
-      <c r="AA37" s="10" t="inlineStr"/>
-      <c r="AB37" s="11" t="inlineStr"/>
+      <c r="Z37" s="10" t="inlineStr"/>
+      <c r="AA37" s="11" t="inlineStr"/>
+      <c r="AB37" s="12" t="inlineStr"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -3179,7 +3319,7 @@
           <t>88.60</t>
         </is>
       </c>
-      <c r="O39" s="12" t="inlineStr">
+      <c r="O39" s="9" t="inlineStr">
         <is>
           <t>70.40</t>
         </is>
@@ -3202,11 +3342,11 @@
       <c r="W39" s="8" t="inlineStr"/>
       <c r="X39" s="8" t="inlineStr"/>
       <c r="Y39" s="8" t="inlineStr"/>
-      <c r="Z39" s="9" t="n">
+      <c r="Z39" s="10" t="n">
         <v>78.64999999999999</v>
       </c>
-      <c r="AA39" s="10" t="inlineStr"/>
-      <c r="AB39" s="11" t="inlineStr"/>
+      <c r="AA39" s="11" t="inlineStr"/>
+      <c r="AB39" s="12" t="inlineStr"/>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="1" t="n"/>
@@ -3231,7 +3371,7 @@
       <c r="L40" s="8" t="inlineStr"/>
       <c r="M40" s="8" t="inlineStr"/>
       <c r="N40" s="8" t="inlineStr"/>
-      <c r="O40" s="12" t="inlineStr"/>
+      <c r="O40" s="9" t="inlineStr"/>
       <c r="P40" s="14" t="inlineStr">
         <is>
           <t>RUNNING</t>
@@ -3246,9 +3386,9 @@
       <c r="W40" s="8" t="inlineStr"/>
       <c r="X40" s="8" t="inlineStr"/>
       <c r="Y40" s="8" t="inlineStr"/>
-      <c r="Z40" s="9" t="inlineStr"/>
-      <c r="AA40" s="10" t="inlineStr"/>
-      <c r="AB40" s="11" t="inlineStr"/>
+      <c r="Z40" s="10" t="inlineStr"/>
+      <c r="AA40" s="11" t="inlineStr"/>
+      <c r="AB40" s="12" t="inlineStr"/>
     </row>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="1" t="n"/>
@@ -3277,7 +3417,7 @@
       <c r="L41" s="8" t="inlineStr"/>
       <c r="M41" s="8" t="inlineStr"/>
       <c r="N41" s="8" t="inlineStr"/>
-      <c r="O41" s="12" t="inlineStr">
+      <c r="O41" s="9" t="inlineStr">
         <is>
           <t>51.15</t>
         </is>
@@ -3300,13 +3440,13 @@
       <c r="W41" s="8" t="inlineStr"/>
       <c r="X41" s="8" t="inlineStr"/>
       <c r="Y41" s="8" t="inlineStr"/>
-      <c r="Z41" s="9" t="n">
+      <c r="Z41" s="10" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="AA41" s="9" t="n">
+      <c r="AA41" s="10" t="n">
         <v>3.250000000000014</v>
       </c>
-      <c r="AB41" s="11" t="n">
+      <c r="AB41" s="12" t="n">
         <v>0.2708333333333345</v>
       </c>
     </row>
@@ -3329,7 +3469,7 @@
       <c r="L42" s="8" t="inlineStr"/>
       <c r="M42" s="8" t="inlineStr"/>
       <c r="N42" s="8" t="inlineStr"/>
-      <c r="O42" s="12" t="inlineStr"/>
+      <c r="O42" s="9" t="inlineStr"/>
       <c r="P42" s="14" t="inlineStr">
         <is>
           <t>RUNNING</t>
@@ -3344,9 +3484,9 @@
       <c r="W42" s="8" t="inlineStr"/>
       <c r="X42" s="8" t="inlineStr"/>
       <c r="Y42" s="8" t="inlineStr"/>
-      <c r="Z42" s="9" t="inlineStr"/>
-      <c r="AA42" s="10" t="inlineStr"/>
-      <c r="AB42" s="11" t="inlineStr"/>
+      <c r="Z42" s="10" t="inlineStr"/>
+      <c r="AA42" s="11" t="inlineStr"/>
+      <c r="AB42" s="12" t="inlineStr"/>
     </row>
     <row r="43" ht="24" customHeight="1">
       <c r="A43" s="1" t="n"/>
@@ -3367,7 +3507,7 @@
       <c r="L43" s="8" t="inlineStr"/>
       <c r="M43" s="8" t="inlineStr"/>
       <c r="N43" s="8" t="inlineStr"/>
-      <c r="O43" s="12" t="inlineStr"/>
+      <c r="O43" s="9" t="inlineStr"/>
       <c r="P43" s="14" t="inlineStr">
         <is>
           <t>RUNNING</t>
@@ -3382,9 +3522,9 @@
       <c r="W43" s="8" t="inlineStr"/>
       <c r="X43" s="8" t="inlineStr"/>
       <c r="Y43" s="8" t="inlineStr"/>
-      <c r="Z43" s="9" t="inlineStr"/>
-      <c r="AA43" s="10" t="inlineStr"/>
-      <c r="AB43" s="11" t="inlineStr"/>
+      <c r="Z43" s="10" t="inlineStr"/>
+      <c r="AA43" s="11" t="inlineStr"/>
+      <c r="AB43" s="12" t="inlineStr"/>
     </row>
     <row r="44" ht="24" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -3480,11 +3620,11 @@
       <c r="W45" s="8" t="inlineStr"/>
       <c r="X45" s="8" t="inlineStr"/>
       <c r="Y45" s="8" t="inlineStr"/>
-      <c r="Z45" s="9" t="n">
+      <c r="Z45" s="10" t="n">
         <v>11.73333333333333</v>
       </c>
-      <c r="AA45" s="10" t="inlineStr"/>
-      <c r="AB45" s="11" t="inlineStr"/>
+      <c r="AA45" s="11" t="inlineStr"/>
+      <c r="AB45" s="12" t="inlineStr"/>
     </row>
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="1" t="n"/>
@@ -3528,9 +3668,9 @@
       <c r="W46" s="8" t="inlineStr"/>
       <c r="X46" s="8" t="inlineStr"/>
       <c r="Y46" s="8" t="inlineStr"/>
-      <c r="Z46" s="9" t="inlineStr"/>
-      <c r="AA46" s="10" t="inlineStr"/>
-      <c r="AB46" s="11" t="inlineStr"/>
+      <c r="Z46" s="10" t="inlineStr"/>
+      <c r="AA46" s="11" t="inlineStr"/>
+      <c r="AB46" s="12" t="inlineStr"/>
     </row>
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="1" t="n"/>
@@ -3574,13 +3714,13 @@
       <c r="W47" s="8" t="inlineStr"/>
       <c r="X47" s="8" t="inlineStr"/>
       <c r="Y47" s="8" t="inlineStr"/>
-      <c r="Z47" s="9" t="n">
+      <c r="Z47" s="10" t="n">
         <v>12.36666666666667</v>
       </c>
-      <c r="AA47" s="9" t="n">
+      <c r="AA47" s="10" t="n">
         <v>0.6333333333333311</v>
       </c>
-      <c r="AB47" s="11" t="n">
+      <c r="AB47" s="12" t="n">
         <v>0.02199074074074066</v>
       </c>
     </row>
@@ -3678,11 +3818,11 @@
       <c r="W49" s="8" t="inlineStr"/>
       <c r="X49" s="8" t="inlineStr"/>
       <c r="Y49" s="8" t="inlineStr"/>
-      <c r="Z49" s="9" t="n">
+      <c r="Z49" s="10" t="n">
         <v>1688.75</v>
       </c>
-      <c r="AA49" s="10" t="inlineStr"/>
-      <c r="AB49" s="11" t="inlineStr"/>
+      <c r="AA49" s="11" t="inlineStr"/>
+      <c r="AB49" s="12" t="inlineStr"/>
     </row>
     <row r="50" ht="24" customHeight="1">
       <c r="A50" s="1" t="n"/>
@@ -3722,9 +3862,9 @@
       <c r="W50" s="8" t="inlineStr"/>
       <c r="X50" s="8" t="inlineStr"/>
       <c r="Y50" s="8" t="inlineStr"/>
-      <c r="Z50" s="9" t="inlineStr"/>
-      <c r="AA50" s="10" t="inlineStr"/>
-      <c r="AB50" s="11" t="inlineStr"/>
+      <c r="Z50" s="10" t="inlineStr"/>
+      <c r="AA50" s="11" t="inlineStr"/>
+      <c r="AB50" s="12" t="inlineStr"/>
     </row>
     <row r="51" ht="24" customHeight="1">
       <c r="A51" s="1" t="n"/>
@@ -3772,13 +3912,13 @@
       <c r="W51" s="8" t="inlineStr"/>
       <c r="X51" s="8" t="inlineStr"/>
       <c r="Y51" s="8" t="inlineStr"/>
-      <c r="Z51" s="9" t="n">
+      <c r="Z51" s="10" t="n">
         <v>1425</v>
       </c>
-      <c r="AA51" s="9" t="n">
+      <c r="AA51" s="10" t="n">
         <v>263.75</v>
       </c>
-      <c r="AB51" s="11" t="n">
+      <c r="AB51" s="12" t="n">
         <v>-0.04010308964846126</v>
       </c>
     </row>
@@ -3820,9 +3960,9 @@
       <c r="W52" s="8" t="inlineStr"/>
       <c r="X52" s="8" t="inlineStr"/>
       <c r="Y52" s="8" t="inlineStr"/>
-      <c r="Z52" s="9" t="inlineStr"/>
-      <c r="AA52" s="10" t="inlineStr"/>
-      <c r="AB52" s="11" t="inlineStr"/>
+      <c r="Z52" s="10" t="inlineStr"/>
+      <c r="AA52" s="11" t="inlineStr"/>
+      <c r="AB52" s="12" t="inlineStr"/>
     </row>
     <row r="53" ht="24" customHeight="1">
       <c r="A53" s="1" t="n"/>
@@ -3862,9 +4002,9 @@
       <c r="W53" s="8" t="inlineStr"/>
       <c r="X53" s="8" t="inlineStr"/>
       <c r="Y53" s="8" t="inlineStr"/>
-      <c r="Z53" s="9" t="inlineStr"/>
-      <c r="AA53" s="10" t="inlineStr"/>
-      <c r="AB53" s="11" t="inlineStr"/>
+      <c r="Z53" s="10" t="inlineStr"/>
+      <c r="AA53" s="11" t="inlineStr"/>
+      <c r="AB53" s="12" t="inlineStr"/>
     </row>
     <row r="54" ht="24" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -3960,11 +4100,11 @@
       <c r="W55" s="8" t="inlineStr"/>
       <c r="X55" s="8" t="inlineStr"/>
       <c r="Y55" s="8" t="inlineStr"/>
-      <c r="Z55" s="9" t="n">
+      <c r="Z55" s="10" t="n">
         <v>57571.66666666666</v>
       </c>
-      <c r="AA55" s="10" t="inlineStr"/>
-      <c r="AB55" s="11" t="inlineStr"/>
+      <c r="AA55" s="11" t="inlineStr"/>
+      <c r="AB55" s="12" t="inlineStr"/>
     </row>
     <row r="56" ht="24" customHeight="1">
       <c r="A56" s="1" t="n"/>
@@ -4000,9 +4140,9 @@
       <c r="W56" s="8" t="inlineStr"/>
       <c r="X56" s="8" t="inlineStr"/>
       <c r="Y56" s="8" t="inlineStr"/>
-      <c r="Z56" s="9" t="inlineStr"/>
-      <c r="AA56" s="10" t="inlineStr"/>
-      <c r="AB56" s="11" t="inlineStr"/>
+      <c r="Z56" s="10" t="inlineStr"/>
+      <c r="AA56" s="11" t="inlineStr"/>
+      <c r="AB56" s="12" t="inlineStr"/>
     </row>
     <row r="57" ht="24" customHeight="1">
       <c r="A57" s="1" t="n"/>
@@ -4046,13 +4186,13 @@
       <c r="W57" s="8" t="inlineStr"/>
       <c r="X57" s="8" t="inlineStr"/>
       <c r="Y57" s="8" t="inlineStr"/>
-      <c r="Z57" s="9" t="n">
+      <c r="Z57" s="10" t="n">
         <v>57908.33333333334</v>
       </c>
-      <c r="AA57" s="9" t="n">
+      <c r="AA57" s="10" t="n">
         <v>336.6666666666715</v>
       </c>
-      <c r="AB57" s="11" t="n">
+      <c r="AB57" s="12" t="n">
         <v>0.01344037728869018</v>
       </c>
     </row>
@@ -4150,11 +4290,11 @@
       <c r="W59" s="8" t="inlineStr"/>
       <c r="X59" s="8" t="inlineStr"/>
       <c r="Y59" s="8" t="inlineStr"/>
-      <c r="Z59" s="9" t="n">
+      <c r="Z59" s="10" t="n">
         <v>195.5833333333333</v>
       </c>
-      <c r="AA59" s="10" t="inlineStr"/>
-      <c r="AB59" s="11" t="inlineStr"/>
+      <c r="AA59" s="11" t="inlineStr"/>
+      <c r="AB59" s="12" t="inlineStr"/>
     </row>
     <row r="60" ht="24" customHeight="1">
       <c r="A60" s="1" t="n"/>
@@ -4190,9 +4330,9 @@
       <c r="W60" s="8" t="inlineStr"/>
       <c r="X60" s="8" t="inlineStr"/>
       <c r="Y60" s="8" t="inlineStr"/>
-      <c r="Z60" s="9" t="inlineStr"/>
-      <c r="AA60" s="10" t="inlineStr"/>
-      <c r="AB60" s="11" t="inlineStr"/>
+      <c r="Z60" s="10" t="inlineStr"/>
+      <c r="AA60" s="11" t="inlineStr"/>
+      <c r="AB60" s="12" t="inlineStr"/>
     </row>
     <row r="61" ht="24" customHeight="1">
       <c r="A61" s="1" t="n"/>
@@ -4236,13 +4376,13 @@
       <c r="W61" s="8" t="inlineStr"/>
       <c r="X61" s="8" t="inlineStr"/>
       <c r="Y61" s="8" t="inlineStr"/>
-      <c r="Z61" s="9" t="n">
+      <c r="Z61" s="10" t="n">
         <v>157.0833333333333</v>
       </c>
-      <c r="AA61" s="9" t="n">
+      <c r="AA61" s="10" t="n">
         <v>38.5</v>
       </c>
-      <c r="AB61" s="11" t="n">
+      <c r="AB61" s="12" t="n">
         <v>-0.02116663917752488</v>
       </c>
     </row>
@@ -4280,9 +4420,9 @@
       <c r="W62" s="8" t="inlineStr"/>
       <c r="X62" s="8" t="inlineStr"/>
       <c r="Y62" s="8" t="inlineStr"/>
-      <c r="Z62" s="9" t="inlineStr"/>
-      <c r="AA62" s="10" t="inlineStr"/>
-      <c r="AB62" s="11" t="inlineStr"/>
+      <c r="Z62" s="10" t="inlineStr"/>
+      <c r="AA62" s="11" t="inlineStr"/>
+      <c r="AB62" s="12" t="inlineStr"/>
     </row>
     <row r="63" ht="24" customHeight="1">
       <c r="A63" s="1" t="n"/>
@@ -4318,9 +4458,9 @@
       <c r="W63" s="8" t="inlineStr"/>
       <c r="X63" s="8" t="inlineStr"/>
       <c r="Y63" s="8" t="inlineStr"/>
-      <c r="Z63" s="9" t="inlineStr"/>
-      <c r="AA63" s="10" t="inlineStr"/>
-      <c r="AB63" s="11" t="inlineStr"/>
+      <c r="Z63" s="10" t="inlineStr"/>
+      <c r="AA63" s="11" t="inlineStr"/>
+      <c r="AB63" s="12" t="inlineStr"/>
     </row>
     <row r="64" ht="24" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -4412,11 +4552,11 @@
       <c r="W65" s="8" t="inlineStr"/>
       <c r="X65" s="8" t="inlineStr"/>
       <c r="Y65" s="8" t="inlineStr"/>
-      <c r="Z65" s="9" t="n">
+      <c r="Z65" s="10" t="n">
         <v>33.45</v>
       </c>
-      <c r="AA65" s="10" t="inlineStr"/>
-      <c r="AB65" s="11" t="inlineStr"/>
+      <c r="AA65" s="11" t="inlineStr"/>
+      <c r="AB65" s="12" t="inlineStr"/>
     </row>
     <row r="66" ht="24" customHeight="1">
       <c r="A66" s="1" t="n"/>
@@ -4452,9 +4592,9 @@
       <c r="W66" s="8" t="inlineStr"/>
       <c r="X66" s="8" t="inlineStr"/>
       <c r="Y66" s="8" t="inlineStr"/>
-      <c r="Z66" s="9" t="inlineStr"/>
-      <c r="AA66" s="10" t="inlineStr"/>
-      <c r="AB66" s="11" t="inlineStr"/>
+      <c r="Z66" s="10" t="inlineStr"/>
+      <c r="AA66" s="11" t="inlineStr"/>
+      <c r="AB66" s="12" t="inlineStr"/>
     </row>
     <row r="67" ht="24" customHeight="1">
       <c r="A67" s="1" t="n"/>
@@ -4498,13 +4638,13 @@
       <c r="W67" s="8" t="inlineStr"/>
       <c r="X67" s="8" t="inlineStr"/>
       <c r="Y67" s="8" t="inlineStr"/>
-      <c r="Z67" s="9" t="n">
+      <c r="Z67" s="10" t="n">
         <v>33.35</v>
       </c>
-      <c r="AA67" s="9" t="n">
+      <c r="AA67" s="10" t="n">
         <v>0.09999999999999432</v>
       </c>
-      <c r="AB67" s="11" t="n">
+      <c r="AB67" s="12" t="n">
         <v>-0.003378378378378186</v>
       </c>
     </row>
@@ -4542,9 +4682,9 @@
       <c r="W68" s="8" t="inlineStr"/>
       <c r="X68" s="8" t="inlineStr"/>
       <c r="Y68" s="8" t="inlineStr"/>
-      <c r="Z68" s="9" t="inlineStr"/>
-      <c r="AA68" s="10" t="inlineStr"/>
-      <c r="AB68" s="11" t="inlineStr"/>
+      <c r="Z68" s="10" t="inlineStr"/>
+      <c r="AA68" s="11" t="inlineStr"/>
+      <c r="AB68" s="12" t="inlineStr"/>
     </row>
     <row r="69" ht="24" customHeight="1">
       <c r="A69" s="1" t="n"/>
@@ -4580,9 +4720,9 @@
       <c r="W69" s="8" t="inlineStr"/>
       <c r="X69" s="8" t="inlineStr"/>
       <c r="Y69" s="8" t="inlineStr"/>
-      <c r="Z69" s="9" t="inlineStr"/>
-      <c r="AA69" s="10" t="inlineStr"/>
-      <c r="AB69" s="11" t="inlineStr"/>
+      <c r="Z69" s="10" t="inlineStr"/>
+      <c r="AA69" s="11" t="inlineStr"/>
+      <c r="AB69" s="12" t="inlineStr"/>
     </row>
     <row r="70" ht="24" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
@@ -4637,7 +4777,7 @@
       </c>
       <c r="C71" s="8" t="inlineStr"/>
       <c r="D71" s="8" t="inlineStr"/>
-      <c r="E71" s="12" t="inlineStr">
+      <c r="E71" s="9" t="inlineStr">
         <is>
           <t>2068.00</t>
         </is>
@@ -4678,11 +4818,11 @@
       <c r="W71" s="8" t="inlineStr"/>
       <c r="X71" s="8" t="inlineStr"/>
       <c r="Y71" s="8" t="inlineStr"/>
-      <c r="Z71" s="9" t="n">
+      <c r="Z71" s="10" t="n">
         <v>1742.375</v>
       </c>
-      <c r="AA71" s="10" t="inlineStr"/>
-      <c r="AB71" s="11" t="inlineStr"/>
+      <c r="AA71" s="11" t="inlineStr"/>
+      <c r="AB71" s="12" t="inlineStr"/>
     </row>
     <row r="72" ht="24" customHeight="1">
       <c r="A72" s="1" t="n"/>
@@ -4693,7 +4833,7 @@
       </c>
       <c r="C72" s="8" t="inlineStr"/>
       <c r="D72" s="8" t="inlineStr"/>
-      <c r="E72" s="12" t="inlineStr">
+      <c r="E72" s="9" t="inlineStr">
         <is>
           <t>2301.00</t>
         </is>
@@ -4734,9 +4874,9 @@
       <c r="W72" s="8" t="inlineStr"/>
       <c r="X72" s="8" t="inlineStr"/>
       <c r="Y72" s="8" t="inlineStr"/>
-      <c r="Z72" s="9" t="inlineStr"/>
-      <c r="AA72" s="10" t="inlineStr"/>
-      <c r="AB72" s="11" t="inlineStr"/>
+      <c r="Z72" s="10" t="inlineStr"/>
+      <c r="AA72" s="11" t="inlineStr"/>
+      <c r="AB72" s="12" t="inlineStr"/>
     </row>
     <row r="73" ht="24" customHeight="1">
       <c r="A73" s="1" t="n"/>
@@ -4747,7 +4887,7 @@
       </c>
       <c r="C73" s="8" t="inlineStr"/>
       <c r="D73" s="8" t="inlineStr"/>
-      <c r="E73" s="12" t="inlineStr">
+      <c r="E73" s="9" t="inlineStr">
         <is>
           <t>2113.50, 2350.50</t>
         </is>
@@ -4796,13 +4936,13 @@
       <c r="W73" s="8" t="inlineStr"/>
       <c r="X73" s="8" t="inlineStr"/>
       <c r="Y73" s="8" t="inlineStr"/>
-      <c r="Z73" s="9" t="n">
+      <c r="Z73" s="10" t="n">
         <v>1986.75</v>
       </c>
-      <c r="AA73" s="9" t="n">
+      <c r="AA73" s="10" t="n">
         <v>244.375</v>
       </c>
-      <c r="AB73" s="11" t="n">
+      <c r="AB73" s="12" t="n">
         <v>0.05723738142639653</v>
       </c>
     </row>
@@ -4815,7 +4955,7 @@
       </c>
       <c r="C74" s="8" t="inlineStr"/>
       <c r="D74" s="8" t="inlineStr"/>
-      <c r="E74" s="12" t="inlineStr"/>
+      <c r="E74" s="9" t="inlineStr"/>
       <c r="F74" s="8" t="inlineStr"/>
       <c r="G74" s="8" t="inlineStr"/>
       <c r="H74" s="8" t="inlineStr"/>
@@ -4844,9 +4984,9 @@
       <c r="W74" s="8" t="inlineStr"/>
       <c r="X74" s="8" t="inlineStr"/>
       <c r="Y74" s="8" t="inlineStr"/>
-      <c r="Z74" s="9" t="inlineStr"/>
-      <c r="AA74" s="10" t="inlineStr"/>
-      <c r="AB74" s="11" t="inlineStr"/>
+      <c r="Z74" s="10" t="inlineStr"/>
+      <c r="AA74" s="11" t="inlineStr"/>
+      <c r="AB74" s="12" t="inlineStr"/>
     </row>
     <row r="75" ht="24" customHeight="1">
       <c r="A75" s="1" t="n"/>
@@ -4857,7 +4997,7 @@
       </c>
       <c r="C75" s="8" t="inlineStr"/>
       <c r="D75" s="8" t="inlineStr"/>
-      <c r="E75" s="12" t="inlineStr"/>
+      <c r="E75" s="9" t="inlineStr"/>
       <c r="F75" s="8" t="inlineStr"/>
       <c r="G75" s="8" t="inlineStr"/>
       <c r="H75" s="8" t="inlineStr"/>
@@ -4882,9 +5022,9 @@
       <c r="W75" s="8" t="inlineStr"/>
       <c r="X75" s="8" t="inlineStr"/>
       <c r="Y75" s="8" t="inlineStr"/>
-      <c r="Z75" s="9" t="inlineStr"/>
-      <c r="AA75" s="10" t="inlineStr"/>
-      <c r="AB75" s="11" t="inlineStr"/>
+      <c r="Z75" s="10" t="inlineStr"/>
+      <c r="AA75" s="11" t="inlineStr"/>
+      <c r="AB75" s="12" t="inlineStr"/>
     </row>
     <row r="76" ht="24" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
@@ -4969,38 +5109,38 @@
       <c r="L77" s="8" t="inlineStr"/>
       <c r="M77" s="8" t="inlineStr"/>
       <c r="N77" s="8" t="inlineStr"/>
-      <c r="O77" s="12" t="inlineStr">
+      <c r="O77" s="9" t="inlineStr">
         <is>
           <t>2486.00</t>
         </is>
       </c>
-      <c r="P77" s="12" t="inlineStr">
+      <c r="P77" s="9" t="inlineStr">
         <is>
           <t>1250.00</t>
         </is>
       </c>
-      <c r="Q77" s="12" t="inlineStr"/>
-      <c r="R77" s="12" t="inlineStr"/>
-      <c r="S77" s="12" t="inlineStr"/>
+      <c r="Q77" s="9" t="inlineStr"/>
+      <c r="R77" s="9" t="inlineStr"/>
+      <c r="S77" s="9" t="inlineStr"/>
       <c r="T77" s="8" t="inlineStr"/>
-      <c r="U77" s="12" t="inlineStr"/>
+      <c r="U77" s="9" t="inlineStr"/>
       <c r="V77" s="8" t="inlineStr"/>
       <c r="W77" s="8" t="inlineStr">
         <is>
           <t>3585.00</t>
         </is>
       </c>
-      <c r="X77" s="12" t="inlineStr">
+      <c r="X77" s="9" t="inlineStr">
         <is>
           <t>2594.00</t>
         </is>
       </c>
       <c r="Y77" s="8" t="inlineStr"/>
-      <c r="Z77" s="9" t="n">
+      <c r="Z77" s="10" t="n">
         <v>3693</v>
       </c>
-      <c r="AA77" s="10" t="inlineStr"/>
-      <c r="AB77" s="11" t="inlineStr"/>
+      <c r="AA77" s="11" t="inlineStr"/>
+      <c r="AB77" s="12" t="inlineStr"/>
     </row>
     <row r="78" ht="24" customHeight="1">
       <c r="A78" s="1" t="n"/>
@@ -5021,28 +5161,28 @@
       <c r="L78" s="8" t="inlineStr"/>
       <c r="M78" s="8" t="inlineStr"/>
       <c r="N78" s="8" t="inlineStr"/>
-      <c r="O78" s="12" t="inlineStr"/>
-      <c r="P78" s="12" t="inlineStr"/>
-      <c r="Q78" s="12" t="inlineStr"/>
-      <c r="R78" s="12" t="inlineStr">
+      <c r="O78" s="9" t="inlineStr"/>
+      <c r="P78" s="9" t="inlineStr"/>
+      <c r="Q78" s="9" t="inlineStr"/>
+      <c r="R78" s="9" t="inlineStr">
         <is>
           <t>2533.00</t>
         </is>
       </c>
-      <c r="S78" s="12" t="inlineStr"/>
+      <c r="S78" s="9" t="inlineStr"/>
       <c r="T78" s="8" t="inlineStr"/>
-      <c r="U78" s="12" t="inlineStr"/>
+      <c r="U78" s="9" t="inlineStr"/>
       <c r="V78" s="8" t="inlineStr"/>
       <c r="W78" s="8" t="inlineStr">
         <is>
           <t>4472.00</t>
         </is>
       </c>
-      <c r="X78" s="12" t="inlineStr"/>
+      <c r="X78" s="9" t="inlineStr"/>
       <c r="Y78" s="8" t="inlineStr"/>
-      <c r="Z78" s="9" t="inlineStr"/>
-      <c r="AA78" s="10" t="inlineStr"/>
-      <c r="AB78" s="11" t="inlineStr"/>
+      <c r="Z78" s="10" t="inlineStr"/>
+      <c r="AA78" s="11" t="inlineStr"/>
+      <c r="AB78" s="12" t="inlineStr"/>
     </row>
     <row r="79" ht="24" customHeight="1">
       <c r="A79" s="1" t="n"/>
@@ -5071,12 +5211,12 @@
       <c r="L79" s="8" t="inlineStr"/>
       <c r="M79" s="8" t="inlineStr"/>
       <c r="N79" s="8" t="inlineStr"/>
-      <c r="O79" s="12" t="inlineStr">
+      <c r="O79" s="9" t="inlineStr">
         <is>
           <t>1024.00</t>
         </is>
       </c>
-      <c r="P79" s="12" t="inlineStr">
+      <c r="P79" s="9" t="inlineStr">
         <is>
           <t>927.00</t>
         </is>
@@ -5112,19 +5252,19 @@
           <t>7531.00</t>
         </is>
       </c>
-      <c r="X79" s="12" t="inlineStr">
+      <c r="X79" s="9" t="inlineStr">
         <is>
           <t>1005.00</t>
         </is>
       </c>
       <c r="Y79" s="8" t="inlineStr"/>
-      <c r="Z79" s="9" t="n">
+      <c r="Z79" s="10" t="n">
         <v>4895.666666666667</v>
       </c>
-      <c r="AA79" s="9" t="n">
+      <c r="AA79" s="10" t="n">
         <v>1202.666666666667</v>
       </c>
-      <c r="AB79" s="11" t="n">
+      <c r="AB79" s="12" t="n">
         <v>0.558107878169134</v>
       </c>
     </row>
@@ -5147,24 +5287,24 @@
       <c r="L80" s="8" t="inlineStr"/>
       <c r="M80" s="8" t="inlineStr"/>
       <c r="N80" s="8" t="inlineStr"/>
-      <c r="O80" s="12" t="inlineStr"/>
-      <c r="P80" s="12" t="inlineStr"/>
-      <c r="Q80" s="12" t="inlineStr"/>
-      <c r="R80" s="12" t="inlineStr"/>
-      <c r="S80" s="12" t="inlineStr"/>
+      <c r="O80" s="9" t="inlineStr"/>
+      <c r="P80" s="9" t="inlineStr"/>
+      <c r="Q80" s="9" t="inlineStr"/>
+      <c r="R80" s="9" t="inlineStr"/>
+      <c r="S80" s="9" t="inlineStr"/>
       <c r="T80" s="8" t="inlineStr"/>
-      <c r="U80" s="12" t="inlineStr"/>
+      <c r="U80" s="9" t="inlineStr"/>
       <c r="V80" s="8" t="inlineStr"/>
       <c r="W80" s="8" t="inlineStr">
         <is>
           <t>5320.00</t>
         </is>
       </c>
-      <c r="X80" s="12" t="inlineStr"/>
+      <c r="X80" s="9" t="inlineStr"/>
       <c r="Y80" s="8" t="inlineStr"/>
-      <c r="Z80" s="9" t="inlineStr"/>
-      <c r="AA80" s="10" t="inlineStr"/>
-      <c r="AB80" s="11" t="inlineStr"/>
+      <c r="Z80" s="10" t="inlineStr"/>
+      <c r="AA80" s="11" t="inlineStr"/>
+      <c r="AB80" s="12" t="inlineStr"/>
     </row>
     <row r="81" ht="24" customHeight="1">
       <c r="A81" s="1" t="n"/>
@@ -5185,24 +5325,24 @@
       <c r="L81" s="8" t="inlineStr"/>
       <c r="M81" s="8" t="inlineStr"/>
       <c r="N81" s="8" t="inlineStr"/>
-      <c r="O81" s="12" t="inlineStr"/>
-      <c r="P81" s="12" t="inlineStr"/>
-      <c r="Q81" s="12" t="inlineStr"/>
-      <c r="R81" s="12" t="inlineStr"/>
-      <c r="S81" s="12" t="inlineStr"/>
+      <c r="O81" s="9" t="inlineStr"/>
+      <c r="P81" s="9" t="inlineStr"/>
+      <c r="Q81" s="9" t="inlineStr"/>
+      <c r="R81" s="9" t="inlineStr"/>
+      <c r="S81" s="9" t="inlineStr"/>
       <c r="T81" s="8" t="inlineStr"/>
-      <c r="U81" s="12" t="inlineStr"/>
+      <c r="U81" s="9" t="inlineStr"/>
       <c r="V81" s="8" t="inlineStr"/>
       <c r="W81" s="8" t="inlineStr">
         <is>
           <t>2516.00</t>
         </is>
       </c>
-      <c r="X81" s="12" t="inlineStr"/>
+      <c r="X81" s="9" t="inlineStr"/>
       <c r="Y81" s="8" t="inlineStr"/>
-      <c r="Z81" s="9" t="inlineStr"/>
-      <c r="AA81" s="10" t="inlineStr"/>
-      <c r="AB81" s="11" t="inlineStr"/>
+      <c r="Z81" s="10" t="inlineStr"/>
+      <c r="AA81" s="11" t="inlineStr"/>
+      <c r="AB81" s="12" t="inlineStr"/>
     </row>
     <row r="82" ht="24" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
@@ -5294,11 +5434,11 @@
       <c r="W83" s="8" t="inlineStr"/>
       <c r="X83" s="8" t="inlineStr"/>
       <c r="Y83" s="8" t="inlineStr"/>
-      <c r="Z83" s="9" t="n">
+      <c r="Z83" s="10" t="n">
         <v>11785.625</v>
       </c>
-      <c r="AA83" s="10" t="inlineStr"/>
-      <c r="AB83" s="11" t="inlineStr"/>
+      <c r="AA83" s="11" t="inlineStr"/>
+      <c r="AB83" s="12" t="inlineStr"/>
     </row>
     <row r="84" ht="24" customHeight="1">
       <c r="A84" s="1" t="n"/>
@@ -5334,9 +5474,9 @@
       <c r="W84" s="8" t="inlineStr"/>
       <c r="X84" s="8" t="inlineStr"/>
       <c r="Y84" s="8" t="inlineStr"/>
-      <c r="Z84" s="9" t="inlineStr"/>
-      <c r="AA84" s="10" t="inlineStr"/>
-      <c r="AB84" s="11" t="inlineStr"/>
+      <c r="Z84" s="10" t="inlineStr"/>
+      <c r="AA84" s="11" t="inlineStr"/>
+      <c r="AB84" s="12" t="inlineStr"/>
     </row>
     <row r="85" ht="24" customHeight="1">
       <c r="A85" s="1" t="n"/>
@@ -5384,13 +5524,13 @@
       <c r="W85" s="8" t="inlineStr"/>
       <c r="X85" s="8" t="inlineStr"/>
       <c r="Y85" s="8" t="inlineStr"/>
-      <c r="Z85" s="9" t="n">
+      <c r="Z85" s="10" t="n">
         <v>13229.25</v>
       </c>
-      <c r="AA85" s="9" t="n">
+      <c r="AA85" s="10" t="n">
         <v>1443.625</v>
       </c>
-      <c r="AB85" s="11" t="n">
+      <c r="AB85" s="12" t="n">
         <v>0.04844476734430894</v>
       </c>
     </row>
@@ -5428,9 +5568,9 @@
       <c r="W86" s="8" t="inlineStr"/>
       <c r="X86" s="8" t="inlineStr"/>
       <c r="Y86" s="8" t="inlineStr"/>
-      <c r="Z86" s="9" t="inlineStr"/>
-      <c r="AA86" s="10" t="inlineStr"/>
-      <c r="AB86" s="11" t="inlineStr"/>
+      <c r="Z86" s="10" t="inlineStr"/>
+      <c r="AA86" s="11" t="inlineStr"/>
+      <c r="AB86" s="12" t="inlineStr"/>
     </row>
     <row r="87" ht="24" customHeight="1">
       <c r="A87" s="1" t="n"/>
@@ -5466,9 +5606,9 @@
       <c r="W87" s="8" t="inlineStr"/>
       <c r="X87" s="8" t="inlineStr"/>
       <c r="Y87" s="8" t="inlineStr"/>
-      <c r="Z87" s="9" t="inlineStr"/>
-      <c r="AA87" s="10" t="inlineStr"/>
-      <c r="AB87" s="11" t="inlineStr"/>
+      <c r="Z87" s="10" t="inlineStr"/>
+      <c r="AA87" s="11" t="inlineStr"/>
+      <c r="AB87" s="12" t="inlineStr"/>
     </row>
     <row r="88" ht="24" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
@@ -5560,11 +5700,11 @@
         </is>
       </c>
       <c r="Y89" s="8" t="inlineStr"/>
-      <c r="Z89" s="9" t="n">
+      <c r="Z89" s="10" t="n">
         <v>473.3333333333333</v>
       </c>
-      <c r="AA89" s="10" t="inlineStr"/>
-      <c r="AB89" s="11" t="inlineStr"/>
+      <c r="AA89" s="11" t="inlineStr"/>
+      <c r="AB89" s="12" t="inlineStr"/>
     </row>
     <row r="90" ht="24" customHeight="1">
       <c r="A90" s="1" t="n"/>
@@ -5600,9 +5740,9 @@
       <c r="W90" s="8" t="inlineStr"/>
       <c r="X90" s="8" t="inlineStr"/>
       <c r="Y90" s="8" t="inlineStr"/>
-      <c r="Z90" s="9" t="inlineStr"/>
-      <c r="AA90" s="10" t="inlineStr"/>
-      <c r="AB90" s="11" t="inlineStr"/>
+      <c r="Z90" s="10" t="inlineStr"/>
+      <c r="AA90" s="11" t="inlineStr"/>
+      <c r="AB90" s="12" t="inlineStr"/>
     </row>
     <row r="91" ht="24" customHeight="1">
       <c r="A91" s="1" t="n"/>
@@ -5646,13 +5786,13 @@
         </is>
       </c>
       <c r="Y91" s="8" t="inlineStr"/>
-      <c r="Z91" s="9" t="n">
+      <c r="Z91" s="10" t="n">
         <v>535.8333333333334</v>
       </c>
-      <c r="AA91" s="9" t="n">
+      <c r="AA91" s="10" t="n">
         <v>62.50000000000006</v>
       </c>
-      <c r="AB91" s="11" t="n">
+      <c r="AB91" s="12" t="n">
         <v>0.2282688093498906</v>
       </c>
     </row>
@@ -5750,11 +5890,11 @@
       <c r="W93" s="8" t="inlineStr"/>
       <c r="X93" s="8" t="inlineStr"/>
       <c r="Y93" s="8" t="inlineStr"/>
-      <c r="Z93" s="9" t="n">
+      <c r="Z93" s="10" t="n">
         <v>1430</v>
       </c>
-      <c r="AA93" s="10" t="inlineStr"/>
-      <c r="AB93" s="11" t="inlineStr"/>
+      <c r="AA93" s="11" t="inlineStr"/>
+      <c r="AB93" s="12" t="inlineStr"/>
     </row>
     <row r="94" ht="24" customHeight="1">
       <c r="A94" s="1" t="n"/>
@@ -5798,9 +5938,9 @@
       <c r="W94" s="8" t="inlineStr"/>
       <c r="X94" s="8" t="inlineStr"/>
       <c r="Y94" s="8" t="inlineStr"/>
-      <c r="Z94" s="9" t="inlineStr"/>
-      <c r="AA94" s="10" t="inlineStr"/>
-      <c r="AB94" s="11" t="inlineStr"/>
+      <c r="Z94" s="10" t="inlineStr"/>
+      <c r="AA94" s="11" t="inlineStr"/>
+      <c r="AB94" s="12" t="inlineStr"/>
     </row>
     <row r="95" ht="24" customHeight="1">
       <c r="A95" s="1" t="n"/>
@@ -5852,13 +5992,13 @@
       <c r="W95" s="8" t="inlineStr"/>
       <c r="X95" s="8" t="inlineStr"/>
       <c r="Y95" s="8" t="inlineStr"/>
-      <c r="Z95" s="9" t="n">
+      <c r="Z95" s="10" t="n">
         <v>1445</v>
       </c>
-      <c r="AA95" s="9" t="n">
+      <c r="AA95" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="AB95" s="11" t="n">
+      <c r="AB95" s="12" t="n">
         <v>0.005028494803888703</v>
       </c>
     </row>
@@ -5933,12 +6073,12 @@
         </is>
       </c>
       <c r="J97" s="8" t="inlineStr"/>
-      <c r="K97" s="12" t="inlineStr">
+      <c r="K97" s="9" t="inlineStr">
         <is>
           <t>4708.50</t>
         </is>
       </c>
-      <c r="L97" s="12" t="inlineStr">
+      <c r="L97" s="9" t="inlineStr">
         <is>
           <t>5913.50</t>
         </is>
@@ -5950,13 +6090,13 @@
           <t>5228.50</t>
         </is>
       </c>
-      <c r="P97" s="12" t="inlineStr"/>
+      <c r="P97" s="9" t="inlineStr"/>
       <c r="Q97" s="8" t="inlineStr">
         <is>
           <t>5599.00</t>
         </is>
       </c>
-      <c r="R97" s="12" t="inlineStr"/>
+      <c r="R97" s="9" t="inlineStr"/>
       <c r="S97" s="8" t="inlineStr"/>
       <c r="T97" s="8" t="inlineStr"/>
       <c r="U97" s="8" t="inlineStr"/>
@@ -5968,11 +6108,11 @@
         </is>
       </c>
       <c r="Y97" s="8" t="inlineStr"/>
-      <c r="Z97" s="9" t="n">
+      <c r="Z97" s="10" t="n">
         <v>5829.625</v>
       </c>
-      <c r="AA97" s="10" t="inlineStr"/>
-      <c r="AB97" s="11" t="inlineStr"/>
+      <c r="AA97" s="11" t="inlineStr"/>
+      <c r="AB97" s="12" t="inlineStr"/>
     </row>
     <row r="98" ht="24" customHeight="1">
       <c r="A98" s="1" t="n"/>
@@ -5989,12 +6129,12 @@
       <c r="H98" s="8" t="inlineStr"/>
       <c r="I98" s="8" t="inlineStr"/>
       <c r="J98" s="8" t="inlineStr"/>
-      <c r="K98" s="12" t="inlineStr">
+      <c r="K98" s="9" t="inlineStr">
         <is>
           <t>4851.00</t>
         </is>
       </c>
-      <c r="L98" s="12" t="inlineStr">
+      <c r="L98" s="9" t="inlineStr">
         <is>
           <t>6044.00</t>
         </is>
@@ -6002,9 +6142,9 @@
       <c r="M98" s="8" t="inlineStr"/>
       <c r="N98" s="8" t="inlineStr"/>
       <c r="O98" s="8" t="inlineStr"/>
-      <c r="P98" s="12" t="inlineStr"/>
+      <c r="P98" s="9" t="inlineStr"/>
       <c r="Q98" s="8" t="inlineStr"/>
-      <c r="R98" s="12" t="inlineStr"/>
+      <c r="R98" s="9" t="inlineStr"/>
       <c r="S98" s="8" t="inlineStr"/>
       <c r="T98" s="8" t="inlineStr"/>
       <c r="U98" s="8" t="inlineStr"/>
@@ -6016,9 +6156,9 @@
         </is>
       </c>
       <c r="Y98" s="8" t="inlineStr"/>
-      <c r="Z98" s="9" t="inlineStr"/>
-      <c r="AA98" s="10" t="inlineStr"/>
-      <c r="AB98" s="11" t="inlineStr"/>
+      <c r="Z98" s="10" t="inlineStr"/>
+      <c r="AA98" s="11" t="inlineStr"/>
+      <c r="AB98" s="12" t="inlineStr"/>
     </row>
     <row r="99" ht="24" customHeight="1">
       <c r="A99" s="1" t="n"/>
@@ -6039,12 +6179,12 @@
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="inlineStr"/>
       <c r="J99" s="8" t="inlineStr"/>
-      <c r="K99" s="12" t="inlineStr">
+      <c r="K99" s="9" t="inlineStr">
         <is>
           <t>5279.50</t>
         </is>
       </c>
-      <c r="L99" s="12" t="inlineStr">
+      <c r="L99" s="9" t="inlineStr">
         <is>
           <t>5889.50</t>
         </is>
@@ -6082,13 +6222,13 @@
         </is>
       </c>
       <c r="Y99" s="8" t="inlineStr"/>
-      <c r="Z99" s="9" t="n">
+      <c r="Z99" s="10" t="n">
         <v>6662.25</v>
       </c>
-      <c r="AA99" s="9" t="n">
+      <c r="AA99" s="10" t="n">
         <v>832.625</v>
       </c>
-      <c r="AB99" s="11" t="n">
+      <c r="AB99" s="12" t="n">
         <v>0.779976580796253</v>
       </c>
     </row>
@@ -6178,11 +6318,11 @@
       <c r="W101" s="8" t="inlineStr"/>
       <c r="X101" s="8" t="inlineStr"/>
       <c r="Y101" s="8" t="inlineStr"/>
-      <c r="Z101" s="9" t="n">
+      <c r="Z101" s="10" t="n">
         <v>25137.5</v>
       </c>
-      <c r="AA101" s="10" t="inlineStr"/>
-      <c r="AB101" s="11" t="inlineStr"/>
+      <c r="AA101" s="11" t="inlineStr"/>
+      <c r="AB101" s="12" t="inlineStr"/>
     </row>
     <row r="102" ht="24" customHeight="1">
       <c r="A102" s="1" t="n"/>
@@ -6218,9 +6358,9 @@
       <c r="W102" s="8" t="inlineStr"/>
       <c r="X102" s="8" t="inlineStr"/>
       <c r="Y102" s="8" t="inlineStr"/>
-      <c r="Z102" s="9" t="inlineStr"/>
-      <c r="AA102" s="10" t="inlineStr"/>
-      <c r="AB102" s="11" t="inlineStr"/>
+      <c r="Z102" s="10" t="inlineStr"/>
+      <c r="AA102" s="11" t="inlineStr"/>
+      <c r="AB102" s="12" t="inlineStr"/>
     </row>
     <row r="103" ht="24" customHeight="1">
       <c r="A103" s="1" t="n"/>
@@ -6260,13 +6400,13 @@
       <c r="W103" s="8" t="inlineStr"/>
       <c r="X103" s="8" t="inlineStr"/>
       <c r="Y103" s="8" t="inlineStr"/>
-      <c r="Z103" s="9" t="n">
+      <c r="Z103" s="10" t="n">
         <v>25177.5</v>
       </c>
-      <c r="AA103" s="9" t="n">
+      <c r="AA103" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="AB103" s="11" t="n">
+      <c r="AB103" s="12" t="n">
         <v>0.001779533584247569</v>
       </c>
     </row>
@@ -6304,9 +6444,9 @@
       <c r="W104" s="8" t="inlineStr"/>
       <c r="X104" s="8" t="inlineStr"/>
       <c r="Y104" s="8" t="inlineStr"/>
-      <c r="Z104" s="9" t="inlineStr"/>
-      <c r="AA104" s="10" t="inlineStr"/>
-      <c r="AB104" s="11" t="inlineStr"/>
+      <c r="Z104" s="10" t="inlineStr"/>
+      <c r="AA104" s="11" t="inlineStr"/>
+      <c r="AB104" s="12" t="inlineStr"/>
     </row>
     <row r="105" ht="24" customHeight="1">
       <c r="A105" s="1" t="n"/>
@@ -6342,9 +6482,9 @@
       <c r="W105" s="8" t="inlineStr"/>
       <c r="X105" s="8" t="inlineStr"/>
       <c r="Y105" s="8" t="inlineStr"/>
-      <c r="Z105" s="9" t="inlineStr"/>
-      <c r="AA105" s="10" t="inlineStr"/>
-      <c r="AB105" s="11" t="inlineStr"/>
+      <c r="Z105" s="10" t="inlineStr"/>
+      <c r="AA105" s="11" t="inlineStr"/>
+      <c r="AB105" s="12" t="inlineStr"/>
     </row>
     <row r="106" ht="24" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
@@ -6436,11 +6576,11 @@
       <c r="W107" s="8" t="inlineStr"/>
       <c r="X107" s="8" t="inlineStr"/>
       <c r="Y107" s="8" t="inlineStr"/>
-      <c r="Z107" s="9" t="n">
+      <c r="Z107" s="10" t="n">
         <v>2071</v>
       </c>
-      <c r="AA107" s="10" t="inlineStr"/>
-      <c r="AB107" s="11" t="inlineStr"/>
+      <c r="AA107" s="11" t="inlineStr"/>
+      <c r="AB107" s="12" t="inlineStr"/>
     </row>
     <row r="108" ht="24" customHeight="1">
       <c r="A108" s="1" t="n"/>
@@ -6476,9 +6616,9 @@
       <c r="W108" s="8" t="inlineStr"/>
       <c r="X108" s="8" t="inlineStr"/>
       <c r="Y108" s="8" t="inlineStr"/>
-      <c r="Z108" s="9" t="inlineStr"/>
-      <c r="AA108" s="10" t="inlineStr"/>
-      <c r="AB108" s="11" t="inlineStr"/>
+      <c r="Z108" s="10" t="inlineStr"/>
+      <c r="AA108" s="11" t="inlineStr"/>
+      <c r="AB108" s="12" t="inlineStr"/>
     </row>
     <row r="109" ht="24" customHeight="1">
       <c r="A109" s="1" t="n"/>
@@ -6518,13 +6658,13 @@
       <c r="W109" s="8" t="inlineStr"/>
       <c r="X109" s="8" t="inlineStr"/>
       <c r="Y109" s="8" t="inlineStr"/>
-      <c r="Z109" s="9" t="n">
+      <c r="Z109" s="10" t="n">
         <v>2068.25</v>
       </c>
-      <c r="AA109" s="9" t="n">
+      <c r="AA109" s="10" t="n">
         <v>2.75</v>
       </c>
-      <c r="AB109" s="11" t="n">
+      <c r="AB109" s="12" t="n">
         <v>-0.0004138885962403865</v>
       </c>
     </row>
@@ -6566,9 +6706,9 @@
       <c r="W110" s="8" t="inlineStr"/>
       <c r="X110" s="8" t="inlineStr"/>
       <c r="Y110" s="8" t="inlineStr"/>
-      <c r="Z110" s="9" t="inlineStr"/>
-      <c r="AA110" s="10" t="inlineStr"/>
-      <c r="AB110" s="11" t="inlineStr"/>
+      <c r="Z110" s="10" t="inlineStr"/>
+      <c r="AA110" s="11" t="inlineStr"/>
+      <c r="AB110" s="12" t="inlineStr"/>
     </row>
     <row r="111" ht="24" customHeight="1">
       <c r="A111" s="1" t="n"/>
@@ -6608,9 +6748,9 @@
       <c r="W111" s="8" t="inlineStr"/>
       <c r="X111" s="8" t="inlineStr"/>
       <c r="Y111" s="8" t="inlineStr"/>
-      <c r="Z111" s="9" t="inlineStr"/>
-      <c r="AA111" s="10" t="inlineStr"/>
-      <c r="AB111" s="11" t="inlineStr"/>
+      <c r="Z111" s="10" t="inlineStr"/>
+      <c r="AA111" s="11" t="inlineStr"/>
+      <c r="AB111" s="12" t="inlineStr"/>
     </row>
     <row r="112" ht="24" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
@@ -6702,11 +6842,11 @@
       <c r="W113" s="8" t="inlineStr"/>
       <c r="X113" s="8" t="inlineStr"/>
       <c r="Y113" s="8" t="inlineStr"/>
-      <c r="Z113" s="9" t="n">
+      <c r="Z113" s="10" t="n">
         <v>8.299999999999999</v>
       </c>
-      <c r="AA113" s="10" t="inlineStr"/>
-      <c r="AB113" s="11" t="inlineStr"/>
+      <c r="AA113" s="11" t="inlineStr"/>
+      <c r="AB113" s="12" t="inlineStr"/>
     </row>
     <row r="114" ht="24" customHeight="1">
       <c r="A114" s="1" t="n"/>
@@ -6758,13 +6898,13 @@
         </is>
       </c>
       <c r="Y114" s="8" t="inlineStr"/>
-      <c r="Z114" s="9" t="n">
+      <c r="Z114" s="10" t="n">
         <v>-0.6333333333333329</v>
       </c>
-      <c r="AA114" s="9" t="n">
+      <c r="AA114" s="10" t="n">
         <v>8.933333333333332</v>
       </c>
-      <c r="AB114" s="11" t="n">
+      <c r="AB114" s="12" t="n">
         <v>-0.2530689329556185</v>
       </c>
     </row>
@@ -6802,9 +6942,9 @@
       <c r="W115" s="8" t="inlineStr"/>
       <c r="X115" s="8" t="inlineStr"/>
       <c r="Y115" s="8" t="inlineStr"/>
-      <c r="Z115" s="9" t="inlineStr"/>
-      <c r="AA115" s="10" t="inlineStr"/>
-      <c r="AB115" s="11" t="inlineStr"/>
+      <c r="Z115" s="10" t="inlineStr"/>
+      <c r="AA115" s="11" t="inlineStr"/>
+      <c r="AB115" s="12" t="inlineStr"/>
     </row>
     <row r="116" ht="24" customHeight="1">
       <c r="A116" s="1" t="n"/>
@@ -6840,9 +6980,9 @@
       <c r="W116" s="8" t="inlineStr"/>
       <c r="X116" s="8" t="inlineStr"/>
       <c r="Y116" s="8" t="inlineStr"/>
-      <c r="Z116" s="9" t="inlineStr"/>
-      <c r="AA116" s="10" t="inlineStr"/>
-      <c r="AB116" s="11" t="inlineStr"/>
+      <c r="Z116" s="10" t="inlineStr"/>
+      <c r="AA116" s="11" t="inlineStr"/>
+      <c r="AB116" s="12" t="inlineStr"/>
     </row>
     <row r="117" ht="24" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
@@ -6915,7 +7055,7 @@
       <c r="L118" s="8" t="inlineStr"/>
       <c r="M118" s="8" t="inlineStr"/>
       <c r="N118" s="8" t="inlineStr"/>
-      <c r="O118" s="12" t="inlineStr">
+      <c r="O118" s="9" t="inlineStr">
         <is>
           <t>100.00</t>
         </is>
@@ -6930,7 +7070,7 @@
           <t>3551.75</t>
         </is>
       </c>
-      <c r="R118" s="12" t="inlineStr"/>
+      <c r="R118" s="9" t="inlineStr"/>
       <c r="S118" s="8" t="inlineStr"/>
       <c r="T118" s="8" t="inlineStr"/>
       <c r="U118" s="8" t="inlineStr"/>
@@ -6942,11 +7082,11 @@
         </is>
       </c>
       <c r="Y118" s="8" t="inlineStr"/>
-      <c r="Z118" s="9" t="n">
+      <c r="Z118" s="10" t="n">
         <v>1002.65</v>
       </c>
-      <c r="AA118" s="10" t="inlineStr"/>
-      <c r="AB118" s="11" t="inlineStr"/>
+      <c r="AA118" s="11" t="inlineStr"/>
+      <c r="AB118" s="12" t="inlineStr"/>
     </row>
     <row r="119" ht="24" customHeight="1">
       <c r="A119" s="1" t="n"/>
@@ -6971,7 +7111,7 @@
       <c r="L119" s="8" t="inlineStr"/>
       <c r="M119" s="8" t="inlineStr"/>
       <c r="N119" s="8" t="inlineStr"/>
-      <c r="O119" s="12" t="inlineStr">
+      <c r="O119" s="9" t="inlineStr">
         <is>
           <t>20.00</t>
         </is>
@@ -7002,13 +7142,13 @@
         </is>
       </c>
       <c r="Y119" s="8" t="inlineStr"/>
-      <c r="Z119" s="9" t="n">
+      <c r="Z119" s="10" t="n">
         <v>152.9875</v>
       </c>
-      <c r="AA119" s="9" t="n">
+      <c r="AA119" s="10" t="n">
         <v>849.6624999999999</v>
       </c>
-      <c r="AB119" s="11" t="n">
+      <c r="AB119" s="12" t="n">
         <v>-0.01221720319096315</v>
       </c>
     </row>
@@ -7077,7 +7217,7 @@
       <c r="F121" s="8" t="inlineStr"/>
       <c r="G121" s="8" t="inlineStr"/>
       <c r="H121" s="8" t="inlineStr"/>
-      <c r="I121" s="12" t="inlineStr">
+      <c r="I121" s="9" t="inlineStr">
         <is>
           <t>2940.00</t>
         </is>
@@ -7098,7 +7238,7 @@
       </c>
       <c r="P121" s="8" t="inlineStr"/>
       <c r="Q121" s="8" t="inlineStr"/>
-      <c r="R121" s="12" t="inlineStr"/>
+      <c r="R121" s="9" t="inlineStr"/>
       <c r="S121" s="8" t="inlineStr"/>
       <c r="T121" s="8" t="inlineStr"/>
       <c r="U121" s="8" t="inlineStr"/>
@@ -7106,11 +7246,11 @@
       <c r="W121" s="8" t="inlineStr"/>
       <c r="X121" s="8" t="inlineStr"/>
       <c r="Y121" s="8" t="inlineStr"/>
-      <c r="Z121" s="9" t="n">
+      <c r="Z121" s="10" t="n">
         <v>2859.0625</v>
       </c>
-      <c r="AA121" s="10" t="inlineStr"/>
-      <c r="AB121" s="11" t="inlineStr"/>
+      <c r="AA121" s="11" t="inlineStr"/>
+      <c r="AB121" s="12" t="inlineStr"/>
     </row>
     <row r="122" ht="24" customHeight="1">
       <c r="A122" s="1" t="n"/>
@@ -7133,7 +7273,7 @@
       <c r="F122" s="8" t="inlineStr"/>
       <c r="G122" s="8" t="inlineStr"/>
       <c r="H122" s="8" t="inlineStr"/>
-      <c r="I122" s="12" t="inlineStr">
+      <c r="I122" s="9" t="inlineStr">
         <is>
           <t>2553.75</t>
         </is>
@@ -7150,7 +7290,7 @@
       </c>
       <c r="P122" s="8" t="inlineStr"/>
       <c r="Q122" s="8" t="inlineStr"/>
-      <c r="R122" s="12" t="inlineStr"/>
+      <c r="R122" s="9" t="inlineStr"/>
       <c r="S122" s="8" t="inlineStr"/>
       <c r="T122" s="8" t="inlineStr"/>
       <c r="U122" s="8" t="inlineStr"/>
@@ -7158,9 +7298,9 @@
       <c r="W122" s="8" t="inlineStr"/>
       <c r="X122" s="8" t="inlineStr"/>
       <c r="Y122" s="8" t="inlineStr"/>
-      <c r="Z122" s="9" t="inlineStr"/>
-      <c r="AA122" s="10" t="inlineStr"/>
-      <c r="AB122" s="11" t="inlineStr"/>
+      <c r="Z122" s="10" t="inlineStr"/>
+      <c r="AA122" s="11" t="inlineStr"/>
+      <c r="AB122" s="12" t="inlineStr"/>
     </row>
     <row r="123" ht="24" customHeight="1">
       <c r="A123" s="1" t="n"/>
@@ -7183,7 +7323,7 @@
       <c r="F123" s="8" t="inlineStr"/>
       <c r="G123" s="8" t="inlineStr"/>
       <c r="H123" s="8" t="inlineStr"/>
-      <c r="I123" s="12" t="inlineStr">
+      <c r="I123" s="9" t="inlineStr">
         <is>
           <t>2338.75</t>
         </is>
@@ -7216,13 +7356,13 @@
       <c r="W123" s="8" t="inlineStr"/>
       <c r="X123" s="8" t="inlineStr"/>
       <c r="Y123" s="8" t="inlineStr"/>
-      <c r="Z123" s="9" t="n">
+      <c r="Z123" s="10" t="n">
         <v>3065.625</v>
       </c>
-      <c r="AA123" s="9" t="n">
+      <c r="AA123" s="10" t="n">
         <v>206.5625</v>
       </c>
-      <c r="AB123" s="11" t="n">
+      <c r="AB123" s="12" t="n">
         <v>0.01554141493179646</v>
       </c>
     </row>
@@ -7285,7 +7425,7 @@
       <c r="H125" s="8" t="inlineStr"/>
       <c r="I125" s="8" t="inlineStr"/>
       <c r="J125" s="8" t="inlineStr"/>
-      <c r="K125" s="12" t="inlineStr">
+      <c r="K125" s="9" t="inlineStr">
         <is>
           <t>8610.00</t>
         </is>
@@ -7316,11 +7456,11 @@
       <c r="W125" s="8" t="inlineStr"/>
       <c r="X125" s="8" t="inlineStr"/>
       <c r="Y125" s="8" t="inlineStr"/>
-      <c r="Z125" s="9" t="n">
+      <c r="Z125" s="10" t="n">
         <v>9045</v>
       </c>
-      <c r="AA125" s="10" t="inlineStr"/>
-      <c r="AB125" s="11" t="inlineStr"/>
+      <c r="AA125" s="11" t="inlineStr"/>
+      <c r="AB125" s="12" t="inlineStr"/>
     </row>
     <row r="126" ht="24" customHeight="1">
       <c r="A126" s="1" t="n"/>
@@ -7337,7 +7477,7 @@
       <c r="H126" s="8" t="inlineStr"/>
       <c r="I126" s="8" t="inlineStr"/>
       <c r="J126" s="8" t="inlineStr"/>
-      <c r="K126" s="12" t="inlineStr"/>
+      <c r="K126" s="9" t="inlineStr"/>
       <c r="L126" s="8" t="inlineStr"/>
       <c r="M126" s="8" t="inlineStr"/>
       <c r="N126" s="8" t="inlineStr"/>
@@ -7364,9 +7504,9 @@
       <c r="W126" s="8" t="inlineStr"/>
       <c r="X126" s="8" t="inlineStr"/>
       <c r="Y126" s="8" t="inlineStr"/>
-      <c r="Z126" s="9" t="inlineStr"/>
-      <c r="AA126" s="10" t="inlineStr"/>
-      <c r="AB126" s="11" t="inlineStr"/>
+      <c r="Z126" s="10" t="inlineStr"/>
+      <c r="AA126" s="11" t="inlineStr"/>
+      <c r="AB126" s="12" t="inlineStr"/>
     </row>
     <row r="127" ht="24" customHeight="1">
       <c r="A127" s="1" t="n"/>
@@ -7383,7 +7523,7 @@
       <c r="H127" s="8" t="inlineStr"/>
       <c r="I127" s="8" t="inlineStr"/>
       <c r="J127" s="8" t="inlineStr"/>
-      <c r="K127" s="12" t="inlineStr">
+      <c r="K127" s="9" t="inlineStr">
         <is>
           <t>8195.00</t>
         </is>
@@ -7418,13 +7558,13 @@
       <c r="W127" s="8" t="inlineStr"/>
       <c r="X127" s="8" t="inlineStr"/>
       <c r="Y127" s="8" t="inlineStr"/>
-      <c r="Z127" s="9" t="n">
+      <c r="Z127" s="10" t="n">
         <v>12731.66666666667</v>
       </c>
-      <c r="AA127" s="9" t="n">
+      <c r="AA127" s="10" t="n">
         <v>3686.666666666666</v>
       </c>
-      <c r="AB127" s="11" t="n">
+      <c r="AB127" s="12" t="n">
         <v>0.4706282845045849</v>
       </c>
     </row>
@@ -7518,11 +7658,11 @@
         </is>
       </c>
       <c r="Y129" s="8" t="inlineStr"/>
-      <c r="Z129" s="9" t="n">
+      <c r="Z129" s="10" t="n">
         <v>460.6666666666667</v>
       </c>
-      <c r="AA129" s="10" t="inlineStr"/>
-      <c r="AB129" s="11" t="inlineStr"/>
+      <c r="AA129" s="11" t="inlineStr"/>
+      <c r="AB129" s="12" t="inlineStr"/>
     </row>
     <row r="130" ht="24" customHeight="1">
       <c r="A130" s="1" t="n"/>
@@ -7562,9 +7702,9 @@
         </is>
       </c>
       <c r="Y130" s="8" t="inlineStr"/>
-      <c r="Z130" s="9" t="inlineStr"/>
-      <c r="AA130" s="10" t="inlineStr"/>
-      <c r="AB130" s="11" t="inlineStr"/>
+      <c r="Z130" s="10" t="inlineStr"/>
+      <c r="AA130" s="11" t="inlineStr"/>
+      <c r="AB130" s="12" t="inlineStr"/>
     </row>
     <row r="131" ht="24" customHeight="1">
       <c r="A131" s="1" t="n"/>
@@ -7608,13 +7748,13 @@
         </is>
       </c>
       <c r="Y131" s="8" t="inlineStr"/>
-      <c r="Z131" s="9" t="n">
+      <c r="Z131" s="10" t="n">
         <v>505.3333333333333</v>
       </c>
-      <c r="AA131" s="9" t="n">
+      <c r="AA131" s="10" t="n">
         <v>44.66666666666663</v>
       </c>
-      <c r="AB131" s="11" t="n">
+      <c r="AB131" s="12" t="n">
         <v>0.001063839077667397</v>
       </c>
     </row>
@@ -7652,9 +7792,9 @@
         </is>
       </c>
       <c r="Y132" s="8" t="inlineStr"/>
-      <c r="Z132" s="9" t="inlineStr"/>
-      <c r="AA132" s="10" t="inlineStr"/>
-      <c r="AB132" s="11" t="inlineStr"/>
+      <c r="Z132" s="10" t="inlineStr"/>
+      <c r="AA132" s="11" t="inlineStr"/>
+      <c r="AB132" s="12" t="inlineStr"/>
     </row>
     <row r="133" ht="24" customHeight="1">
       <c r="A133" s="1" t="n"/>
@@ -7690,9 +7830,9 @@
         </is>
       </c>
       <c r="Y133" s="8" t="inlineStr"/>
-      <c r="Z133" s="9" t="inlineStr"/>
-      <c r="AA133" s="10" t="inlineStr"/>
-      <c r="AB133" s="11" t="inlineStr"/>
+      <c r="Z133" s="10" t="inlineStr"/>
+      <c r="AA133" s="11" t="inlineStr"/>
+      <c r="AB133" s="12" t="inlineStr"/>
     </row>
     <row r="134" ht="24" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
@@ -7775,7 +7915,7 @@
           <t>6541.00, 6151.00, 6281.50, 5752.50</t>
         </is>
       </c>
-      <c r="Q135" s="12" t="inlineStr">
+      <c r="Q135" s="9" t="inlineStr">
         <is>
           <t>3203.50, 3308.00, 3088.00, 3095.00</t>
         </is>
@@ -7788,11 +7928,11 @@
       <c r="W135" s="8" t="inlineStr"/>
       <c r="X135" s="8" t="inlineStr"/>
       <c r="Y135" s="8" t="inlineStr"/>
-      <c r="Z135" s="9" t="n">
+      <c r="Z135" s="10" t="n">
         <v>5931.25</v>
       </c>
-      <c r="AA135" s="10" t="inlineStr"/>
-      <c r="AB135" s="11" t="inlineStr"/>
+      <c r="AA135" s="11" t="inlineStr"/>
+      <c r="AB135" s="12" t="inlineStr"/>
     </row>
     <row r="136" ht="24" customHeight="1">
       <c r="A136" s="1" t="n"/>
@@ -7823,7 +7963,7 @@
           <t>7178.00</t>
         </is>
       </c>
-      <c r="Q136" s="12" t="inlineStr">
+      <c r="Q136" s="9" t="inlineStr">
         <is>
           <t>3066.00</t>
         </is>
@@ -7836,9 +7976,9 @@
       <c r="W136" s="8" t="inlineStr"/>
       <c r="X136" s="8" t="inlineStr"/>
       <c r="Y136" s="8" t="inlineStr"/>
-      <c r="Z136" s="9" t="inlineStr"/>
-      <c r="AA136" s="10" t="inlineStr"/>
-      <c r="AB136" s="11" t="inlineStr"/>
+      <c r="Z136" s="10" t="inlineStr"/>
+      <c r="AA136" s="11" t="inlineStr"/>
+      <c r="AB136" s="12" t="inlineStr"/>
     </row>
     <row r="137" ht="24" customHeight="1">
       <c r="A137" s="1" t="n"/>
@@ -7869,7 +8009,7 @@
           <t>6658.00</t>
         </is>
       </c>
-      <c r="Q137" s="12" t="inlineStr">
+      <c r="Q137" s="9" t="inlineStr">
         <is>
           <t>2974.50</t>
         </is>
@@ -7886,13 +8026,13 @@
       <c r="W137" s="8" t="inlineStr"/>
       <c r="X137" s="8" t="inlineStr"/>
       <c r="Y137" s="8" t="inlineStr"/>
-      <c r="Z137" s="9" t="n">
+      <c r="Z137" s="10" t="n">
         <v>6350.5</v>
       </c>
-      <c r="AA137" s="9" t="n">
+      <c r="AA137" s="10" t="n">
         <v>419.25</v>
       </c>
-      <c r="AB137" s="11" t="n">
+      <c r="AB137" s="12" t="n">
         <v>0.03756787756052975</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[convert_csv_to_excel.py](/media/storage_data/ai2lab/choemj/STORM/results/convert_csv_to_excel.py)를 수정했습니다. 실행할 때 현재 모든 job queue를 읽어 예정 실험을 QUEUED와 파란색 배경으로 표시합니다. 큐에서 빠지면 다음 변환 때 표시도 사라집니다.
</commit_message>
<xml_diff>
--- a/results/converted_results.xlsx
+++ b/results/converted_results.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="+0.00;-0.00;0.00"/>
     <numFmt numFmtId="165" formatCode="+0.0000;-0.0000;0.0000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,7 +55,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00006100"/>
+      <color rgb="001F4E78"/>
       <sz val="16"/>
     </font>
     <font>
@@ -65,8 +65,14 @@
       <color rgb="00808080"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +87,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -159,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -180,8 +191,10 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -264,18 +277,18 @@
     <author>STORM</author>
   </authors>
   <commentList>
-    <comment ref="AB1" authorId="0" shapeId="0">
+    <comment ref="AE1" authorId="0" shapeId="0">
       <text>
         <t>Retrieval 미사용과 target: 16 양쪽에 유효한 점수가 있는 공통 시드만 사용합니다. update_tex.py의 EXCLUDED_SEEDS에 지정된 시드는 제외합니다. 각 시드에 여러 결과가 있으면 첫 번째 점수를 사용합니다.</t>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0" shapeId="0">
+    <comment ref="AF1" authorId="0" shapeId="0">
       <text>
         <t>STORM (논문) 행: Retrieval 미사용의 공통 시드 평균 − STORM 논문 점수.
 target: 16 행: |target: 16의 공통 시드 평균 − Retrieval 미사용의 공통 시드 평균|.</t>
       </text>
     </comment>
-    <comment ref="AD1" authorId="0" shapeId="0">
+    <comment ref="AG1" authorId="0" shapeId="0">
       <text>
         <t>STORM (논문) 행: (Retrieval 미사용 평균 − STORM 논문 점수) / (Human − Random).
 target: 16 행: (target: 16 평균 − Retrieval 미사용 평균) / (Human − Random).
@@ -452,6 +465,30 @@
 초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
+    <comment ref="T29" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:3
+python -u train.py -n "BankHeist-6050" -seed 6050 -config_path "config_files/STORM.yaml" -env_name "ALE/BankHeist-v5" -trajectory_path "D_TRAJ/BankHeist.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="U29" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:7
+python -u train.py -n "BankHeist-6060" -seed 6060 -config_path "config_files/STORM.yaml" -env_name "ALE/BankHeist-v5" -trajectory_path "D_TRAJ/BankHeist.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="V29" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:12
+python -u train.py -n "BankHeist-6070" -seed 6070 -config_path "config_files/STORM.yaml" -env_name "ALE/BankHeist-v5" -trajectory_path "D_TRAJ/BankHeist.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="Q30" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: BankHeist, seed 6020
@@ -588,6 +625,22 @@
     <comment ref="R41" authorId="0" shapeId="0">
       <text>
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="S41" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:8
+python -u train.py -n "Boxing-6040" -seed 6040 -config_path "config_files/STORM.yaml" -env_name "ALE/Boxing-v5" -trajectory_path "D_TRAJ/Boxing.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="T41" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:13
+python -u train.py -n "Boxing-6050" -seed 6050 -config_path "config_files/STORM.yaml" -env_name "ALE/Boxing-v5" -trajectory_path "D_TRAJ/Boxing.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
     <comment ref="O42" authorId="0" shapeId="0">
@@ -626,11 +679,27 @@
 초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
+    <comment ref="L57" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_3090.txt:1
+python -u train.py -n "CrazyClimber-2010" -seed 2010 -config_path "config_files/STORM.yaml" -env_name "ALE/CrazyClimber-v5" -trajectory_path "D_TRAJ/CrazyClimber.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="O57" authorId="0" shapeId="0">
       <text>
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
+    <comment ref="P57" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:11
+python -u train.py -n "CrazyClimber-6010" -seed 6010 -config_path "config_files/STORM.yaml" -env_name "ALE/CrazyClimber-v5" -trajectory_path "D_TRAJ/CrazyClimber.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="R67" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Freeway, seed 6030
@@ -643,6 +712,22 @@
         <t>EXCLUDED_SEEDS: Freeway, seed 6030
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
+      </text>
+    </comment>
+    <comment ref="C69" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_pro6k.txt:1
+python -u train.py -n "Freeway-1" -seed 1 -config_path "config_files/STORM.yaml" -env_name "ALE/Freeway-v5" -trajectory_path "D_TRAJ/Freeway.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="D69" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_pro6k.txt:4
+python -u train.py -n "Freeway-2" -seed 2 -config_path "config_files/STORM.yaml" -env_name "ALE/Freeway-v5" -trajectory_path "D_TRAJ/Freeway.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
     <comment ref="R69" authorId="0" shapeId="0">
@@ -653,6 +738,14 @@
 초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
+    <comment ref="AC69" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_titan.txt:2
+python -u train.py -n "Freeway-9999" -seed 9999 -config_path "config_files/STORM.yaml" -env_name "ALE/Freeway-v5" -trajectory_path "D_TRAJ/Freeway.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="R70" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Freeway, seed 6030
@@ -737,21 +830,21 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="V79" authorId="0" shapeId="0">
+    <comment ref="Y79" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9995
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="W79" authorId="0" shapeId="0">
+    <comment ref="Z79" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9996
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="Z79" authorId="0" shapeId="0">
+    <comment ref="AC79" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -793,21 +886,21 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="V80" authorId="0" shapeId="0">
+    <comment ref="Y80" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9995
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="W80" authorId="0" shapeId="0">
+    <comment ref="Z80" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9996
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="Z80" authorId="0" shapeId="0">
+    <comment ref="AC80" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -852,7 +945,31 @@
 초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
-    <comment ref="V81" authorId="0" shapeId="0">
+    <comment ref="T81" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:5
+python -u train.py -n "Gopher-6050" -seed 6050 -config_path "config_files/STORM.yaml" -env_name "ALE/Gopher-v5" -trajectory_path "D_TRAJ/Gopher.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="U81" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:9
+python -u train.py -n "Gopher-6060" -seed 6060 -config_path "config_files/STORM.yaml" -env_name "ALE/Gopher-v5" -trajectory_path "D_TRAJ/Gopher.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="X81" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_titan.txt:1
+python -u train.py -n "Gopher-9994" -seed 9994 -config_path "config_files/STORM.yaml" -env_name "ALE/Gopher-v5" -trajectory_path "D_TRAJ/Gopher.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="Y81" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9995
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -860,7 +977,7 @@
 초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
-    <comment ref="W81" authorId="0" shapeId="0">
+    <comment ref="Z81" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9996
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -868,12 +985,12 @@
 초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
-    <comment ref="X81" authorId="0" shapeId="0">
+    <comment ref="AA81" authorId="0" shapeId="0">
       <text>
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
-    <comment ref="Z81" authorId="0" shapeId="0">
+    <comment ref="AC81" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -915,21 +1032,21 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="V82" authorId="0" shapeId="0">
+    <comment ref="Y82" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9995
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="W82" authorId="0" shapeId="0">
+    <comment ref="Z82" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9996
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="Z82" authorId="0" shapeId="0">
+    <comment ref="AC82" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -971,21 +1088,21 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="V83" authorId="0" shapeId="0">
+    <comment ref="Y83" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9995
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="W83" authorId="0" shapeId="0">
+    <comment ref="Z83" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9996
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="Z83" authorId="0" shapeId="0">
+    <comment ref="AC83" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Gopher, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -1004,7 +1121,7 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="Z95" authorId="0" shapeId="0">
+    <comment ref="AC95" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Kangaroo, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -1018,13 +1135,21 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="Z96" authorId="0" shapeId="0">
+    <comment ref="AC96" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Kangaroo, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="C97" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_pro6k.txt:2
+python -u train.py -n "Kangaroo-1" -seed 1 -config_path "config_files/STORM.yaml" -env_name "ALE/Kangaroo-v5" -trajectory_path "D_TRAJ/Kangaroo.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="P97" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Kangaroo, seed 6010
@@ -1042,7 +1167,15 @@
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
-    <comment ref="Z97" authorId="0" shapeId="0">
+    <comment ref="S97" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:10
+python -u train.py -n "Kangaroo-6040" -seed 6040 -config_path "config_files/STORM.yaml" -env_name "ALE/Kangaroo-v5" -trajectory_path "D_TRAJ/Kangaroo.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="AC97" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Kangaroo, seed 9999
 STORM/results/update_tex.py의 EXCLUDED_SEEDS에 지정되어 공통 시드 평균, Δ Score, Δ HNS 및 LaTeX 결과 집계에서 제외되는 시드입니다.
@@ -1106,6 +1239,14 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="C101" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_pro6k.txt:3
+python -u train.py -n "Krull-1" -seed 1 -config_path "config_files/STORM.yaml" -env_name "ALE/Krull-v5" -trajectory_path "D_TRAJ/Krull.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="K101" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: Krull, seed 2000
@@ -1141,6 +1282,30 @@
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
+    <comment ref="T101" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:1
+STORM_AMP_DTYPE=fp16 python -u train.py -n "Krull-6050" -seed 6050 -config_path "config_files/STORM.yaml" -env_name "ALE/Krull-v5" -trajectory_path "D_TRAJ/Krull.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="U101" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:4
+python -u train.py -n "Krull-6060" -seed 6060 -config_path "config_files/STORM.yaml" -env_name "ALE/Krull-v5" -trajectory_path "D_TRAJ/Krull.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="AB101" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_titan.txt:4
+python -u train.py -n "Krull-9998" -seed 9998 -config_path "config_files/STORM.yaml" -env_name "ALE/Krull-v5" -trajectory_path "D_TRAJ/Krull.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="L105" authorId="0" shapeId="0">
       <text>
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
@@ -1160,7 +1325,7 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
-    <comment ref="Z116" authorId="0" shapeId="0">
+    <comment ref="AC116" authorId="0" shapeId="0">
       <text>
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
@@ -1258,6 +1423,13 @@
 취소선은 제외된 시드, 노란색 배경은 실행 중인 run을 뜻합니다.</t>
       </text>
     </comment>
+    <comment ref="S126" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:2
+python -u train.py --resume_warmup ckpt/RoadRunner-6040_Shared/shared_warmup_50507 -n RoadRunner-6040 -seed 6040 JointTrainAgent.Retrieval.enable "['baseline']"</t>
+      </text>
+    </comment>
     <comment ref="K127" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: RoadRunner, seed 2000
@@ -1301,6 +1473,22 @@
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
+    <comment ref="U128" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_A6000.txt:6
+python -u train.py -n "RoadRunner-6060" -seed 6060 -config_path "config_files/STORM.yaml" -env_name "ALE/RoadRunner-v5" -trajectory_path "D_TRAJ/RoadRunner.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
+    <comment ref="AC128" authorId="0" shapeId="0">
+      <text>
+        <t>QUEUED (파란색): 엑셀 생성 시 현재 job queue에 남아 있는 예정 실험입니다. RUNNING과 함께 있으면 실행 중을 뜻하는 노란색을 우선합니다. 기존 점수는 유지하며 대기 표시는 점수 집계에 포함하지 않습니다.
+job_queue_titan.txt:3
+python -u train.py -n "RoadRunner-9999" -seed 9999 -config_path "config_files/STORM.yaml" -env_name "ALE/RoadRunner-v5" -trajectory_path "D_TRAJ/RoadRunner.pkl" JointTrainAgent.Retrieval.enable "['retrieval']" JointTrainAgent.Retrieval.save_warmup True
+초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
+      </text>
+    </comment>
     <comment ref="Q136" authorId="0" shapeId="0">
       <text>
         <t>EXCLUDED_SEEDS: UpNDown, seed 6020
@@ -1327,7 +1515,7 @@
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
     </comment>
-    <comment ref="Z138" authorId="0" shapeId="0">
+    <comment ref="AC138" authorId="0" shapeId="0">
       <text>
         <t>초록색 테두리: 이 셀에 표시된 run 중 config 또는 실행 인자에서 JointTrainAgent.Retrieval.save_warmup=True인 run이 있습니다. 자식 분기는 재저장을 방지하기 위해 최종 config가 False일 수 있습니다.</t>
       </text>
@@ -1625,18 +1813,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD138"/>
+  <dimension ref="A1:AG138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27.5" customWidth="1" min="1" max="1"/>
     <col width="54.7" customWidth="1" min="2" max="2"/>
     <col width="3" customWidth="1" min="10" max="10"/>
     <col width="3" customWidth="1" min="13" max="13"/>
-    <col width="3" customWidth="1" min="21" max="21"/>
-    <col width="3" customWidth="1" min="27" max="27"/>
-    <col width="30" customWidth="1" min="28" max="28"/>
-    <col width="46" customWidth="1" min="29" max="29"/>
-    <col width="32" customWidth="1" min="30" max="30"/>
+    <col width="3" customWidth="1" min="23" max="23"/>
+    <col width="3" customWidth="1" min="30" max="30"/>
+    <col width="30" customWidth="1" min="31" max="31"/>
+    <col width="46" customWidth="1" min="32" max="32"/>
+    <col width="32" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1708,42 +1896,51 @@
       <c r="T1" s="1" t="n">
         <v>6050</v>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="n">
+        <v>6060</v>
+      </c>
+      <c r="V1" s="1" t="n">
+        <v>6070</v>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>    </t>
         </is>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="X1" s="1" t="n">
+        <v>9994</v>
+      </c>
+      <c r="Y1" s="1" t="n">
         <v>9995</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="Z1" s="1" t="n">
         <v>9996</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="AA1" s="1" t="n">
         <v>9997</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="AB1" s="1" t="n">
         <v>9998</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="AC1" s="1" t="n">
         <v>9999</v>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>   </t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Mean (공통 시드)</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Δ Score (행별 비교)</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Δ HNS (행별 비교)</t>
         </is>
@@ -1787,11 +1984,14 @@
       <c r="Y2" s="4" t="inlineStr"/>
       <c r="Z2" s="4" t="inlineStr"/>
       <c r="AA2" s="4" t="inlineStr"/>
-      <c r="AB2" s="5" t="inlineStr"/>
-      <c r="AC2" s="6" t="n">
+      <c r="AB2" s="4" t="inlineStr"/>
+      <c r="AC2" s="4" t="inlineStr"/>
+      <c r="AD2" s="4" t="inlineStr"/>
+      <c r="AE2" s="5" t="inlineStr"/>
+      <c r="AF2" s="6" t="n">
         <v>107.625</v>
       </c>
-      <c r="AD2" s="7" t="n">
+      <c r="AG2" s="7" t="n">
         <v>0.01559805214568327</v>
       </c>
     </row>
@@ -1851,11 +2051,14 @@
       <c r="Y3" s="8" t="inlineStr"/>
       <c r="Z3" s="8" t="inlineStr"/>
       <c r="AA3" s="8" t="inlineStr"/>
-      <c r="AB3" s="10" t="n">
+      <c r="AB3" s="8" t="inlineStr"/>
+      <c r="AC3" s="8" t="inlineStr"/>
+      <c r="AD3" s="8" t="inlineStr"/>
+      <c r="AE3" s="10" t="n">
         <v>1091.625</v>
       </c>
-      <c r="AC3" s="11" t="inlineStr"/>
-      <c r="AD3" s="12" t="inlineStr"/>
+      <c r="AF3" s="11" t="inlineStr"/>
+      <c r="AG3" s="12" t="inlineStr"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="1" t="n"/>
@@ -1905,9 +2108,12 @@
       <c r="Y4" s="8" t="inlineStr"/>
       <c r="Z4" s="8" t="inlineStr"/>
       <c r="AA4" s="8" t="inlineStr"/>
-      <c r="AB4" s="10" t="inlineStr"/>
-      <c r="AC4" s="11" t="inlineStr"/>
-      <c r="AD4" s="12" t="inlineStr"/>
+      <c r="AB4" s="8" t="inlineStr"/>
+      <c r="AC4" s="8" t="inlineStr"/>
+      <c r="AD4" s="8" t="inlineStr"/>
+      <c r="AE4" s="10" t="inlineStr"/>
+      <c r="AF4" s="11" t="inlineStr"/>
+      <c r="AG4" s="12" t="inlineStr"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="1" t="n"/>
@@ -1961,13 +2167,16 @@
       <c r="Y5" s="8" t="inlineStr"/>
       <c r="Z5" s="8" t="inlineStr"/>
       <c r="AA5" s="8" t="inlineStr"/>
-      <c r="AB5" s="10" t="n">
+      <c r="AB5" s="8" t="inlineStr"/>
+      <c r="AC5" s="8" t="inlineStr"/>
+      <c r="AD5" s="8" t="inlineStr"/>
+      <c r="AE5" s="10" t="n">
         <v>1147.875</v>
       </c>
-      <c r="AC5" s="10" t="n">
+      <c r="AF5" s="10" t="n">
         <v>56.25</v>
       </c>
-      <c r="AD5" s="12" t="n">
+      <c r="AG5" s="12" t="n">
         <v>0.0081522920622038</v>
       </c>
     </row>
@@ -2007,9 +2216,12 @@
       <c r="Y6" s="8" t="inlineStr"/>
       <c r="Z6" s="8" t="inlineStr"/>
       <c r="AA6" s="8" t="inlineStr"/>
-      <c r="AB6" s="10" t="inlineStr"/>
-      <c r="AC6" s="11" t="inlineStr"/>
-      <c r="AD6" s="12" t="inlineStr"/>
+      <c r="AB6" s="8" t="inlineStr"/>
+      <c r="AC6" s="8" t="inlineStr"/>
+      <c r="AD6" s="8" t="inlineStr"/>
+      <c r="AE6" s="10" t="inlineStr"/>
+      <c r="AF6" s="11" t="inlineStr"/>
+      <c r="AG6" s="12" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="1" t="n"/>
@@ -2047,9 +2259,12 @@
       <c r="Y7" s="8" t="inlineStr"/>
       <c r="Z7" s="8" t="inlineStr"/>
       <c r="AA7" s="8" t="inlineStr"/>
-      <c r="AB7" s="10" t="inlineStr"/>
-      <c r="AC7" s="11" t="inlineStr"/>
-      <c r="AD7" s="12" t="inlineStr"/>
+      <c r="AB7" s="8" t="inlineStr"/>
+      <c r="AC7" s="8" t="inlineStr"/>
+      <c r="AD7" s="8" t="inlineStr"/>
+      <c r="AE7" s="10" t="inlineStr"/>
+      <c r="AF7" s="11" t="inlineStr"/>
+      <c r="AG7" s="12" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -2089,11 +2304,14 @@
       <c r="Y8" s="4" t="inlineStr"/>
       <c r="Z8" s="4" t="inlineStr"/>
       <c r="AA8" s="4" t="inlineStr"/>
-      <c r="AB8" s="5" t="inlineStr"/>
-      <c r="AC8" s="6" t="n">
+      <c r="AB8" s="4" t="inlineStr"/>
+      <c r="AC8" s="4" t="inlineStr"/>
+      <c r="AD8" s="4" t="inlineStr"/>
+      <c r="AE8" s="5" t="inlineStr"/>
+      <c r="AF8" s="6" t="n">
         <v>3.599999999999994</v>
       </c>
-      <c r="AD8" s="7" t="n">
+      <c r="AG8" s="7" t="n">
         <v>0.002100717745229617</v>
       </c>
     </row>
@@ -2153,11 +2371,14 @@
       <c r="Y9" s="8" t="inlineStr"/>
       <c r="Z9" s="8" t="inlineStr"/>
       <c r="AA9" s="8" t="inlineStr"/>
-      <c r="AB9" s="10" t="n">
+      <c r="AB9" s="8" t="inlineStr"/>
+      <c r="AC9" s="8" t="inlineStr"/>
+      <c r="AD9" s="8" t="inlineStr"/>
+      <c r="AE9" s="10" t="n">
         <v>208.6</v>
       </c>
-      <c r="AC9" s="11" t="inlineStr"/>
-      <c r="AD9" s="12" t="inlineStr"/>
+      <c r="AF9" s="11" t="inlineStr"/>
+      <c r="AG9" s="12" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -2207,9 +2428,12 @@
       <c r="Y10" s="8" t="inlineStr"/>
       <c r="Z10" s="8" t="inlineStr"/>
       <c r="AA10" s="8" t="inlineStr"/>
-      <c r="AB10" s="10" t="inlineStr"/>
-      <c r="AC10" s="11" t="inlineStr"/>
-      <c r="AD10" s="12" t="inlineStr"/>
+      <c r="AB10" s="8" t="inlineStr"/>
+      <c r="AC10" s="8" t="inlineStr"/>
+      <c r="AD10" s="8" t="inlineStr"/>
+      <c r="AE10" s="10" t="inlineStr"/>
+      <c r="AF10" s="11" t="inlineStr"/>
+      <c r="AG10" s="12" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="1" t="n"/>
@@ -2263,13 +2487,16 @@
       <c r="Y11" s="8" t="inlineStr"/>
       <c r="Z11" s="8" t="inlineStr"/>
       <c r="AA11" s="8" t="inlineStr"/>
-      <c r="AB11" s="10" t="n">
+      <c r="AB11" s="8" t="inlineStr"/>
+      <c r="AC11" s="8" t="inlineStr"/>
+      <c r="AD11" s="8" t="inlineStr"/>
+      <c r="AE11" s="10" t="n">
         <v>169.15</v>
       </c>
-      <c r="AC11" s="10" t="n">
+      <c r="AF11" s="10" t="n">
         <v>39.44999999999999</v>
       </c>
-      <c r="AD11" s="12" t="n">
+      <c r="AG11" s="12" t="n">
         <v>-0.02302036529147458</v>
       </c>
     </row>
@@ -2309,9 +2536,12 @@
       <c r="Y12" s="8" t="inlineStr"/>
       <c r="Z12" s="8" t="inlineStr"/>
       <c r="AA12" s="8" t="inlineStr"/>
-      <c r="AB12" s="10" t="inlineStr"/>
-      <c r="AC12" s="11" t="inlineStr"/>
-      <c r="AD12" s="12" t="inlineStr"/>
+      <c r="AB12" s="8" t="inlineStr"/>
+      <c r="AC12" s="8" t="inlineStr"/>
+      <c r="AD12" s="8" t="inlineStr"/>
+      <c r="AE12" s="10" t="inlineStr"/>
+      <c r="AF12" s="11" t="inlineStr"/>
+      <c r="AG12" s="12" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="1" t="n"/>
@@ -2349,9 +2579,12 @@
       <c r="Y13" s="8" t="inlineStr"/>
       <c r="Z13" s="8" t="inlineStr"/>
       <c r="AA13" s="8" t="inlineStr"/>
-      <c r="AB13" s="10" t="inlineStr"/>
-      <c r="AC13" s="11" t="inlineStr"/>
-      <c r="AD13" s="12" t="inlineStr"/>
+      <c r="AB13" s="8" t="inlineStr"/>
+      <c r="AC13" s="8" t="inlineStr"/>
+      <c r="AD13" s="8" t="inlineStr"/>
+      <c r="AE13" s="10" t="inlineStr"/>
+      <c r="AF13" s="11" t="inlineStr"/>
+      <c r="AG13" s="12" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -2391,11 +2624,14 @@
       <c r="Y14" s="4" t="inlineStr"/>
       <c r="Z14" s="4" t="inlineStr"/>
       <c r="AA14" s="4" t="inlineStr"/>
-      <c r="AB14" s="5" t="inlineStr"/>
-      <c r="AC14" s="6" t="n">
+      <c r="AB14" s="4" t="inlineStr"/>
+      <c r="AC14" s="4" t="inlineStr"/>
+      <c r="AD14" s="4" t="inlineStr"/>
+      <c r="AE14" s="5" t="inlineStr"/>
+      <c r="AF14" s="6" t="n">
         <v>20.11249999999995</v>
       </c>
-      <c r="AD14" s="7" t="n">
+      <c r="AG14" s="7" t="n">
         <v>0.03870765973826011</v>
       </c>
     </row>
@@ -2455,11 +2691,14 @@
       <c r="Y15" s="8" t="inlineStr"/>
       <c r="Z15" s="8" t="inlineStr"/>
       <c r="AA15" s="8" t="inlineStr"/>
-      <c r="AB15" s="10" t="n">
+      <c r="AB15" s="8" t="inlineStr"/>
+      <c r="AC15" s="8" t="inlineStr"/>
+      <c r="AD15" s="8" t="inlineStr"/>
+      <c r="AE15" s="10" t="n">
         <v>821.1125</v>
       </c>
-      <c r="AC15" s="11" t="inlineStr"/>
-      <c r="AD15" s="12" t="inlineStr"/>
+      <c r="AF15" s="11" t="inlineStr"/>
+      <c r="AG15" s="12" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="1" t="n"/>
@@ -2509,9 +2748,12 @@
       <c r="Y16" s="8" t="inlineStr"/>
       <c r="Z16" s="8" t="inlineStr"/>
       <c r="AA16" s="8" t="inlineStr"/>
-      <c r="AB16" s="10" t="inlineStr"/>
-      <c r="AC16" s="11" t="inlineStr"/>
-      <c r="AD16" s="12" t="inlineStr"/>
+      <c r="AB16" s="8" t="inlineStr"/>
+      <c r="AC16" s="8" t="inlineStr"/>
+      <c r="AD16" s="8" t="inlineStr"/>
+      <c r="AE16" s="10" t="inlineStr"/>
+      <c r="AF16" s="11" t="inlineStr"/>
+      <c r="AG16" s="12" t="inlineStr"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="1" t="n"/>
@@ -2577,13 +2819,16 @@
       <c r="Y17" s="8" t="inlineStr"/>
       <c r="Z17" s="8" t="inlineStr"/>
       <c r="AA17" s="8" t="inlineStr"/>
-      <c r="AB17" s="10" t="n">
+      <c r="AB17" s="8" t="inlineStr"/>
+      <c r="AC17" s="8" t="inlineStr"/>
+      <c r="AD17" s="8" t="inlineStr"/>
+      <c r="AE17" s="10" t="n">
         <v>723.6625</v>
       </c>
-      <c r="AC17" s="10" t="n">
+      <c r="AF17" s="10" t="n">
         <v>97.44999999999993</v>
       </c>
-      <c r="AD17" s="12" t="n">
+      <c r="AG17" s="12" t="n">
         <v>-0.1875481139337951</v>
       </c>
     </row>
@@ -2623,9 +2868,12 @@
       <c r="Y18" s="8" t="inlineStr"/>
       <c r="Z18" s="8" t="inlineStr"/>
       <c r="AA18" s="8" t="inlineStr"/>
-      <c r="AB18" s="10" t="inlineStr"/>
-      <c r="AC18" s="11" t="inlineStr"/>
-      <c r="AD18" s="12" t="inlineStr"/>
+      <c r="AB18" s="8" t="inlineStr"/>
+      <c r="AC18" s="8" t="inlineStr"/>
+      <c r="AD18" s="8" t="inlineStr"/>
+      <c r="AE18" s="10" t="inlineStr"/>
+      <c r="AF18" s="11" t="inlineStr"/>
+      <c r="AG18" s="12" t="inlineStr"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="1" t="n"/>
@@ -2663,9 +2911,12 @@
       <c r="Y19" s="8" t="inlineStr"/>
       <c r="Z19" s="8" t="inlineStr"/>
       <c r="AA19" s="8" t="inlineStr"/>
-      <c r="AB19" s="10" t="inlineStr"/>
-      <c r="AC19" s="11" t="inlineStr"/>
-      <c r="AD19" s="12" t="inlineStr"/>
+      <c r="AB19" s="8" t="inlineStr"/>
+      <c r="AC19" s="8" t="inlineStr"/>
+      <c r="AD19" s="8" t="inlineStr"/>
+      <c r="AE19" s="10" t="inlineStr"/>
+      <c r="AF19" s="11" t="inlineStr"/>
+      <c r="AG19" s="12" t="inlineStr"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2705,11 +2956,14 @@
       <c r="Y20" s="4" t="inlineStr"/>
       <c r="Z20" s="4" t="inlineStr"/>
       <c r="AA20" s="4" t="inlineStr"/>
-      <c r="AB20" s="5" t="inlineStr"/>
-      <c r="AC20" s="6" t="n">
+      <c r="AB20" s="4" t="inlineStr"/>
+      <c r="AC20" s="4" t="inlineStr"/>
+      <c r="AD20" s="4" t="inlineStr"/>
+      <c r="AE20" s="5" t="inlineStr"/>
+      <c r="AF20" s="6" t="n">
         <v>-350.5</v>
       </c>
-      <c r="AD20" s="7" t="n">
+      <c r="AG20" s="7" t="n">
         <v>-0.04226303160382478</v>
       </c>
     </row>
@@ -2765,11 +3019,14 @@
       <c r="Y21" s="8" t="inlineStr"/>
       <c r="Z21" s="8" t="inlineStr"/>
       <c r="AA21" s="8" t="inlineStr"/>
-      <c r="AB21" s="10" t="n">
+      <c r="AB21" s="8" t="inlineStr"/>
+      <c r="AC21" s="8" t="inlineStr"/>
+      <c r="AD21" s="8" t="inlineStr"/>
+      <c r="AE21" s="10" t="n">
         <v>677.5</v>
       </c>
-      <c r="AC21" s="11" t="inlineStr"/>
-      <c r="AD21" s="12" t="inlineStr"/>
+      <c r="AF21" s="11" t="inlineStr"/>
+      <c r="AG21" s="12" t="inlineStr"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="1" t="n"/>
@@ -2815,9 +3072,12 @@
       <c r="Y22" s="8" t="inlineStr"/>
       <c r="Z22" s="8" t="inlineStr"/>
       <c r="AA22" s="8" t="inlineStr"/>
-      <c r="AB22" s="10" t="inlineStr"/>
-      <c r="AC22" s="11" t="inlineStr"/>
-      <c r="AD22" s="12" t="inlineStr"/>
+      <c r="AB22" s="8" t="inlineStr"/>
+      <c r="AC22" s="8" t="inlineStr"/>
+      <c r="AD22" s="8" t="inlineStr"/>
+      <c r="AE22" s="10" t="inlineStr"/>
+      <c r="AF22" s="11" t="inlineStr"/>
+      <c r="AG22" s="12" t="inlineStr"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="1" t="n"/>
@@ -2867,13 +3127,16 @@
       <c r="Y23" s="8" t="inlineStr"/>
       <c r="Z23" s="8" t="inlineStr"/>
       <c r="AA23" s="8" t="inlineStr"/>
-      <c r="AB23" s="10" t="n">
+      <c r="AB23" s="8" t="inlineStr"/>
+      <c r="AC23" s="8" t="inlineStr"/>
+      <c r="AD23" s="8" t="inlineStr"/>
+      <c r="AE23" s="10" t="n">
         <v>759.375</v>
       </c>
-      <c r="AC23" s="10" t="n">
+      <c r="AF23" s="10" t="n">
         <v>81.875</v>
       </c>
-      <c r="AD23" s="12" t="n">
+      <c r="AG23" s="12" t="n">
         <v>0.009872427139980468</v>
       </c>
     </row>
@@ -2913,9 +3176,12 @@
       <c r="Y24" s="8" t="inlineStr"/>
       <c r="Z24" s="8" t="inlineStr"/>
       <c r="AA24" s="8" t="inlineStr"/>
-      <c r="AB24" s="10" t="inlineStr"/>
-      <c r="AC24" s="11" t="inlineStr"/>
-      <c r="AD24" s="12" t="inlineStr"/>
+      <c r="AB24" s="8" t="inlineStr"/>
+      <c r="AC24" s="8" t="inlineStr"/>
+      <c r="AD24" s="8" t="inlineStr"/>
+      <c r="AE24" s="10" t="inlineStr"/>
+      <c r="AF24" s="11" t="inlineStr"/>
+      <c r="AG24" s="12" t="inlineStr"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="1" t="n"/>
@@ -2953,9 +3219,12 @@
       <c r="Y25" s="8" t="inlineStr"/>
       <c r="Z25" s="8" t="inlineStr"/>
       <c r="AA25" s="8" t="inlineStr"/>
-      <c r="AB25" s="10" t="inlineStr"/>
-      <c r="AC25" s="11" t="inlineStr"/>
-      <c r="AD25" s="12" t="inlineStr"/>
+      <c r="AB25" s="8" t="inlineStr"/>
+      <c r="AC25" s="8" t="inlineStr"/>
+      <c r="AD25" s="8" t="inlineStr"/>
+      <c r="AE25" s="10" t="inlineStr"/>
+      <c r="AF25" s="11" t="inlineStr"/>
+      <c r="AG25" s="12" t="inlineStr"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2995,11 +3264,14 @@
       <c r="Y26" s="4" t="inlineStr"/>
       <c r="Z26" s="4" t="inlineStr"/>
       <c r="AA26" s="4" t="inlineStr"/>
-      <c r="AB26" s="5" t="inlineStr"/>
-      <c r="AC26" s="6" t="n">
+      <c r="AB26" s="4" t="inlineStr"/>
+      <c r="AC26" s="4" t="inlineStr"/>
+      <c r="AD26" s="4" t="inlineStr"/>
+      <c r="AE26" s="5" t="inlineStr"/>
+      <c r="AF26" s="6" t="n">
         <v>-84.75</v>
       </c>
-      <c r="AD26" s="7" t="n">
+      <c r="AG26" s="7" t="n">
         <v>-0.1146975233455136</v>
       </c>
     </row>
@@ -3056,22 +3328,25 @@
       <c r="V27" s="8" t="inlineStr"/>
       <c r="W27" s="8" t="inlineStr"/>
       <c r="X27" s="8" t="inlineStr"/>
-      <c r="Y27" s="8" t="inlineStr">
+      <c r="Y27" s="8" t="inlineStr"/>
+      <c r="Z27" s="8" t="inlineStr"/>
+      <c r="AA27" s="8" t="inlineStr"/>
+      <c r="AB27" s="8" t="inlineStr">
         <is>
           <t>694.50</t>
         </is>
       </c>
-      <c r="Z27" s="8" t="inlineStr">
+      <c r="AC27" s="8" t="inlineStr">
         <is>
           <t>668.50</t>
         </is>
       </c>
-      <c r="AA27" s="8" t="inlineStr"/>
-      <c r="AB27" s="10" t="n">
+      <c r="AD27" s="8" t="inlineStr"/>
+      <c r="AE27" s="10" t="n">
         <v>556.25</v>
       </c>
-      <c r="AC27" s="11" t="inlineStr"/>
-      <c r="AD27" s="12" t="inlineStr"/>
+      <c r="AF27" s="11" t="inlineStr"/>
+      <c r="AG27" s="12" t="inlineStr"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="1" t="n"/>
@@ -3103,15 +3378,18 @@
       <c r="W28" s="8" t="inlineStr"/>
       <c r="X28" s="8" t="inlineStr"/>
       <c r="Y28" s="8" t="inlineStr"/>
-      <c r="Z28" s="8" t="inlineStr">
+      <c r="Z28" s="8" t="inlineStr"/>
+      <c r="AA28" s="8" t="inlineStr"/>
+      <c r="AB28" s="8" t="inlineStr"/>
+      <c r="AC28" s="8" t="inlineStr">
         <is>
           <t>507.50</t>
         </is>
       </c>
-      <c r="AA28" s="8" t="inlineStr"/>
-      <c r="AB28" s="10" t="inlineStr"/>
-      <c r="AC28" s="11" t="inlineStr"/>
-      <c r="AD28" s="12" t="inlineStr"/>
+      <c r="AD28" s="8" t="inlineStr"/>
+      <c r="AE28" s="10" t="inlineStr"/>
+      <c r="AF28" s="11" t="inlineStr"/>
+      <c r="AG28" s="12" t="inlineStr"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="1" t="n"/>
@@ -3157,29 +3435,44 @@
           <t>179.00</t>
         </is>
       </c>
-      <c r="T29" s="8" t="inlineStr"/>
-      <c r="U29" s="8" t="inlineStr"/>
-      <c r="V29" s="8" t="inlineStr"/>
+      <c r="T29" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="U29" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="V29" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="W29" s="8" t="inlineStr"/>
       <c r="X29" s="8" t="inlineStr"/>
-      <c r="Y29" s="8" t="inlineStr">
+      <c r="Y29" s="8" t="inlineStr"/>
+      <c r="Z29" s="8" t="inlineStr"/>
+      <c r="AA29" s="8" t="inlineStr"/>
+      <c r="AB29" s="8" t="inlineStr">
         <is>
           <t>566.00</t>
         </is>
       </c>
-      <c r="Z29" s="8" t="inlineStr">
+      <c r="AC29" s="8" t="inlineStr">
         <is>
           <t>565.00</t>
         </is>
       </c>
-      <c r="AA29" s="8" t="inlineStr"/>
-      <c r="AB29" s="10" t="n">
+      <c r="AD29" s="8" t="inlineStr"/>
+      <c r="AE29" s="10" t="n">
         <v>483.5</v>
       </c>
-      <c r="AC29" s="10" t="n">
+      <c r="AF29" s="10" t="n">
         <v>72.75</v>
       </c>
-      <c r="AD29" s="12" t="n">
+      <c r="AG29" s="12" t="n">
         <v>-0.09845716605765327</v>
       </c>
     </row>
@@ -3213,15 +3506,18 @@
       <c r="W30" s="8" t="inlineStr"/>
       <c r="X30" s="8" t="inlineStr"/>
       <c r="Y30" s="8" t="inlineStr"/>
-      <c r="Z30" s="8" t="inlineStr">
+      <c r="Z30" s="8" t="inlineStr"/>
+      <c r="AA30" s="8" t="inlineStr"/>
+      <c r="AB30" s="8" t="inlineStr"/>
+      <c r="AC30" s="8" t="inlineStr">
         <is>
           <t>652.50</t>
         </is>
       </c>
-      <c r="AA30" s="8" t="inlineStr"/>
-      <c r="AB30" s="10" t="inlineStr"/>
-      <c r="AC30" s="11" t="inlineStr"/>
-      <c r="AD30" s="12" t="inlineStr"/>
+      <c r="AD30" s="8" t="inlineStr"/>
+      <c r="AE30" s="10" t="inlineStr"/>
+      <c r="AF30" s="11" t="inlineStr"/>
+      <c r="AG30" s="12" t="inlineStr"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="1" t="n"/>
@@ -3253,15 +3549,18 @@
       <c r="W31" s="8" t="inlineStr"/>
       <c r="X31" s="8" t="inlineStr"/>
       <c r="Y31" s="8" t="inlineStr"/>
-      <c r="Z31" s="8" t="inlineStr">
+      <c r="Z31" s="8" t="inlineStr"/>
+      <c r="AA31" s="8" t="inlineStr"/>
+      <c r="AB31" s="8" t="inlineStr"/>
+      <c r="AC31" s="8" t="inlineStr">
         <is>
           <t>381.50</t>
         </is>
       </c>
-      <c r="AA31" s="8" t="inlineStr"/>
-      <c r="AB31" s="10" t="inlineStr"/>
-      <c r="AC31" s="11" t="inlineStr"/>
-      <c r="AD31" s="12" t="inlineStr"/>
+      <c r="AD31" s="8" t="inlineStr"/>
+      <c r="AE31" s="10" t="inlineStr"/>
+      <c r="AF31" s="11" t="inlineStr"/>
+      <c r="AG31" s="12" t="inlineStr"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -3301,11 +3600,14 @@
       <c r="Y32" s="4" t="inlineStr"/>
       <c r="Z32" s="4" t="inlineStr"/>
       <c r="AA32" s="4" t="inlineStr"/>
-      <c r="AB32" s="5" t="inlineStr"/>
-      <c r="AC32" s="6" t="n">
+      <c r="AB32" s="4" t="inlineStr"/>
+      <c r="AC32" s="4" t="inlineStr"/>
+      <c r="AD32" s="4" t="inlineStr"/>
+      <c r="AE32" s="5" t="inlineStr"/>
+      <c r="AF32" s="6" t="n">
         <v>-1327.5</v>
       </c>
-      <c r="AD32" s="7" t="n">
+      <c r="AG32" s="7" t="n">
         <v>-0.03811643098126481</v>
       </c>
     </row>
@@ -3365,11 +3667,14 @@
       <c r="Y33" s="8" t="inlineStr"/>
       <c r="Z33" s="8" t="inlineStr"/>
       <c r="AA33" s="8" t="inlineStr"/>
-      <c r="AB33" s="10" t="n">
+      <c r="AB33" s="8" t="inlineStr"/>
+      <c r="AC33" s="8" t="inlineStr"/>
+      <c r="AD33" s="8" t="inlineStr"/>
+      <c r="AE33" s="10" t="n">
         <v>12212.5</v>
       </c>
-      <c r="AC33" s="11" t="inlineStr"/>
-      <c r="AD33" s="12" t="inlineStr"/>
+      <c r="AF33" s="11" t="inlineStr"/>
+      <c r="AG33" s="12" t="inlineStr"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="1" t="n"/>
@@ -3423,9 +3728,12 @@
       <c r="Y34" s="8" t="inlineStr"/>
       <c r="Z34" s="8" t="inlineStr"/>
       <c r="AA34" s="8" t="inlineStr"/>
-      <c r="AB34" s="10" t="inlineStr"/>
-      <c r="AC34" s="11" t="inlineStr"/>
-      <c r="AD34" s="12" t="inlineStr"/>
+      <c r="AB34" s="8" t="inlineStr"/>
+      <c r="AC34" s="8" t="inlineStr"/>
+      <c r="AD34" s="8" t="inlineStr"/>
+      <c r="AE34" s="10" t="inlineStr"/>
+      <c r="AF34" s="11" t="inlineStr"/>
+      <c r="AG34" s="12" t="inlineStr"/>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="1" t="n"/>
@@ -3483,13 +3791,16 @@
       <c r="Y35" s="8" t="inlineStr"/>
       <c r="Z35" s="8" t="inlineStr"/>
       <c r="AA35" s="8" t="inlineStr"/>
-      <c r="AB35" s="10" t="n">
+      <c r="AB35" s="8" t="inlineStr"/>
+      <c r="AC35" s="8" t="inlineStr"/>
+      <c r="AD35" s="8" t="inlineStr"/>
+      <c r="AE35" s="10" t="n">
         <v>13125</v>
       </c>
-      <c r="AC35" s="10" t="n">
+      <c r="AF35" s="10" t="n">
         <v>912.5</v>
       </c>
-      <c r="AD35" s="12" t="n">
+      <c r="AG35" s="12" t="n">
         <v>0.026200559902376</v>
       </c>
     </row>
@@ -3533,9 +3844,12 @@
       <c r="Y36" s="8" t="inlineStr"/>
       <c r="Z36" s="8" t="inlineStr"/>
       <c r="AA36" s="8" t="inlineStr"/>
-      <c r="AB36" s="10" t="inlineStr"/>
-      <c r="AC36" s="11" t="inlineStr"/>
-      <c r="AD36" s="12" t="inlineStr"/>
+      <c r="AB36" s="8" t="inlineStr"/>
+      <c r="AC36" s="8" t="inlineStr"/>
+      <c r="AD36" s="8" t="inlineStr"/>
+      <c r="AE36" s="10" t="inlineStr"/>
+      <c r="AF36" s="11" t="inlineStr"/>
+      <c r="AG36" s="12" t="inlineStr"/>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="1" t="n"/>
@@ -3577,9 +3891,12 @@
       <c r="Y37" s="8" t="inlineStr"/>
       <c r="Z37" s="8" t="inlineStr"/>
       <c r="AA37" s="8" t="inlineStr"/>
-      <c r="AB37" s="10" t="inlineStr"/>
-      <c r="AC37" s="11" t="inlineStr"/>
-      <c r="AD37" s="12" t="inlineStr"/>
+      <c r="AB37" s="8" t="inlineStr"/>
+      <c r="AC37" s="8" t="inlineStr"/>
+      <c r="AD37" s="8" t="inlineStr"/>
+      <c r="AE37" s="10" t="inlineStr"/>
+      <c r="AF37" s="11" t="inlineStr"/>
+      <c r="AG37" s="12" t="inlineStr"/>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -3619,11 +3936,14 @@
       <c r="Y38" s="4" t="inlineStr"/>
       <c r="Z38" s="4" t="inlineStr"/>
       <c r="AA38" s="4" t="inlineStr"/>
-      <c r="AB38" s="5" t="inlineStr"/>
-      <c r="AC38" s="6" t="n">
+      <c r="AB38" s="4" t="inlineStr"/>
+      <c r="AC38" s="4" t="inlineStr"/>
+      <c r="AD38" s="4" t="inlineStr"/>
+      <c r="AE38" s="5" t="inlineStr"/>
+      <c r="AF38" s="6" t="n">
         <v>-1.350000000000009</v>
       </c>
-      <c r="AD38" s="7" t="n">
+      <c r="AG38" s="7" t="n">
         <v>-0.1125000000000007</v>
       </c>
     </row>
@@ -3687,11 +4007,14 @@
       <c r="Y39" s="8" t="inlineStr"/>
       <c r="Z39" s="8" t="inlineStr"/>
       <c r="AA39" s="8" t="inlineStr"/>
-      <c r="AB39" s="10" t="n">
+      <c r="AB39" s="8" t="inlineStr"/>
+      <c r="AC39" s="8" t="inlineStr"/>
+      <c r="AD39" s="8" t="inlineStr"/>
+      <c r="AE39" s="10" t="n">
         <v>78.64999999999999</v>
       </c>
-      <c r="AC39" s="11" t="inlineStr"/>
-      <c r="AD39" s="12" t="inlineStr"/>
+      <c r="AF39" s="11" t="inlineStr"/>
+      <c r="AG39" s="12" t="inlineStr"/>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="1" t="n"/>
@@ -3733,9 +4056,12 @@
       <c r="Y40" s="8" t="inlineStr"/>
       <c r="Z40" s="8" t="inlineStr"/>
       <c r="AA40" s="8" t="inlineStr"/>
-      <c r="AB40" s="10" t="inlineStr"/>
-      <c r="AC40" s="11" t="inlineStr"/>
-      <c r="AD40" s="12" t="inlineStr"/>
+      <c r="AB40" s="8" t="inlineStr"/>
+      <c r="AC40" s="8" t="inlineStr"/>
+      <c r="AD40" s="8" t="inlineStr"/>
+      <c r="AE40" s="10" t="inlineStr"/>
+      <c r="AF40" s="11" t="inlineStr"/>
+      <c r="AG40" s="12" t="inlineStr"/>
     </row>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="1" t="n"/>
@@ -3779,13 +4105,21 @@
           <t>87.90</t>
         </is>
       </c>
-      <c r="R41" s="14" t="inlineStr">
+      <c r="R41" s="15" t="inlineStr">
         <is>
           <t>RUNNING</t>
         </is>
       </c>
-      <c r="S41" s="8" t="inlineStr"/>
-      <c r="T41" s="8" t="inlineStr"/>
+      <c r="S41" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="T41" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="U41" s="8" t="inlineStr"/>
       <c r="V41" s="8" t="inlineStr"/>
       <c r="W41" s="8" t="inlineStr"/>
@@ -3793,13 +4127,16 @@
       <c r="Y41" s="8" t="inlineStr"/>
       <c r="Z41" s="8" t="inlineStr"/>
       <c r="AA41" s="8" t="inlineStr"/>
-      <c r="AB41" s="10" t="n">
+      <c r="AB41" s="8" t="inlineStr"/>
+      <c r="AC41" s="8" t="inlineStr"/>
+      <c r="AD41" s="8" t="inlineStr"/>
+      <c r="AE41" s="10" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="AC41" s="10" t="n">
+      <c r="AF41" s="10" t="n">
         <v>3.250000000000014</v>
       </c>
-      <c r="AD41" s="12" t="n">
+      <c r="AG41" s="12" t="n">
         <v>0.2708333333333345</v>
       </c>
     </row>
@@ -3839,9 +4176,12 @@
       <c r="Y42" s="8" t="inlineStr"/>
       <c r="Z42" s="8" t="inlineStr"/>
       <c r="AA42" s="8" t="inlineStr"/>
-      <c r="AB42" s="10" t="inlineStr"/>
-      <c r="AC42" s="11" t="inlineStr"/>
-      <c r="AD42" s="12" t="inlineStr"/>
+      <c r="AB42" s="8" t="inlineStr"/>
+      <c r="AC42" s="8" t="inlineStr"/>
+      <c r="AD42" s="8" t="inlineStr"/>
+      <c r="AE42" s="10" t="inlineStr"/>
+      <c r="AF42" s="11" t="inlineStr"/>
+      <c r="AG42" s="12" t="inlineStr"/>
     </row>
     <row r="43" ht="24" customHeight="1">
       <c r="A43" s="1" t="n"/>
@@ -3879,9 +4219,12 @@
       <c r="Y43" s="8" t="inlineStr"/>
       <c r="Z43" s="8" t="inlineStr"/>
       <c r="AA43" s="8" t="inlineStr"/>
-      <c r="AB43" s="10" t="inlineStr"/>
-      <c r="AC43" s="11" t="inlineStr"/>
-      <c r="AD43" s="12" t="inlineStr"/>
+      <c r="AB43" s="8" t="inlineStr"/>
+      <c r="AC43" s="8" t="inlineStr"/>
+      <c r="AD43" s="8" t="inlineStr"/>
+      <c r="AE43" s="10" t="inlineStr"/>
+      <c r="AF43" s="11" t="inlineStr"/>
+      <c r="AG43" s="12" t="inlineStr"/>
     </row>
     <row r="44" ht="24" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -3921,11 +4264,14 @@
       <c r="Y44" s="4" t="inlineStr"/>
       <c r="Z44" s="4" t="inlineStr"/>
       <c r="AA44" s="4" t="inlineStr"/>
-      <c r="AB44" s="5" t="inlineStr"/>
-      <c r="AC44" s="6" t="n">
+      <c r="AB44" s="4" t="inlineStr"/>
+      <c r="AC44" s="4" t="inlineStr"/>
+      <c r="AD44" s="4" t="inlineStr"/>
+      <c r="AE44" s="5" t="inlineStr"/>
+      <c r="AF44" s="6" t="n">
         <v>-4.266666666666666</v>
       </c>
-      <c r="AD44" s="7" t="n">
+      <c r="AG44" s="7" t="n">
         <v>-0.1481481481481481</v>
       </c>
     </row>
@@ -3981,11 +4327,14 @@
       <c r="Y45" s="8" t="inlineStr"/>
       <c r="Z45" s="8" t="inlineStr"/>
       <c r="AA45" s="8" t="inlineStr"/>
-      <c r="AB45" s="10" t="n">
+      <c r="AB45" s="8" t="inlineStr"/>
+      <c r="AC45" s="8" t="inlineStr"/>
+      <c r="AD45" s="8" t="inlineStr"/>
+      <c r="AE45" s="10" t="n">
         <v>11.73333333333333</v>
       </c>
-      <c r="AC45" s="11" t="inlineStr"/>
-      <c r="AD45" s="12" t="inlineStr"/>
+      <c r="AF45" s="11" t="inlineStr"/>
+      <c r="AG45" s="12" t="inlineStr"/>
     </row>
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="1" t="n"/>
@@ -4031,9 +4380,12 @@
       <c r="Y46" s="8" t="inlineStr"/>
       <c r="Z46" s="8" t="inlineStr"/>
       <c r="AA46" s="8" t="inlineStr"/>
-      <c r="AB46" s="10" t="inlineStr"/>
-      <c r="AC46" s="11" t="inlineStr"/>
-      <c r="AD46" s="12" t="inlineStr"/>
+      <c r="AB46" s="8" t="inlineStr"/>
+      <c r="AC46" s="8" t="inlineStr"/>
+      <c r="AD46" s="8" t="inlineStr"/>
+      <c r="AE46" s="10" t="inlineStr"/>
+      <c r="AF46" s="11" t="inlineStr"/>
+      <c r="AG46" s="12" t="inlineStr"/>
     </row>
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="1" t="n"/>
@@ -4083,13 +4435,16 @@
       <c r="Y47" s="8" t="inlineStr"/>
       <c r="Z47" s="8" t="inlineStr"/>
       <c r="AA47" s="8" t="inlineStr"/>
-      <c r="AB47" s="10" t="n">
+      <c r="AB47" s="8" t="inlineStr"/>
+      <c r="AC47" s="8" t="inlineStr"/>
+      <c r="AD47" s="8" t="inlineStr"/>
+      <c r="AE47" s="10" t="n">
         <v>12.36666666666667</v>
       </c>
-      <c r="AC47" s="10" t="n">
+      <c r="AF47" s="10" t="n">
         <v>0.6333333333333311</v>
       </c>
-      <c r="AD47" s="12" t="n">
+      <c r="AG47" s="12" t="n">
         <v>0.02199074074074066</v>
       </c>
     </row>
@@ -4131,11 +4486,14 @@
       <c r="Y48" s="4" t="inlineStr"/>
       <c r="Z48" s="4" t="inlineStr"/>
       <c r="AA48" s="4" t="inlineStr"/>
-      <c r="AB48" s="5" t="inlineStr"/>
-      <c r="AC48" s="6" t="n">
+      <c r="AB48" s="4" t="inlineStr"/>
+      <c r="AC48" s="4" t="inlineStr"/>
+      <c r="AD48" s="4" t="inlineStr"/>
+      <c r="AE48" s="5" t="inlineStr"/>
+      <c r="AF48" s="6" t="n">
         <v>-199.25</v>
       </c>
-      <c r="AD48" s="7" t="n">
+      <c r="AG48" s="7" t="n">
         <v>-0.03029588857803187</v>
       </c>
     </row>
@@ -4191,11 +4549,14 @@
       <c r="Y49" s="8" t="inlineStr"/>
       <c r="Z49" s="8" t="inlineStr"/>
       <c r="AA49" s="8" t="inlineStr"/>
-      <c r="AB49" s="10" t="n">
+      <c r="AB49" s="8" t="inlineStr"/>
+      <c r="AC49" s="8" t="inlineStr"/>
+      <c r="AD49" s="8" t="inlineStr"/>
+      <c r="AE49" s="10" t="n">
         <v>1688.75</v>
       </c>
-      <c r="AC49" s="11" t="inlineStr"/>
-      <c r="AD49" s="12" t="inlineStr"/>
+      <c r="AF49" s="11" t="inlineStr"/>
+      <c r="AG49" s="12" t="inlineStr"/>
     </row>
     <row r="50" ht="24" customHeight="1">
       <c r="A50" s="1" t="n"/>
@@ -4237,9 +4598,12 @@
       <c r="Y50" s="8" t="inlineStr"/>
       <c r="Z50" s="8" t="inlineStr"/>
       <c r="AA50" s="8" t="inlineStr"/>
-      <c r="AB50" s="10" t="inlineStr"/>
-      <c r="AC50" s="11" t="inlineStr"/>
-      <c r="AD50" s="12" t="inlineStr"/>
+      <c r="AB50" s="8" t="inlineStr"/>
+      <c r="AC50" s="8" t="inlineStr"/>
+      <c r="AD50" s="8" t="inlineStr"/>
+      <c r="AE50" s="10" t="inlineStr"/>
+      <c r="AF50" s="11" t="inlineStr"/>
+      <c r="AG50" s="12" t="inlineStr"/>
     </row>
     <row r="51" ht="24" customHeight="1">
       <c r="A51" s="1" t="n"/>
@@ -4289,13 +4653,16 @@
       <c r="Y51" s="8" t="inlineStr"/>
       <c r="Z51" s="8" t="inlineStr"/>
       <c r="AA51" s="8" t="inlineStr"/>
-      <c r="AB51" s="10" t="n">
+      <c r="AB51" s="8" t="inlineStr"/>
+      <c r="AC51" s="8" t="inlineStr"/>
+      <c r="AD51" s="8" t="inlineStr"/>
+      <c r="AE51" s="10" t="n">
         <v>1425</v>
       </c>
-      <c r="AC51" s="10" t="n">
+      <c r="AF51" s="10" t="n">
         <v>263.75</v>
       </c>
-      <c r="AD51" s="12" t="n">
+      <c r="AG51" s="12" t="n">
         <v>-0.04010308964846126</v>
       </c>
     </row>
@@ -4339,9 +4706,12 @@
       <c r="Y52" s="8" t="inlineStr"/>
       <c r="Z52" s="8" t="inlineStr"/>
       <c r="AA52" s="8" t="inlineStr"/>
-      <c r="AB52" s="10" t="inlineStr"/>
-      <c r="AC52" s="11" t="inlineStr"/>
-      <c r="AD52" s="12" t="inlineStr"/>
+      <c r="AB52" s="8" t="inlineStr"/>
+      <c r="AC52" s="8" t="inlineStr"/>
+      <c r="AD52" s="8" t="inlineStr"/>
+      <c r="AE52" s="10" t="inlineStr"/>
+      <c r="AF52" s="11" t="inlineStr"/>
+      <c r="AG52" s="12" t="inlineStr"/>
     </row>
     <row r="53" ht="24" customHeight="1">
       <c r="A53" s="1" t="n"/>
@@ -4383,9 +4753,12 @@
       <c r="Y53" s="8" t="inlineStr"/>
       <c r="Z53" s="8" t="inlineStr"/>
       <c r="AA53" s="8" t="inlineStr"/>
-      <c r="AB53" s="10" t="inlineStr"/>
-      <c r="AC53" s="11" t="inlineStr"/>
-      <c r="AD53" s="12" t="inlineStr"/>
+      <c r="AB53" s="8" t="inlineStr"/>
+      <c r="AC53" s="8" t="inlineStr"/>
+      <c r="AD53" s="8" t="inlineStr"/>
+      <c r="AE53" s="10" t="inlineStr"/>
+      <c r="AF53" s="11" t="inlineStr"/>
+      <c r="AG53" s="12" t="inlineStr"/>
     </row>
     <row r="54" ht="24" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -4425,11 +4798,14 @@
       <c r="Y54" s="4" t="inlineStr"/>
       <c r="Z54" s="4" t="inlineStr"/>
       <c r="AA54" s="4" t="inlineStr"/>
-      <c r="AB54" s="5" t="inlineStr"/>
-      <c r="AC54" s="6" t="n">
+      <c r="AB54" s="4" t="inlineStr"/>
+      <c r="AC54" s="4" t="inlineStr"/>
+      <c r="AD54" s="4" t="inlineStr"/>
+      <c r="AE54" s="5" t="inlineStr"/>
+      <c r="AF54" s="6" t="n">
         <v>-9204.333333333336</v>
       </c>
-      <c r="AD54" s="7" t="n">
+      <c r="AG54" s="7" t="n">
         <v>-0.3674545921510859</v>
       </c>
     </row>
@@ -4485,11 +4861,14 @@
       <c r="Y55" s="8" t="inlineStr"/>
       <c r="Z55" s="8" t="inlineStr"/>
       <c r="AA55" s="8" t="inlineStr"/>
-      <c r="AB55" s="10" t="n">
+      <c r="AB55" s="8" t="inlineStr"/>
+      <c r="AC55" s="8" t="inlineStr"/>
+      <c r="AD55" s="8" t="inlineStr"/>
+      <c r="AE55" s="10" t="n">
         <v>57571.66666666666</v>
       </c>
-      <c r="AC55" s="11" t="inlineStr"/>
-      <c r="AD55" s="12" t="inlineStr"/>
+      <c r="AF55" s="11" t="inlineStr"/>
+      <c r="AG55" s="12" t="inlineStr"/>
     </row>
     <row r="56" ht="24" customHeight="1">
       <c r="A56" s="1" t="n"/>
@@ -4527,9 +4906,12 @@
       <c r="Y56" s="8" t="inlineStr"/>
       <c r="Z56" s="8" t="inlineStr"/>
       <c r="AA56" s="8" t="inlineStr"/>
-      <c r="AB56" s="10" t="inlineStr"/>
-      <c r="AC56" s="11" t="inlineStr"/>
-      <c r="AD56" s="12" t="inlineStr"/>
+      <c r="AB56" s="8" t="inlineStr"/>
+      <c r="AC56" s="8" t="inlineStr"/>
+      <c r="AD56" s="8" t="inlineStr"/>
+      <c r="AE56" s="10" t="inlineStr"/>
+      <c r="AF56" s="11" t="inlineStr"/>
+      <c r="AG56" s="12" t="inlineStr"/>
     </row>
     <row r="57" ht="24" customHeight="1">
       <c r="A57" s="1" t="n"/>
@@ -4559,15 +4941,23 @@
           <t>63275.00</t>
         </is>
       </c>
-      <c r="L57" s="8" t="inlineStr"/>
+      <c r="L57" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="M57" s="8" t="inlineStr"/>
       <c r="N57" s="8" t="inlineStr"/>
-      <c r="O57" s="14" t="inlineStr">
+      <c r="O57" s="15" t="inlineStr">
         <is>
           <t>RUNNING</t>
         </is>
       </c>
-      <c r="P57" s="8" t="inlineStr"/>
+      <c r="P57" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="Q57" s="8" t="inlineStr"/>
       <c r="R57" s="8" t="inlineStr"/>
       <c r="S57" s="8" t="inlineStr"/>
@@ -4579,13 +4969,16 @@
       <c r="Y57" s="8" t="inlineStr"/>
       <c r="Z57" s="8" t="inlineStr"/>
       <c r="AA57" s="8" t="inlineStr"/>
-      <c r="AB57" s="10" t="n">
+      <c r="AB57" s="8" t="inlineStr"/>
+      <c r="AC57" s="8" t="inlineStr"/>
+      <c r="AD57" s="8" t="inlineStr"/>
+      <c r="AE57" s="10" t="n">
         <v>57908.33333333334</v>
       </c>
-      <c r="AC57" s="10" t="n">
+      <c r="AF57" s="10" t="n">
         <v>336.6666666666715</v>
       </c>
-      <c r="AD57" s="12" t="n">
+      <c r="AG57" s="12" t="n">
         <v>0.01344037728869018</v>
       </c>
     </row>
@@ -4625,9 +5018,12 @@
       <c r="Y58" s="8" t="inlineStr"/>
       <c r="Z58" s="8" t="inlineStr"/>
       <c r="AA58" s="8" t="inlineStr"/>
-      <c r="AB58" s="10" t="inlineStr"/>
-      <c r="AC58" s="11" t="inlineStr"/>
-      <c r="AD58" s="12" t="inlineStr"/>
+      <c r="AB58" s="8" t="inlineStr"/>
+      <c r="AC58" s="8" t="inlineStr"/>
+      <c r="AD58" s="8" t="inlineStr"/>
+      <c r="AE58" s="10" t="inlineStr"/>
+      <c r="AF58" s="11" t="inlineStr"/>
+      <c r="AG58" s="12" t="inlineStr"/>
     </row>
     <row r="59" ht="24" customHeight="1">
       <c r="A59" s="1" t="n"/>
@@ -4665,9 +5061,12 @@
       <c r="Y59" s="8" t="inlineStr"/>
       <c r="Z59" s="8" t="inlineStr"/>
       <c r="AA59" s="8" t="inlineStr"/>
-      <c r="AB59" s="10" t="inlineStr"/>
-      <c r="AC59" s="11" t="inlineStr"/>
-      <c r="AD59" s="12" t="inlineStr"/>
+      <c r="AB59" s="8" t="inlineStr"/>
+      <c r="AC59" s="8" t="inlineStr"/>
+      <c r="AD59" s="8" t="inlineStr"/>
+      <c r="AE59" s="10" t="inlineStr"/>
+      <c r="AF59" s="11" t="inlineStr"/>
+      <c r="AG59" s="12" t="inlineStr"/>
     </row>
     <row r="60" ht="24" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -4707,11 +5106,14 @@
       <c r="Y60" s="4" t="inlineStr"/>
       <c r="Z60" s="4" t="inlineStr"/>
       <c r="AA60" s="4" t="inlineStr"/>
-      <c r="AB60" s="5" t="inlineStr"/>
-      <c r="AC60" s="6" t="n">
+      <c r="AB60" s="4" t="inlineStr"/>
+      <c r="AC60" s="4" t="inlineStr"/>
+      <c r="AD60" s="4" t="inlineStr"/>
+      <c r="AE60" s="5" t="inlineStr"/>
+      <c r="AF60" s="6" t="n">
         <v>16.625</v>
       </c>
-      <c r="AD60" s="7" t="n">
+      <c r="AG60" s="7" t="n">
         <v>0.009140139644840287</v>
       </c>
     </row>
@@ -4767,11 +5169,14 @@
       <c r="Y61" s="8" t="inlineStr"/>
       <c r="Z61" s="8" t="inlineStr"/>
       <c r="AA61" s="8" t="inlineStr"/>
-      <c r="AB61" s="10" t="n">
+      <c r="AB61" s="8" t="inlineStr"/>
+      <c r="AC61" s="8" t="inlineStr"/>
+      <c r="AD61" s="8" t="inlineStr"/>
+      <c r="AE61" s="10" t="n">
         <v>181.625</v>
       </c>
-      <c r="AC61" s="11" t="inlineStr"/>
-      <c r="AD61" s="12" t="inlineStr"/>
+      <c r="AF61" s="11" t="inlineStr"/>
+      <c r="AG61" s="12" t="inlineStr"/>
     </row>
     <row r="62" ht="24" customHeight="1">
       <c r="A62" s="1" t="n"/>
@@ -4813,9 +5218,12 @@
       <c r="Y62" s="8" t="inlineStr"/>
       <c r="Z62" s="8" t="inlineStr"/>
       <c r="AA62" s="8" t="inlineStr"/>
-      <c r="AB62" s="10" t="inlineStr"/>
-      <c r="AC62" s="11" t="inlineStr"/>
-      <c r="AD62" s="12" t="inlineStr"/>
+      <c r="AB62" s="8" t="inlineStr"/>
+      <c r="AC62" s="8" t="inlineStr"/>
+      <c r="AD62" s="8" t="inlineStr"/>
+      <c r="AE62" s="10" t="inlineStr"/>
+      <c r="AF62" s="11" t="inlineStr"/>
+      <c r="AG62" s="12" t="inlineStr"/>
     </row>
     <row r="63" ht="24" customHeight="1">
       <c r="A63" s="1" t="n"/>
@@ -4865,13 +5273,16 @@
       <c r="Y63" s="8" t="inlineStr"/>
       <c r="Z63" s="8" t="inlineStr"/>
       <c r="AA63" s="8" t="inlineStr"/>
-      <c r="AB63" s="10" t="n">
+      <c r="AB63" s="8" t="inlineStr"/>
+      <c r="AC63" s="8" t="inlineStr"/>
+      <c r="AD63" s="8" t="inlineStr"/>
+      <c r="AE63" s="10" t="n">
         <v>155.125</v>
       </c>
-      <c r="AC63" s="10" t="n">
+      <c r="AF63" s="10" t="n">
         <v>26.5</v>
       </c>
-      <c r="AD63" s="12" t="n">
+      <c r="AG63" s="12" t="n">
         <v>-0.01456924514816647</v>
       </c>
     </row>
@@ -4915,9 +5326,12 @@
       <c r="Y64" s="8" t="inlineStr"/>
       <c r="Z64" s="8" t="inlineStr"/>
       <c r="AA64" s="8" t="inlineStr"/>
-      <c r="AB64" s="10" t="inlineStr"/>
-      <c r="AC64" s="11" t="inlineStr"/>
-      <c r="AD64" s="12" t="inlineStr"/>
+      <c r="AB64" s="8" t="inlineStr"/>
+      <c r="AC64" s="8" t="inlineStr"/>
+      <c r="AD64" s="8" t="inlineStr"/>
+      <c r="AE64" s="10" t="inlineStr"/>
+      <c r="AF64" s="11" t="inlineStr"/>
+      <c r="AG64" s="12" t="inlineStr"/>
     </row>
     <row r="65" ht="24" customHeight="1">
       <c r="A65" s="1" t="n"/>
@@ -4959,9 +5373,12 @@
       <c r="Y65" s="8" t="inlineStr"/>
       <c r="Z65" s="8" t="inlineStr"/>
       <c r="AA65" s="8" t="inlineStr"/>
-      <c r="AB65" s="10" t="inlineStr"/>
-      <c r="AC65" s="11" t="inlineStr"/>
-      <c r="AD65" s="12" t="inlineStr"/>
+      <c r="AB65" s="8" t="inlineStr"/>
+      <c r="AC65" s="8" t="inlineStr"/>
+      <c r="AD65" s="8" t="inlineStr"/>
+      <c r="AE65" s="10" t="inlineStr"/>
+      <c r="AF65" s="11" t="inlineStr"/>
+      <c r="AG65" s="12" t="inlineStr"/>
     </row>
     <row r="66" ht="24" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
@@ -5001,11 +5418,14 @@
       <c r="Y66" s="4" t="inlineStr"/>
       <c r="Z66" s="4" t="inlineStr"/>
       <c r="AA66" s="4" t="inlineStr"/>
-      <c r="AB66" s="5" t="inlineStr"/>
-      <c r="AC66" s="6" t="n">
+      <c r="AB66" s="4" t="inlineStr"/>
+      <c r="AC66" s="4" t="inlineStr"/>
+      <c r="AD66" s="4" t="inlineStr"/>
+      <c r="AE66" s="5" t="inlineStr"/>
+      <c r="AF66" s="6" t="n">
         <v>-0.5500000000000043</v>
       </c>
-      <c r="AD66" s="7" t="n">
+      <c r="AG66" s="7" t="n">
         <v>-0.01858108108108122</v>
       </c>
     </row>
@@ -5057,11 +5477,14 @@
       <c r="Y67" s="8" t="inlineStr"/>
       <c r="Z67" s="8" t="inlineStr"/>
       <c r="AA67" s="8" t="inlineStr"/>
-      <c r="AB67" s="10" t="n">
+      <c r="AB67" s="8" t="inlineStr"/>
+      <c r="AC67" s="8" t="inlineStr"/>
+      <c r="AD67" s="8" t="inlineStr"/>
+      <c r="AE67" s="10" t="n">
         <v>33.45</v>
       </c>
-      <c r="AC67" s="11" t="inlineStr"/>
-      <c r="AD67" s="12" t="inlineStr"/>
+      <c r="AF67" s="11" t="inlineStr"/>
+      <c r="AG67" s="12" t="inlineStr"/>
     </row>
     <row r="68" ht="24" customHeight="1">
       <c r="A68" s="1" t="n"/>
@@ -5099,9 +5522,12 @@
       <c r="Y68" s="8" t="inlineStr"/>
       <c r="Z68" s="8" t="inlineStr"/>
       <c r="AA68" s="8" t="inlineStr"/>
-      <c r="AB68" s="10" t="inlineStr"/>
-      <c r="AC68" s="11" t="inlineStr"/>
-      <c r="AD68" s="12" t="inlineStr"/>
+      <c r="AB68" s="8" t="inlineStr"/>
+      <c r="AC68" s="8" t="inlineStr"/>
+      <c r="AD68" s="8" t="inlineStr"/>
+      <c r="AE68" s="10" t="inlineStr"/>
+      <c r="AF68" s="11" t="inlineStr"/>
+      <c r="AG68" s="12" t="inlineStr"/>
     </row>
     <row r="69" ht="24" customHeight="1">
       <c r="A69" s="1" t="n"/>
@@ -5110,8 +5536,16 @@
           <t>target: 16 (anchor 미설정)</t>
         </is>
       </c>
-      <c r="C69" s="8" t="inlineStr"/>
-      <c r="D69" s="8" t="inlineStr"/>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="E69" s="8" t="inlineStr"/>
       <c r="F69" s="8" t="inlineStr"/>
       <c r="G69" s="8" t="inlineStr"/>
@@ -5151,13 +5585,20 @@
       <c r="Y69" s="8" t="inlineStr"/>
       <c r="Z69" s="8" t="inlineStr"/>
       <c r="AA69" s="8" t="inlineStr"/>
-      <c r="AB69" s="10" t="n">
+      <c r="AB69" s="8" t="inlineStr"/>
+      <c r="AC69" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="AD69" s="8" t="inlineStr"/>
+      <c r="AE69" s="10" t="n">
         <v>33.35</v>
       </c>
-      <c r="AC69" s="10" t="n">
+      <c r="AF69" s="10" t="n">
         <v>0.09999999999999432</v>
       </c>
-      <c r="AD69" s="12" t="n">
+      <c r="AG69" s="12" t="n">
         <v>-0.003378378378378186</v>
       </c>
     </row>
@@ -5197,9 +5638,12 @@
       <c r="Y70" s="8" t="inlineStr"/>
       <c r="Z70" s="8" t="inlineStr"/>
       <c r="AA70" s="8" t="inlineStr"/>
-      <c r="AB70" s="10" t="inlineStr"/>
-      <c r="AC70" s="11" t="inlineStr"/>
-      <c r="AD70" s="12" t="inlineStr"/>
+      <c r="AB70" s="8" t="inlineStr"/>
+      <c r="AC70" s="8" t="inlineStr"/>
+      <c r="AD70" s="8" t="inlineStr"/>
+      <c r="AE70" s="10" t="inlineStr"/>
+      <c r="AF70" s="11" t="inlineStr"/>
+      <c r="AG70" s="12" t="inlineStr"/>
     </row>
     <row r="71" ht="24" customHeight="1">
       <c r="A71" s="1" t="n"/>
@@ -5237,9 +5681,12 @@
       <c r="Y71" s="8" t="inlineStr"/>
       <c r="Z71" s="8" t="inlineStr"/>
       <c r="AA71" s="8" t="inlineStr"/>
-      <c r="AB71" s="10" t="inlineStr"/>
-      <c r="AC71" s="11" t="inlineStr"/>
-      <c r="AD71" s="12" t="inlineStr"/>
+      <c r="AB71" s="8" t="inlineStr"/>
+      <c r="AC71" s="8" t="inlineStr"/>
+      <c r="AD71" s="8" t="inlineStr"/>
+      <c r="AE71" s="10" t="inlineStr"/>
+      <c r="AF71" s="11" t="inlineStr"/>
+      <c r="AG71" s="12" t="inlineStr"/>
     </row>
     <row r="72" ht="24" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
@@ -5279,11 +5726,14 @@
       <c r="Y72" s="4" t="inlineStr"/>
       <c r="Z72" s="4" t="inlineStr"/>
       <c r="AA72" s="4" t="inlineStr"/>
-      <c r="AB72" s="5" t="inlineStr"/>
-      <c r="AC72" s="6" t="n">
+      <c r="AB72" s="4" t="inlineStr"/>
+      <c r="AC72" s="4" t="inlineStr"/>
+      <c r="AD72" s="4" t="inlineStr"/>
+      <c r="AE72" s="5" t="inlineStr"/>
+      <c r="AF72" s="6" t="n">
         <v>426.375</v>
       </c>
-      <c r="AD72" s="7" t="n">
+      <c r="AG72" s="7" t="n">
         <v>0.09986532380840848</v>
       </c>
     </row>
@@ -5339,11 +5789,14 @@
       <c r="Y73" s="8" t="inlineStr"/>
       <c r="Z73" s="8" t="inlineStr"/>
       <c r="AA73" s="8" t="inlineStr"/>
-      <c r="AB73" s="10" t="n">
+      <c r="AB73" s="8" t="inlineStr"/>
+      <c r="AC73" s="8" t="inlineStr"/>
+      <c r="AD73" s="8" t="inlineStr"/>
+      <c r="AE73" s="10" t="n">
         <v>1742.375</v>
       </c>
-      <c r="AC73" s="11" t="inlineStr"/>
-      <c r="AD73" s="12" t="inlineStr"/>
+      <c r="AF73" s="11" t="inlineStr"/>
+      <c r="AG73" s="12" t="inlineStr"/>
     </row>
     <row r="74" ht="24" customHeight="1">
       <c r="A74" s="1" t="n"/>
@@ -5397,9 +5850,12 @@
       <c r="Y74" s="8" t="inlineStr"/>
       <c r="Z74" s="8" t="inlineStr"/>
       <c r="AA74" s="8" t="inlineStr"/>
-      <c r="AB74" s="10" t="inlineStr"/>
-      <c r="AC74" s="11" t="inlineStr"/>
-      <c r="AD74" s="12" t="inlineStr"/>
+      <c r="AB74" s="8" t="inlineStr"/>
+      <c r="AC74" s="8" t="inlineStr"/>
+      <c r="AD74" s="8" t="inlineStr"/>
+      <c r="AE74" s="10" t="inlineStr"/>
+      <c r="AF74" s="11" t="inlineStr"/>
+      <c r="AG74" s="12" t="inlineStr"/>
     </row>
     <row r="75" ht="24" customHeight="1">
       <c r="A75" s="1" t="n"/>
@@ -5461,13 +5917,16 @@
       <c r="Y75" s="8" t="inlineStr"/>
       <c r="Z75" s="8" t="inlineStr"/>
       <c r="AA75" s="8" t="inlineStr"/>
-      <c r="AB75" s="10" t="n">
+      <c r="AB75" s="8" t="inlineStr"/>
+      <c r="AC75" s="8" t="inlineStr"/>
+      <c r="AD75" s="8" t="inlineStr"/>
+      <c r="AE75" s="10" t="n">
         <v>1986.75</v>
       </c>
-      <c r="AC75" s="10" t="n">
+      <c r="AF75" s="10" t="n">
         <v>244.375</v>
       </c>
-      <c r="AD75" s="12" t="n">
+      <c r="AG75" s="12" t="n">
         <v>0.05723738142639653</v>
       </c>
     </row>
@@ -5511,9 +5970,12 @@
       <c r="Y76" s="8" t="inlineStr"/>
       <c r="Z76" s="8" t="inlineStr"/>
       <c r="AA76" s="8" t="inlineStr"/>
-      <c r="AB76" s="10" t="inlineStr"/>
-      <c r="AC76" s="11" t="inlineStr"/>
-      <c r="AD76" s="12" t="inlineStr"/>
+      <c r="AB76" s="8" t="inlineStr"/>
+      <c r="AC76" s="8" t="inlineStr"/>
+      <c r="AD76" s="8" t="inlineStr"/>
+      <c r="AE76" s="10" t="inlineStr"/>
+      <c r="AF76" s="11" t="inlineStr"/>
+      <c r="AG76" s="12" t="inlineStr"/>
     </row>
     <row r="77" ht="24" customHeight="1">
       <c r="A77" s="1" t="n"/>
@@ -5551,9 +6013,12 @@
       <c r="Y77" s="8" t="inlineStr"/>
       <c r="Z77" s="8" t="inlineStr"/>
       <c r="AA77" s="8" t="inlineStr"/>
-      <c r="AB77" s="10" t="inlineStr"/>
-      <c r="AC77" s="11" t="inlineStr"/>
-      <c r="AD77" s="12" t="inlineStr"/>
+      <c r="AB77" s="8" t="inlineStr"/>
+      <c r="AC77" s="8" t="inlineStr"/>
+      <c r="AD77" s="8" t="inlineStr"/>
+      <c r="AE77" s="10" t="inlineStr"/>
+      <c r="AF77" s="11" t="inlineStr"/>
+      <c r="AG77" s="12" t="inlineStr"/>
     </row>
     <row r="78" ht="24" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
@@ -5593,11 +6058,14 @@
       <c r="Y78" s="4" t="inlineStr"/>
       <c r="Z78" s="4" t="inlineStr"/>
       <c r="AA78" s="4" t="inlineStr"/>
-      <c r="AB78" s="5" t="inlineStr"/>
-      <c r="AC78" s="6" t="n">
+      <c r="AB78" s="4" t="inlineStr"/>
+      <c r="AC78" s="4" t="inlineStr"/>
+      <c r="AD78" s="4" t="inlineStr"/>
+      <c r="AE78" s="5" t="inlineStr"/>
+      <c r="AF78" s="6" t="n">
         <v>-3430.5</v>
       </c>
-      <c r="AD78" s="7" t="n">
+      <c r="AG78" s="7" t="n">
         <v>-1.591953222887373</v>
       </c>
     </row>
@@ -5655,29 +6123,32 @@
       <c r="S79" s="9" t="inlineStr"/>
       <c r="T79" s="8" t="inlineStr"/>
       <c r="U79" s="8" t="inlineStr"/>
-      <c r="V79" s="9" t="inlineStr"/>
-      <c r="W79" s="9" t="inlineStr"/>
-      <c r="X79" s="8" t="inlineStr">
+      <c r="V79" s="8" t="inlineStr"/>
+      <c r="W79" s="8" t="inlineStr"/>
+      <c r="X79" s="8" t="inlineStr"/>
+      <c r="Y79" s="9" t="inlineStr"/>
+      <c r="Z79" s="9" t="inlineStr"/>
+      <c r="AA79" s="8" t="inlineStr">
         <is>
           <t>8159.00</t>
         </is>
       </c>
-      <c r="Y79" s="8" t="inlineStr">
+      <c r="AB79" s="8" t="inlineStr">
         <is>
           <t>3585.00</t>
         </is>
       </c>
-      <c r="Z79" s="9" t="inlineStr">
+      <c r="AC79" s="9" t="inlineStr">
         <is>
           <t>2594.00</t>
         </is>
       </c>
-      <c r="AA79" s="8" t="inlineStr"/>
-      <c r="AB79" s="10" t="n">
+      <c r="AD79" s="8" t="inlineStr"/>
+      <c r="AE79" s="10" t="n">
         <v>4809.5</v>
       </c>
-      <c r="AC79" s="11" t="inlineStr"/>
-      <c r="AD79" s="12" t="inlineStr"/>
+      <c r="AF79" s="11" t="inlineStr"/>
+      <c r="AG79" s="12" t="inlineStr"/>
     </row>
     <row r="80" ht="24" customHeight="1">
       <c r="A80" s="1" t="n"/>
@@ -5709,19 +6180,22 @@
       <c r="S80" s="9" t="inlineStr"/>
       <c r="T80" s="8" t="inlineStr"/>
       <c r="U80" s="8" t="inlineStr"/>
-      <c r="V80" s="9" t="inlineStr"/>
-      <c r="W80" s="9" t="inlineStr"/>
+      <c r="V80" s="8" t="inlineStr"/>
+      <c r="W80" s="8" t="inlineStr"/>
       <c r="X80" s="8" t="inlineStr"/>
-      <c r="Y80" s="8" t="inlineStr">
-        <is>
-          <t>4472.00</t>
-        </is>
-      </c>
+      <c r="Y80" s="9" t="inlineStr"/>
       <c r="Z80" s="9" t="inlineStr"/>
       <c r="AA80" s="8" t="inlineStr"/>
-      <c r="AB80" s="10" t="inlineStr"/>
-      <c r="AC80" s="11" t="inlineStr"/>
-      <c r="AD80" s="12" t="inlineStr"/>
+      <c r="AB80" s="8" t="inlineStr">
+        <is>
+          <t>4472.00</t>
+        </is>
+      </c>
+      <c r="AC80" s="9" t="inlineStr"/>
+      <c r="AD80" s="8" t="inlineStr"/>
+      <c r="AE80" s="10" t="inlineStr"/>
+      <c r="AF80" s="11" t="inlineStr"/>
+      <c r="AG80" s="12" t="inlineStr"/>
     </row>
     <row r="81" ht="24" customHeight="1">
       <c r="A81" s="1" t="n"/>
@@ -5775,41 +6249,56 @@
           <t>2775.00</t>
         </is>
       </c>
-      <c r="T81" s="8" t="inlineStr"/>
-      <c r="U81" s="8" t="inlineStr"/>
-      <c r="V81" s="13" t="inlineStr">
+      <c r="T81" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="U81" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="V81" s="8" t="inlineStr"/>
+      <c r="W81" s="8" t="inlineStr"/>
+      <c r="X81" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="Y81" s="13" t="inlineStr">
         <is>
           <t>1437.00</t>
         </is>
       </c>
-      <c r="W81" s="13" t="inlineStr">
+      <c r="Z81" s="13" t="inlineStr">
         <is>
           <t>3061.00</t>
         </is>
       </c>
-      <c r="X81" s="15" t="inlineStr">
+      <c r="AA81" s="16" t="inlineStr">
         <is>
           <t>8373.00</t>
         </is>
       </c>
-      <c r="Y81" s="8" t="inlineStr">
+      <c r="AB81" s="8" t="inlineStr">
         <is>
           <t>7531.00</t>
         </is>
       </c>
-      <c r="Z81" s="9" t="inlineStr">
+      <c r="AC81" s="9" t="inlineStr">
         <is>
           <t>1005.00</t>
         </is>
       </c>
-      <c r="AA81" s="8" t="inlineStr"/>
-      <c r="AB81" s="10" t="n">
+      <c r="AD81" s="8" t="inlineStr"/>
+      <c r="AE81" s="10" t="n">
         <v>5765</v>
       </c>
-      <c r="AC81" s="10" t="n">
+      <c r="AF81" s="10" t="n">
         <v>955.5</v>
       </c>
-      <c r="AD81" s="12" t="n">
+      <c r="AG81" s="12" t="n">
         <v>0.4434080467771126</v>
       </c>
     </row>
@@ -5839,19 +6328,22 @@
       <c r="S82" s="9" t="inlineStr"/>
       <c r="T82" s="8" t="inlineStr"/>
       <c r="U82" s="8" t="inlineStr"/>
-      <c r="V82" s="9" t="inlineStr"/>
-      <c r="W82" s="9" t="inlineStr"/>
+      <c r="V82" s="8" t="inlineStr"/>
+      <c r="W82" s="8" t="inlineStr"/>
       <c r="X82" s="8" t="inlineStr"/>
-      <c r="Y82" s="8" t="inlineStr">
-        <is>
-          <t>5320.00</t>
-        </is>
-      </c>
+      <c r="Y82" s="9" t="inlineStr"/>
       <c r="Z82" s="9" t="inlineStr"/>
       <c r="AA82" s="8" t="inlineStr"/>
-      <c r="AB82" s="10" t="inlineStr"/>
-      <c r="AC82" s="11" t="inlineStr"/>
-      <c r="AD82" s="12" t="inlineStr"/>
+      <c r="AB82" s="8" t="inlineStr">
+        <is>
+          <t>5320.00</t>
+        </is>
+      </c>
+      <c r="AC82" s="9" t="inlineStr"/>
+      <c r="AD82" s="8" t="inlineStr"/>
+      <c r="AE82" s="10" t="inlineStr"/>
+      <c r="AF82" s="11" t="inlineStr"/>
+      <c r="AG82" s="12" t="inlineStr"/>
     </row>
     <row r="83" ht="24" customHeight="1">
       <c r="A83" s="1" t="n"/>
@@ -5879,19 +6371,22 @@
       <c r="S83" s="9" t="inlineStr"/>
       <c r="T83" s="8" t="inlineStr"/>
       <c r="U83" s="8" t="inlineStr"/>
-      <c r="V83" s="9" t="inlineStr"/>
-      <c r="W83" s="9" t="inlineStr"/>
+      <c r="V83" s="8" t="inlineStr"/>
+      <c r="W83" s="8" t="inlineStr"/>
       <c r="X83" s="8" t="inlineStr"/>
-      <c r="Y83" s="8" t="inlineStr">
-        <is>
-          <t>2516.00</t>
-        </is>
-      </c>
+      <c r="Y83" s="9" t="inlineStr"/>
       <c r="Z83" s="9" t="inlineStr"/>
       <c r="AA83" s="8" t="inlineStr"/>
-      <c r="AB83" s="10" t="inlineStr"/>
-      <c r="AC83" s="11" t="inlineStr"/>
-      <c r="AD83" s="12" t="inlineStr"/>
+      <c r="AB83" s="8" t="inlineStr">
+        <is>
+          <t>2516.00</t>
+        </is>
+      </c>
+      <c r="AC83" s="9" t="inlineStr"/>
+      <c r="AD83" s="8" t="inlineStr"/>
+      <c r="AE83" s="10" t="inlineStr"/>
+      <c r="AF83" s="11" t="inlineStr"/>
+      <c r="AG83" s="12" t="inlineStr"/>
     </row>
     <row r="84" ht="24" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
@@ -5931,11 +6426,14 @@
       <c r="Y84" s="4" t="inlineStr"/>
       <c r="Z84" s="4" t="inlineStr"/>
       <c r="AA84" s="4" t="inlineStr"/>
-      <c r="AB84" s="5" t="inlineStr"/>
-      <c r="AC84" s="6" t="n">
+      <c r="AB84" s="4" t="inlineStr"/>
+      <c r="AC84" s="4" t="inlineStr"/>
+      <c r="AD84" s="4" t="inlineStr"/>
+      <c r="AE84" s="5" t="inlineStr"/>
+      <c r="AF84" s="6" t="n">
         <v>741.625</v>
       </c>
-      <c r="AD84" s="7" t="n">
+      <c r="AG84" s="7" t="n">
         <v>0.02488724605193393</v>
       </c>
     </row>
@@ -5987,11 +6485,14 @@
       <c r="Y85" s="8" t="inlineStr"/>
       <c r="Z85" s="8" t="inlineStr"/>
       <c r="AA85" s="8" t="inlineStr"/>
-      <c r="AB85" s="10" t="n">
+      <c r="AB85" s="8" t="inlineStr"/>
+      <c r="AC85" s="8" t="inlineStr"/>
+      <c r="AD85" s="8" t="inlineStr"/>
+      <c r="AE85" s="10" t="n">
         <v>11785.625</v>
       </c>
-      <c r="AC85" s="11" t="inlineStr"/>
-      <c r="AD85" s="12" t="inlineStr"/>
+      <c r="AF85" s="11" t="inlineStr"/>
+      <c r="AG85" s="12" t="inlineStr"/>
     </row>
     <row r="86" ht="24" customHeight="1">
       <c r="A86" s="1" t="n"/>
@@ -6029,9 +6530,12 @@
       <c r="Y86" s="8" t="inlineStr"/>
       <c r="Z86" s="8" t="inlineStr"/>
       <c r="AA86" s="8" t="inlineStr"/>
-      <c r="AB86" s="10" t="inlineStr"/>
-      <c r="AC86" s="11" t="inlineStr"/>
-      <c r="AD86" s="12" t="inlineStr"/>
+      <c r="AB86" s="8" t="inlineStr"/>
+      <c r="AC86" s="8" t="inlineStr"/>
+      <c r="AD86" s="8" t="inlineStr"/>
+      <c r="AE86" s="10" t="inlineStr"/>
+      <c r="AF86" s="11" t="inlineStr"/>
+      <c r="AG86" s="12" t="inlineStr"/>
     </row>
     <row r="87" ht="24" customHeight="1">
       <c r="A87" s="1" t="n"/>
@@ -6081,13 +6585,16 @@
       <c r="Y87" s="8" t="inlineStr"/>
       <c r="Z87" s="8" t="inlineStr"/>
       <c r="AA87" s="8" t="inlineStr"/>
-      <c r="AB87" s="10" t="n">
+      <c r="AB87" s="8" t="inlineStr"/>
+      <c r="AC87" s="8" t="inlineStr"/>
+      <c r="AD87" s="8" t="inlineStr"/>
+      <c r="AE87" s="10" t="n">
         <v>13229.25</v>
       </c>
-      <c r="AC87" s="10" t="n">
+      <c r="AF87" s="10" t="n">
         <v>1443.625</v>
       </c>
-      <c r="AD87" s="12" t="n">
+      <c r="AG87" s="12" t="n">
         <v>0.04844476734430894</v>
       </c>
     </row>
@@ -6127,9 +6634,12 @@
       <c r="Y88" s="8" t="inlineStr"/>
       <c r="Z88" s="8" t="inlineStr"/>
       <c r="AA88" s="8" t="inlineStr"/>
-      <c r="AB88" s="10" t="inlineStr"/>
-      <c r="AC88" s="11" t="inlineStr"/>
-      <c r="AD88" s="12" t="inlineStr"/>
+      <c r="AB88" s="8" t="inlineStr"/>
+      <c r="AC88" s="8" t="inlineStr"/>
+      <c r="AD88" s="8" t="inlineStr"/>
+      <c r="AE88" s="10" t="inlineStr"/>
+      <c r="AF88" s="11" t="inlineStr"/>
+      <c r="AG88" s="12" t="inlineStr"/>
     </row>
     <row r="89" ht="24" customHeight="1">
       <c r="A89" s="1" t="n"/>
@@ -6167,9 +6677,12 @@
       <c r="Y89" s="8" t="inlineStr"/>
       <c r="Z89" s="8" t="inlineStr"/>
       <c r="AA89" s="8" t="inlineStr"/>
-      <c r="AB89" s="10" t="inlineStr"/>
-      <c r="AC89" s="11" t="inlineStr"/>
-      <c r="AD89" s="12" t="inlineStr"/>
+      <c r="AB89" s="8" t="inlineStr"/>
+      <c r="AC89" s="8" t="inlineStr"/>
+      <c r="AD89" s="8" t="inlineStr"/>
+      <c r="AE89" s="10" t="inlineStr"/>
+      <c r="AF89" s="11" t="inlineStr"/>
+      <c r="AG89" s="12" t="inlineStr"/>
     </row>
     <row r="90" ht="24" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
@@ -6209,11 +6722,14 @@
       <c r="Y90" s="4" t="inlineStr"/>
       <c r="Z90" s="4" t="inlineStr"/>
       <c r="AA90" s="4" t="inlineStr"/>
-      <c r="AB90" s="5" t="inlineStr"/>
-      <c r="AC90" s="6" t="n">
+      <c r="AB90" s="4" t="inlineStr"/>
+      <c r="AC90" s="4" t="inlineStr"/>
+      <c r="AD90" s="4" t="inlineStr"/>
+      <c r="AE90" s="5" t="inlineStr"/>
+      <c r="AF90" s="6" t="n">
         <v>-35.66666666666669</v>
       </c>
-      <c r="AD90" s="7" t="n">
+      <c r="AG90" s="7" t="n">
         <v>-0.1302654005356709</v>
       </c>
     </row>
@@ -6259,17 +6775,20 @@
       <c r="W91" s="8" t="inlineStr"/>
       <c r="X91" s="8" t="inlineStr"/>
       <c r="Y91" s="8" t="inlineStr"/>
-      <c r="Z91" s="8" t="inlineStr">
+      <c r="Z91" s="8" t="inlineStr"/>
+      <c r="AA91" s="8" t="inlineStr"/>
+      <c r="AB91" s="8" t="inlineStr"/>
+      <c r="AC91" s="8" t="inlineStr">
         <is>
           <t>365.00</t>
         </is>
       </c>
-      <c r="AA91" s="8" t="inlineStr"/>
-      <c r="AB91" s="10" t="n">
+      <c r="AD91" s="8" t="inlineStr"/>
+      <c r="AE91" s="10" t="n">
         <v>473.3333333333333</v>
       </c>
-      <c r="AC91" s="11" t="inlineStr"/>
-      <c r="AD91" s="12" t="inlineStr"/>
+      <c r="AF91" s="11" t="inlineStr"/>
+      <c r="AG91" s="12" t="inlineStr"/>
     </row>
     <row r="92" ht="24" customHeight="1">
       <c r="A92" s="1" t="n"/>
@@ -6307,9 +6826,12 @@
       <c r="Y92" s="8" t="inlineStr"/>
       <c r="Z92" s="8" t="inlineStr"/>
       <c r="AA92" s="8" t="inlineStr"/>
-      <c r="AB92" s="10" t="inlineStr"/>
-      <c r="AC92" s="11" t="inlineStr"/>
-      <c r="AD92" s="12" t="inlineStr"/>
+      <c r="AB92" s="8" t="inlineStr"/>
+      <c r="AC92" s="8" t="inlineStr"/>
+      <c r="AD92" s="8" t="inlineStr"/>
+      <c r="AE92" s="10" t="inlineStr"/>
+      <c r="AF92" s="11" t="inlineStr"/>
+      <c r="AG92" s="12" t="inlineStr"/>
     </row>
     <row r="93" ht="24" customHeight="1">
       <c r="A93" s="1" t="n"/>
@@ -6318,7 +6840,7 @@
           <t>target: 16 (anchor 미설정)</t>
         </is>
       </c>
-      <c r="C93" s="14" t="inlineStr">
+      <c r="C93" s="15" t="inlineStr">
         <is>
           <t>RUNNING</t>
         </is>
@@ -6353,19 +6875,22 @@
       <c r="W93" s="8" t="inlineStr"/>
       <c r="X93" s="8" t="inlineStr"/>
       <c r="Y93" s="8" t="inlineStr"/>
-      <c r="Z93" s="8" t="inlineStr">
+      <c r="Z93" s="8" t="inlineStr"/>
+      <c r="AA93" s="8" t="inlineStr"/>
+      <c r="AB93" s="8" t="inlineStr"/>
+      <c r="AC93" s="8" t="inlineStr">
         <is>
           <t>375.00</t>
         </is>
       </c>
-      <c r="AA93" s="8" t="inlineStr"/>
-      <c r="AB93" s="10" t="n">
+      <c r="AD93" s="8" t="inlineStr"/>
+      <c r="AE93" s="10" t="n">
         <v>535.8333333333334</v>
       </c>
-      <c r="AC93" s="10" t="n">
+      <c r="AF93" s="10" t="n">
         <v>62.50000000000006</v>
       </c>
-      <c r="AD93" s="12" t="n">
+      <c r="AG93" s="12" t="n">
         <v>0.2282688093498906</v>
       </c>
     </row>
@@ -6407,11 +6932,14 @@
       <c r="Y94" s="4" t="inlineStr"/>
       <c r="Z94" s="4" t="inlineStr"/>
       <c r="AA94" s="4" t="inlineStr"/>
-      <c r="AB94" s="5" t="inlineStr"/>
-      <c r="AC94" s="6" t="n">
+      <c r="AB94" s="4" t="inlineStr"/>
+      <c r="AC94" s="4" t="inlineStr"/>
+      <c r="AD94" s="4" t="inlineStr"/>
+      <c r="AE94" s="5" t="inlineStr"/>
+      <c r="AF94" s="6" t="n">
         <v>-2611.333333333333</v>
       </c>
-      <c r="AD94" s="7" t="n">
+      <c r="AG94" s="7" t="n">
         <v>-0.8754050731925354</v>
       </c>
     </row>
@@ -6465,13 +6993,16 @@
       <c r="W95" s="8" t="inlineStr"/>
       <c r="X95" s="8" t="inlineStr"/>
       <c r="Y95" s="8" t="inlineStr"/>
-      <c r="Z95" s="9" t="inlineStr"/>
+      <c r="Z95" s="8" t="inlineStr"/>
       <c r="AA95" s="8" t="inlineStr"/>
-      <c r="AB95" s="10" t="n">
+      <c r="AB95" s="8" t="inlineStr"/>
+      <c r="AC95" s="9" t="inlineStr"/>
+      <c r="AD95" s="8" t="inlineStr"/>
+      <c r="AE95" s="10" t="n">
         <v>1596.666666666667</v>
       </c>
-      <c r="AC95" s="11" t="inlineStr"/>
-      <c r="AD95" s="12" t="inlineStr"/>
+      <c r="AF95" s="11" t="inlineStr"/>
+      <c r="AG95" s="12" t="inlineStr"/>
     </row>
     <row r="96" ht="24" customHeight="1">
       <c r="A96" s="1" t="n"/>
@@ -6515,11 +7046,14 @@
       <c r="W96" s="8" t="inlineStr"/>
       <c r="X96" s="8" t="inlineStr"/>
       <c r="Y96" s="8" t="inlineStr"/>
-      <c r="Z96" s="9" t="inlineStr"/>
+      <c r="Z96" s="8" t="inlineStr"/>
       <c r="AA96" s="8" t="inlineStr"/>
-      <c r="AB96" s="10" t="inlineStr"/>
-      <c r="AC96" s="11" t="inlineStr"/>
-      <c r="AD96" s="12" t="inlineStr"/>
+      <c r="AB96" s="8" t="inlineStr"/>
+      <c r="AC96" s="9" t="inlineStr"/>
+      <c r="AD96" s="8" t="inlineStr"/>
+      <c r="AE96" s="10" t="inlineStr"/>
+      <c r="AF96" s="11" t="inlineStr"/>
+      <c r="AG96" s="12" t="inlineStr"/>
     </row>
     <row r="97" ht="24" customHeight="1">
       <c r="A97" s="1" t="n"/>
@@ -6528,7 +7062,11 @@
           <t>target: 16 (anchor 미설정)</t>
         </is>
       </c>
-      <c r="C97" s="8" t="inlineStr"/>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="D97" s="8" t="inlineStr"/>
       <c r="E97" s="8" t="inlineStr">
         <is>
@@ -6558,36 +7096,43 @@
           <t>760.00</t>
         </is>
       </c>
-      <c r="Q97" s="14" t="inlineStr">
+      <c r="Q97" s="15" t="inlineStr">
         <is>
           <t>RUNNING</t>
         </is>
       </c>
-      <c r="R97" s="15" t="inlineStr">
+      <c r="R97" s="16" t="inlineStr">
         <is>
           <t>2900.00</t>
         </is>
       </c>
-      <c r="S97" s="8" t="inlineStr"/>
+      <c r="S97" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="T97" s="8" t="inlineStr"/>
       <c r="U97" s="8" t="inlineStr"/>
       <c r="V97" s="8" t="inlineStr"/>
       <c r="W97" s="8" t="inlineStr"/>
       <c r="X97" s="8" t="inlineStr"/>
       <c r="Y97" s="8" t="inlineStr"/>
-      <c r="Z97" s="13" t="inlineStr">
+      <c r="Z97" s="8" t="inlineStr"/>
+      <c r="AA97" s="8" t="inlineStr"/>
+      <c r="AB97" s="8" t="inlineStr"/>
+      <c r="AC97" s="13" t="inlineStr">
         <is>
           <t>1760.00</t>
         </is>
       </c>
-      <c r="AA97" s="8" t="inlineStr"/>
-      <c r="AB97" s="10" t="n">
+      <c r="AD97" s="8" t="inlineStr"/>
+      <c r="AE97" s="10" t="n">
         <v>1673.333333333333</v>
       </c>
-      <c r="AC97" s="10" t="n">
+      <c r="AF97" s="10" t="n">
         <v>76.66666666666652</v>
       </c>
-      <c r="AD97" s="12" t="n">
+      <c r="AG97" s="12" t="n">
         <v>0.02570119566431998</v>
       </c>
     </row>
@@ -6629,11 +7174,14 @@
       <c r="Y98" s="4" t="inlineStr"/>
       <c r="Z98" s="4" t="inlineStr"/>
       <c r="AA98" s="4" t="inlineStr"/>
-      <c r="AB98" s="5" t="inlineStr"/>
-      <c r="AC98" s="6" t="n">
+      <c r="AB98" s="4" t="inlineStr"/>
+      <c r="AC98" s="4" t="inlineStr"/>
+      <c r="AD98" s="4" t="inlineStr"/>
+      <c r="AE98" s="5" t="inlineStr"/>
+      <c r="AF98" s="6" t="n">
         <v>-2583.375</v>
       </c>
-      <c r="AD98" s="7" t="n">
+      <c r="AG98" s="7" t="n">
         <v>-2.420023419203747</v>
       </c>
     </row>
@@ -6695,17 +7243,20 @@
       <c r="W99" s="8" t="inlineStr"/>
       <c r="X99" s="8" t="inlineStr"/>
       <c r="Y99" s="8" t="inlineStr"/>
-      <c r="Z99" s="8" t="inlineStr">
+      <c r="Z99" s="8" t="inlineStr"/>
+      <c r="AA99" s="8" t="inlineStr"/>
+      <c r="AB99" s="8" t="inlineStr"/>
+      <c r="AC99" s="8" t="inlineStr">
         <is>
           <t>6289.00</t>
         </is>
       </c>
-      <c r="AA99" s="8" t="inlineStr"/>
-      <c r="AB99" s="10" t="n">
+      <c r="AD99" s="8" t="inlineStr"/>
+      <c r="AE99" s="10" t="n">
         <v>5829.625</v>
       </c>
-      <c r="AC99" s="11" t="inlineStr"/>
-      <c r="AD99" s="12" t="inlineStr"/>
+      <c r="AF99" s="11" t="inlineStr"/>
+      <c r="AG99" s="12" t="inlineStr"/>
     </row>
     <row r="100" ht="24" customHeight="1">
       <c r="A100" s="1" t="n"/>
@@ -6745,15 +7296,18 @@
       <c r="W100" s="8" t="inlineStr"/>
       <c r="X100" s="8" t="inlineStr"/>
       <c r="Y100" s="8" t="inlineStr"/>
-      <c r="Z100" s="8" t="inlineStr">
+      <c r="Z100" s="8" t="inlineStr"/>
+      <c r="AA100" s="8" t="inlineStr"/>
+      <c r="AB100" s="8" t="inlineStr"/>
+      <c r="AC100" s="8" t="inlineStr">
         <is>
           <t>6587.00</t>
         </is>
       </c>
-      <c r="AA100" s="8" t="inlineStr"/>
-      <c r="AB100" s="10" t="inlineStr"/>
-      <c r="AC100" s="11" t="inlineStr"/>
-      <c r="AD100" s="12" t="inlineStr"/>
+      <c r="AD100" s="8" t="inlineStr"/>
+      <c r="AE100" s="10" t="inlineStr"/>
+      <c r="AF100" s="11" t="inlineStr"/>
+      <c r="AG100" s="12" t="inlineStr"/>
     </row>
     <row r="101" ht="24" customHeight="1">
       <c r="A101" s="1" t="n"/>
@@ -6762,7 +7316,11 @@
           <t>target: 16 (anchor 미설정)</t>
         </is>
       </c>
-      <c r="C101" s="8" t="inlineStr"/>
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="D101" s="8" t="inlineStr"/>
       <c r="E101" s="8" t="inlineStr">
         <is>
@@ -6806,30 +7364,45 @@
           <t>5596.50</t>
         </is>
       </c>
-      <c r="S101" s="15" t="inlineStr">
+      <c r="S101" s="16" t="inlineStr">
         <is>
           <t>6424.00</t>
         </is>
       </c>
-      <c r="T101" s="8" t="inlineStr"/>
-      <c r="U101" s="8" t="inlineStr"/>
+      <c r="T101" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="U101" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="V101" s="8" t="inlineStr"/>
       <c r="W101" s="8" t="inlineStr"/>
       <c r="X101" s="8" t="inlineStr"/>
       <c r="Y101" s="8" t="inlineStr"/>
-      <c r="Z101" s="8" t="inlineStr">
+      <c r="Z101" s="8" t="inlineStr"/>
+      <c r="AA101" s="8" t="inlineStr"/>
+      <c r="AB101" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="AC101" s="8" t="inlineStr">
         <is>
           <t>6796.50</t>
         </is>
       </c>
-      <c r="AA101" s="8" t="inlineStr"/>
-      <c r="AB101" s="10" t="n">
+      <c r="AD101" s="8" t="inlineStr"/>
+      <c r="AE101" s="10" t="n">
         <v>6662.25</v>
       </c>
-      <c r="AC101" s="10" t="n">
+      <c r="AF101" s="10" t="n">
         <v>832.625</v>
       </c>
-      <c r="AD101" s="12" t="n">
+      <c r="AG101" s="12" t="n">
         <v>0.779976580796253</v>
       </c>
     </row>
@@ -6871,11 +7444,14 @@
       <c r="Y102" s="4" t="inlineStr"/>
       <c r="Z102" s="4" t="inlineStr"/>
       <c r="AA102" s="4" t="inlineStr"/>
-      <c r="AB102" s="5" t="inlineStr"/>
-      <c r="AC102" s="6" t="n">
+      <c r="AB102" s="4" t="inlineStr"/>
+      <c r="AC102" s="4" t="inlineStr"/>
+      <c r="AD102" s="4" t="inlineStr"/>
+      <c r="AE102" s="5" t="inlineStr"/>
+      <c r="AF102" s="6" t="n">
         <v>-1044.5</v>
       </c>
-      <c r="AD102" s="7" t="n">
+      <c r="AG102" s="7" t="n">
         <v>-0.04646807071866464</v>
       </c>
     </row>
@@ -6923,11 +7499,14 @@
       <c r="Y103" s="8" t="inlineStr"/>
       <c r="Z103" s="8" t="inlineStr"/>
       <c r="AA103" s="8" t="inlineStr"/>
-      <c r="AB103" s="10" t="n">
+      <c r="AB103" s="8" t="inlineStr"/>
+      <c r="AC103" s="8" t="inlineStr"/>
+      <c r="AD103" s="8" t="inlineStr"/>
+      <c r="AE103" s="10" t="n">
         <v>25137.5</v>
       </c>
-      <c r="AC103" s="11" t="inlineStr"/>
-      <c r="AD103" s="12" t="inlineStr"/>
+      <c r="AF103" s="11" t="inlineStr"/>
+      <c r="AG103" s="12" t="inlineStr"/>
     </row>
     <row r="104" ht="24" customHeight="1">
       <c r="A104" s="1" t="n"/>
@@ -6965,9 +7544,12 @@
       <c r="Y104" s="8" t="inlineStr"/>
       <c r="Z104" s="8" t="inlineStr"/>
       <c r="AA104" s="8" t="inlineStr"/>
-      <c r="AB104" s="10" t="inlineStr"/>
-      <c r="AC104" s="11" t="inlineStr"/>
-      <c r="AD104" s="12" t="inlineStr"/>
+      <c r="AB104" s="8" t="inlineStr"/>
+      <c r="AC104" s="8" t="inlineStr"/>
+      <c r="AD104" s="8" t="inlineStr"/>
+      <c r="AE104" s="10" t="inlineStr"/>
+      <c r="AF104" s="11" t="inlineStr"/>
+      <c r="AG104" s="12" t="inlineStr"/>
     </row>
     <row r="105" ht="24" customHeight="1">
       <c r="A105" s="1" t="n"/>
@@ -6993,7 +7575,7 @@
           <t>20245.00</t>
         </is>
       </c>
-      <c r="L105" s="14" t="inlineStr">
+      <c r="L105" s="15" t="inlineStr">
         <is>
           <t>RUNNING</t>
         </is>
@@ -7013,13 +7595,16 @@
       <c r="Y105" s="8" t="inlineStr"/>
       <c r="Z105" s="8" t="inlineStr"/>
       <c r="AA105" s="8" t="inlineStr"/>
-      <c r="AB105" s="10" t="n">
+      <c r="AB105" s="8" t="inlineStr"/>
+      <c r="AC105" s="8" t="inlineStr"/>
+      <c r="AD105" s="8" t="inlineStr"/>
+      <c r="AE105" s="10" t="n">
         <v>25177.5</v>
       </c>
-      <c r="AC105" s="10" t="n">
+      <c r="AF105" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="AD105" s="12" t="n">
+      <c r="AG105" s="12" t="n">
         <v>0.001779533584247569</v>
       </c>
     </row>
@@ -7059,9 +7644,12 @@
       <c r="Y106" s="8" t="inlineStr"/>
       <c r="Z106" s="8" t="inlineStr"/>
       <c r="AA106" s="8" t="inlineStr"/>
-      <c r="AB106" s="10" t="inlineStr"/>
-      <c r="AC106" s="11" t="inlineStr"/>
-      <c r="AD106" s="12" t="inlineStr"/>
+      <c r="AB106" s="8" t="inlineStr"/>
+      <c r="AC106" s="8" t="inlineStr"/>
+      <c r="AD106" s="8" t="inlineStr"/>
+      <c r="AE106" s="10" t="inlineStr"/>
+      <c r="AF106" s="11" t="inlineStr"/>
+      <c r="AG106" s="12" t="inlineStr"/>
     </row>
     <row r="107" ht="24" customHeight="1">
       <c r="A107" s="1" t="n"/>
@@ -7099,9 +7687,12 @@
       <c r="Y107" s="8" t="inlineStr"/>
       <c r="Z107" s="8" t="inlineStr"/>
       <c r="AA107" s="8" t="inlineStr"/>
-      <c r="AB107" s="10" t="inlineStr"/>
-      <c r="AC107" s="11" t="inlineStr"/>
-      <c r="AD107" s="12" t="inlineStr"/>
+      <c r="AB107" s="8" t="inlineStr"/>
+      <c r="AC107" s="8" t="inlineStr"/>
+      <c r="AD107" s="8" t="inlineStr"/>
+      <c r="AE107" s="10" t="inlineStr"/>
+      <c r="AF107" s="11" t="inlineStr"/>
+      <c r="AG107" s="12" t="inlineStr"/>
     </row>
     <row r="108" ht="24" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
@@ -7141,11 +7732,14 @@
       <c r="Y108" s="4" t="inlineStr"/>
       <c r="Z108" s="4" t="inlineStr"/>
       <c r="AA108" s="4" t="inlineStr"/>
-      <c r="AB108" s="5" t="inlineStr"/>
-      <c r="AC108" s="6" t="n">
+      <c r="AB108" s="4" t="inlineStr"/>
+      <c r="AC108" s="4" t="inlineStr"/>
+      <c r="AD108" s="4" t="inlineStr"/>
+      <c r="AE108" s="5" t="inlineStr"/>
+      <c r="AF108" s="6" t="n">
         <v>-699.3333333333333</v>
       </c>
-      <c r="AD108" s="7" t="n">
+      <c r="AG108" s="7" t="n">
         <v>-0.1052531242317977</v>
       </c>
     </row>
@@ -7201,11 +7795,14 @@
       <c r="Y109" s="8" t="inlineStr"/>
       <c r="Z109" s="8" t="inlineStr"/>
       <c r="AA109" s="8" t="inlineStr"/>
-      <c r="AB109" s="10" t="n">
+      <c r="AB109" s="8" t="inlineStr"/>
+      <c r="AC109" s="8" t="inlineStr"/>
+      <c r="AD109" s="8" t="inlineStr"/>
+      <c r="AE109" s="10" t="n">
         <v>1973.666666666667</v>
       </c>
-      <c r="AC109" s="11" t="inlineStr"/>
-      <c r="AD109" s="12" t="inlineStr"/>
+      <c r="AF109" s="11" t="inlineStr"/>
+      <c r="AG109" s="12" t="inlineStr"/>
     </row>
     <row r="110" ht="24" customHeight="1">
       <c r="A110" s="1" t="n"/>
@@ -7243,9 +7840,12 @@
       <c r="Y110" s="8" t="inlineStr"/>
       <c r="Z110" s="8" t="inlineStr"/>
       <c r="AA110" s="8" t="inlineStr"/>
-      <c r="AB110" s="10" t="inlineStr"/>
-      <c r="AC110" s="11" t="inlineStr"/>
-      <c r="AD110" s="12" t="inlineStr"/>
+      <c r="AB110" s="8" t="inlineStr"/>
+      <c r="AC110" s="8" t="inlineStr"/>
+      <c r="AD110" s="8" t="inlineStr"/>
+      <c r="AE110" s="10" t="inlineStr"/>
+      <c r="AF110" s="11" t="inlineStr"/>
+      <c r="AG110" s="12" t="inlineStr"/>
     </row>
     <row r="111" ht="24" customHeight="1">
       <c r="A111" s="1" t="n"/>
@@ -7291,13 +7891,16 @@
       <c r="Y111" s="8" t="inlineStr"/>
       <c r="Z111" s="8" t="inlineStr"/>
       <c r="AA111" s="8" t="inlineStr"/>
-      <c r="AB111" s="10" t="n">
+      <c r="AB111" s="8" t="inlineStr"/>
+      <c r="AC111" s="8" t="inlineStr"/>
+      <c r="AD111" s="8" t="inlineStr"/>
+      <c r="AE111" s="10" t="n">
         <v>2007.166666666667</v>
       </c>
-      <c r="AC111" s="10" t="n">
+      <c r="AF111" s="10" t="n">
         <v>33.5</v>
       </c>
-      <c r="AD111" s="12" t="n">
+      <c r="AG111" s="12" t="n">
         <v>0.005041915626928344</v>
       </c>
     </row>
@@ -7341,9 +7944,12 @@
       <c r="Y112" s="8" t="inlineStr"/>
       <c r="Z112" s="8" t="inlineStr"/>
       <c r="AA112" s="8" t="inlineStr"/>
-      <c r="AB112" s="10" t="inlineStr"/>
-      <c r="AC112" s="11" t="inlineStr"/>
-      <c r="AD112" s="12" t="inlineStr"/>
+      <c r="AB112" s="8" t="inlineStr"/>
+      <c r="AC112" s="8" t="inlineStr"/>
+      <c r="AD112" s="8" t="inlineStr"/>
+      <c r="AE112" s="10" t="inlineStr"/>
+      <c r="AF112" s="11" t="inlineStr"/>
+      <c r="AG112" s="12" t="inlineStr"/>
     </row>
     <row r="113" ht="24" customHeight="1">
       <c r="A113" s="1" t="n"/>
@@ -7385,9 +7991,12 @@
       <c r="Y113" s="8" t="inlineStr"/>
       <c r="Z113" s="8" t="inlineStr"/>
       <c r="AA113" s="8" t="inlineStr"/>
-      <c r="AB113" s="10" t="inlineStr"/>
-      <c r="AC113" s="11" t="inlineStr"/>
-      <c r="AD113" s="12" t="inlineStr"/>
+      <c r="AB113" s="8" t="inlineStr"/>
+      <c r="AC113" s="8" t="inlineStr"/>
+      <c r="AD113" s="8" t="inlineStr"/>
+      <c r="AE113" s="10" t="inlineStr"/>
+      <c r="AF113" s="11" t="inlineStr"/>
+      <c r="AG113" s="12" t="inlineStr"/>
     </row>
     <row r="114" ht="24" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
@@ -7427,11 +8036,14 @@
       <c r="Y114" s="4" t="inlineStr"/>
       <c r="Z114" s="4" t="inlineStr"/>
       <c r="AA114" s="4" t="inlineStr"/>
-      <c r="AB114" s="5" t="inlineStr"/>
-      <c r="AC114" s="6" t="n">
+      <c r="AB114" s="4" t="inlineStr"/>
+      <c r="AC114" s="4" t="inlineStr"/>
+      <c r="AD114" s="4" t="inlineStr"/>
+      <c r="AE114" s="5" t="inlineStr"/>
+      <c r="AF114" s="6" t="n">
         <v>-5.4</v>
       </c>
-      <c r="AD114" s="7" t="n">
+      <c r="AG114" s="7" t="n">
         <v>-0.1529745042492918</v>
       </c>
     </row>
@@ -7483,11 +8095,14 @@
       <c r="Y115" s="8" t="inlineStr"/>
       <c r="Z115" s="8" t="inlineStr"/>
       <c r="AA115" s="8" t="inlineStr"/>
-      <c r="AB115" s="10" t="n">
+      <c r="AB115" s="8" t="inlineStr"/>
+      <c r="AC115" s="8" t="inlineStr"/>
+      <c r="AD115" s="8" t="inlineStr"/>
+      <c r="AE115" s="10" t="n">
         <v>5.6</v>
       </c>
-      <c r="AC115" s="11" t="inlineStr"/>
-      <c r="AD115" s="12" t="inlineStr"/>
+      <c r="AF115" s="11" t="inlineStr"/>
+      <c r="AG115" s="12" t="inlineStr"/>
     </row>
     <row r="116" ht="24" customHeight="1">
       <c r="A116" s="1" t="n"/>
@@ -7535,19 +8150,22 @@
       <c r="W116" s="8" t="inlineStr"/>
       <c r="X116" s="8" t="inlineStr"/>
       <c r="Y116" s="8" t="inlineStr"/>
-      <c r="Z116" s="15" t="inlineStr">
+      <c r="Z116" s="8" t="inlineStr"/>
+      <c r="AA116" s="8" t="inlineStr"/>
+      <c r="AB116" s="8" t="inlineStr"/>
+      <c r="AC116" s="16" t="inlineStr">
         <is>
           <t>16.30</t>
         </is>
       </c>
-      <c r="AA116" s="8" t="inlineStr"/>
-      <c r="AB116" s="10" t="n">
+      <c r="AD116" s="8" t="inlineStr"/>
+      <c r="AE116" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="AC116" s="10" t="n">
+      <c r="AF116" s="10" t="n">
         <v>3.4</v>
       </c>
-      <c r="AD116" s="12" t="n">
+      <c r="AG116" s="12" t="n">
         <v>0.09631728045325781</v>
       </c>
     </row>
@@ -7587,9 +8205,12 @@
       <c r="Y117" s="8" t="inlineStr"/>
       <c r="Z117" s="8" t="inlineStr"/>
       <c r="AA117" s="8" t="inlineStr"/>
-      <c r="AB117" s="10" t="inlineStr"/>
-      <c r="AC117" s="11" t="inlineStr"/>
-      <c r="AD117" s="12" t="inlineStr"/>
+      <c r="AB117" s="8" t="inlineStr"/>
+      <c r="AC117" s="8" t="inlineStr"/>
+      <c r="AD117" s="8" t="inlineStr"/>
+      <c r="AE117" s="10" t="inlineStr"/>
+      <c r="AF117" s="11" t="inlineStr"/>
+      <c r="AG117" s="12" t="inlineStr"/>
     </row>
     <row r="118" ht="24" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
@@ -7629,11 +8250,14 @@
       <c r="Y118" s="4" t="inlineStr"/>
       <c r="Z118" s="4" t="inlineStr"/>
       <c r="AA118" s="4" t="inlineStr"/>
-      <c r="AB118" s="5" t="inlineStr"/>
-      <c r="AC118" s="6" t="n">
+      <c r="AB118" s="4" t="inlineStr"/>
+      <c r="AC118" s="4" t="inlineStr"/>
+      <c r="AD118" s="4" t="inlineStr"/>
+      <c r="AE118" s="5" t="inlineStr"/>
+      <c r="AF118" s="6" t="n">
         <v>-6778.35</v>
       </c>
-      <c r="AD118" s="7" t="n">
+      <c r="AG118" s="7" t="n">
         <v>-0.09746514557187719</v>
       </c>
     </row>
@@ -7687,17 +8311,20 @@
       <c r="W119" s="8" t="inlineStr"/>
       <c r="X119" s="8" t="inlineStr"/>
       <c r="Y119" s="8" t="inlineStr"/>
-      <c r="Z119" s="8" t="inlineStr">
+      <c r="Z119" s="8" t="inlineStr"/>
+      <c r="AA119" s="8" t="inlineStr"/>
+      <c r="AB119" s="8" t="inlineStr"/>
+      <c r="AC119" s="8" t="inlineStr">
         <is>
           <t>159.50</t>
         </is>
       </c>
-      <c r="AA119" s="8" t="inlineStr"/>
-      <c r="AB119" s="10" t="n">
+      <c r="AD119" s="8" t="inlineStr"/>
+      <c r="AE119" s="10" t="n">
         <v>1002.65</v>
       </c>
-      <c r="AC119" s="11" t="inlineStr"/>
-      <c r="AD119" s="12" t="inlineStr"/>
+      <c r="AF119" s="11" t="inlineStr"/>
+      <c r="AG119" s="12" t="inlineStr"/>
     </row>
     <row r="120" ht="24" customHeight="1">
       <c r="A120" s="1" t="n"/>
@@ -7749,19 +8376,22 @@
       <c r="W120" s="8" t="inlineStr"/>
       <c r="X120" s="8" t="inlineStr"/>
       <c r="Y120" s="8" t="inlineStr"/>
-      <c r="Z120" s="8" t="inlineStr">
+      <c r="Z120" s="8" t="inlineStr"/>
+      <c r="AA120" s="8" t="inlineStr"/>
+      <c r="AB120" s="8" t="inlineStr"/>
+      <c r="AC120" s="8" t="inlineStr">
         <is>
           <t>153.20</t>
         </is>
       </c>
-      <c r="AA120" s="8" t="inlineStr"/>
-      <c r="AB120" s="10" t="n">
+      <c r="AD120" s="8" t="inlineStr"/>
+      <c r="AE120" s="10" t="n">
         <v>152.9875</v>
       </c>
-      <c r="AC120" s="10" t="n">
+      <c r="AF120" s="10" t="n">
         <v>849.6624999999999</v>
       </c>
-      <c r="AD120" s="12" t="n">
+      <c r="AG120" s="12" t="n">
         <v>-0.01221720319096315</v>
       </c>
     </row>
@@ -7803,11 +8433,14 @@
       <c r="Y121" s="4" t="inlineStr"/>
       <c r="Z121" s="4" t="inlineStr"/>
       <c r="AA121" s="4" t="inlineStr"/>
-      <c r="AB121" s="5" t="inlineStr"/>
-      <c r="AC121" s="6" t="n">
+      <c r="AB121" s="4" t="inlineStr"/>
+      <c r="AC121" s="4" t="inlineStr"/>
+      <c r="AD121" s="4" t="inlineStr"/>
+      <c r="AE121" s="5" t="inlineStr"/>
+      <c r="AF121" s="6" t="n">
         <v>-1662.9375</v>
       </c>
-      <c r="AD121" s="7" t="n">
+      <c r="AG121" s="7" t="n">
         <v>-0.1251166193919239</v>
       </c>
     </row>
@@ -7863,11 +8496,14 @@
       <c r="Y122" s="8" t="inlineStr"/>
       <c r="Z122" s="8" t="inlineStr"/>
       <c r="AA122" s="8" t="inlineStr"/>
-      <c r="AB122" s="10" t="n">
+      <c r="AB122" s="8" t="inlineStr"/>
+      <c r="AC122" s="8" t="inlineStr"/>
+      <c r="AD122" s="8" t="inlineStr"/>
+      <c r="AE122" s="10" t="n">
         <v>2859.0625</v>
       </c>
-      <c r="AC122" s="11" t="inlineStr"/>
-      <c r="AD122" s="12" t="inlineStr"/>
+      <c r="AF122" s="11" t="inlineStr"/>
+      <c r="AG122" s="12" t="inlineStr"/>
     </row>
     <row r="123" ht="24" customHeight="1">
       <c r="A123" s="1" t="n"/>
@@ -7917,9 +8553,12 @@
       <c r="Y123" s="8" t="inlineStr"/>
       <c r="Z123" s="8" t="inlineStr"/>
       <c r="AA123" s="8" t="inlineStr"/>
-      <c r="AB123" s="10" t="inlineStr"/>
-      <c r="AC123" s="11" t="inlineStr"/>
-      <c r="AD123" s="12" t="inlineStr"/>
+      <c r="AB123" s="8" t="inlineStr"/>
+      <c r="AC123" s="8" t="inlineStr"/>
+      <c r="AD123" s="8" t="inlineStr"/>
+      <c r="AE123" s="10" t="inlineStr"/>
+      <c r="AF123" s="11" t="inlineStr"/>
+      <c r="AG123" s="12" t="inlineStr"/>
     </row>
     <row r="124" ht="24" customHeight="1">
       <c r="A124" s="1" t="n"/>
@@ -7977,13 +8616,16 @@
       <c r="Y124" s="8" t="inlineStr"/>
       <c r="Z124" s="8" t="inlineStr"/>
       <c r="AA124" s="8" t="inlineStr"/>
-      <c r="AB124" s="10" t="n">
+      <c r="AB124" s="8" t="inlineStr"/>
+      <c r="AC124" s="8" t="inlineStr"/>
+      <c r="AD124" s="8" t="inlineStr"/>
+      <c r="AE124" s="10" t="n">
         <v>3065.625</v>
       </c>
-      <c r="AC124" s="10" t="n">
+      <c r="AF124" s="10" t="n">
         <v>206.5625</v>
       </c>
-      <c r="AD124" s="12" t="n">
+      <c r="AG124" s="12" t="n">
         <v>0.01554141493179646</v>
       </c>
     </row>
@@ -8025,11 +8667,14 @@
       <c r="Y125" s="4" t="inlineStr"/>
       <c r="Z125" s="4" t="inlineStr"/>
       <c r="AA125" s="4" t="inlineStr"/>
-      <c r="AB125" s="5" t="inlineStr"/>
-      <c r="AC125" s="6" t="n">
+      <c r="AB125" s="4" t="inlineStr"/>
+      <c r="AC125" s="4" t="inlineStr"/>
+      <c r="AD125" s="4" t="inlineStr"/>
+      <c r="AE125" s="5" t="inlineStr"/>
+      <c r="AF125" s="6" t="n">
         <v>-5012.333333333334</v>
       </c>
-      <c r="AD125" s="7" t="n">
+      <c r="AG125" s="7" t="n">
         <v>-0.6398587264100765</v>
       </c>
     </row>
@@ -8076,7 +8721,11 @@
           <t>17810.00</t>
         </is>
       </c>
-      <c r="S126" s="8" t="inlineStr"/>
+      <c r="S126" s="17" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="T126" s="8" t="inlineStr"/>
       <c r="U126" s="8" t="inlineStr"/>
       <c r="V126" s="8" t="inlineStr"/>
@@ -8085,11 +8734,14 @@
       <c r="Y126" s="8" t="inlineStr"/>
       <c r="Z126" s="8" t="inlineStr"/>
       <c r="AA126" s="8" t="inlineStr"/>
-      <c r="AB126" s="10" t="n">
+      <c r="AB126" s="8" t="inlineStr"/>
+      <c r="AC126" s="8" t="inlineStr"/>
+      <c r="AD126" s="8" t="inlineStr"/>
+      <c r="AE126" s="10" t="n">
         <v>12551.66666666667</v>
       </c>
-      <c r="AC126" s="11" t="inlineStr"/>
-      <c r="AD126" s="12" t="inlineStr"/>
+      <c r="AF126" s="11" t="inlineStr"/>
+      <c r="AG126" s="12" t="inlineStr"/>
     </row>
     <row r="127" ht="24" customHeight="1">
       <c r="A127" s="1" t="n"/>
@@ -8135,9 +8787,12 @@
       <c r="Y127" s="8" t="inlineStr"/>
       <c r="Z127" s="8" t="inlineStr"/>
       <c r="AA127" s="8" t="inlineStr"/>
-      <c r="AB127" s="10" t="inlineStr"/>
-      <c r="AC127" s="11" t="inlineStr"/>
-      <c r="AD127" s="12" t="inlineStr"/>
+      <c r="AB127" s="8" t="inlineStr"/>
+      <c r="AC127" s="8" t="inlineStr"/>
+      <c r="AD127" s="8" t="inlineStr"/>
+      <c r="AE127" s="10" t="inlineStr"/>
+      <c r="AF127" s="11" t="inlineStr"/>
+      <c r="AG127" s="12" t="inlineStr"/>
     </row>
     <row r="128" ht="24" customHeight="1">
       <c r="A128" s="1" t="n"/>
@@ -8177,35 +8832,46 @@
           <t>16980.00</t>
         </is>
       </c>
-      <c r="R128" s="15" t="inlineStr">
+      <c r="R128" s="16" t="inlineStr">
         <is>
           <t>16410.00</t>
         </is>
       </c>
-      <c r="S128" s="15" t="inlineStr">
+      <c r="S128" s="16" t="inlineStr">
         <is>
           <t>18865.00</t>
         </is>
       </c>
-      <c r="T128" s="14" t="inlineStr">
+      <c r="T128" s="15" t="inlineStr">
         <is>
           <t>RUNNING</t>
         </is>
       </c>
-      <c r="U128" s="8" t="inlineStr"/>
+      <c r="U128" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
       <c r="V128" s="8" t="inlineStr"/>
       <c r="W128" s="8" t="inlineStr"/>
       <c r="X128" s="8" t="inlineStr"/>
       <c r="Y128" s="8" t="inlineStr"/>
       <c r="Z128" s="8" t="inlineStr"/>
       <c r="AA128" s="8" t="inlineStr"/>
-      <c r="AB128" s="10" t="n">
+      <c r="AB128" s="8" t="inlineStr"/>
+      <c r="AC128" s="14" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="AD128" s="8" t="inlineStr"/>
+      <c r="AE128" s="10" t="n">
         <v>15426.66666666667</v>
       </c>
-      <c r="AC128" s="10" t="n">
+      <c r="AF128" s="10" t="n">
         <v>2875</v>
       </c>
-      <c r="AD128" s="12" t="n">
+      <c r="AG128" s="12" t="n">
         <v>0.3670134677985575</v>
       </c>
     </row>
@@ -8247,11 +8913,14 @@
       <c r="Y129" s="4" t="inlineStr"/>
       <c r="Z129" s="4" t="inlineStr"/>
       <c r="AA129" s="4" t="inlineStr"/>
-      <c r="AB129" s="5" t="inlineStr"/>
-      <c r="AC129" s="6" t="n">
+      <c r="AB129" s="4" t="inlineStr"/>
+      <c r="AC129" s="4" t="inlineStr"/>
+      <c r="AD129" s="4" t="inlineStr"/>
+      <c r="AE129" s="5" t="inlineStr"/>
+      <c r="AF129" s="6" t="n">
         <v>-64.33333333333331</v>
       </c>
-      <c r="AD129" s="7" t="n">
+      <c r="AG129" s="7" t="n">
         <v>-0.001532245835744834</v>
       </c>
     </row>
@@ -8297,17 +8966,20 @@
       <c r="W130" s="8" t="inlineStr"/>
       <c r="X130" s="8" t="inlineStr"/>
       <c r="Y130" s="8" t="inlineStr"/>
-      <c r="Z130" s="8" t="inlineStr">
+      <c r="Z130" s="8" t="inlineStr"/>
+      <c r="AA130" s="8" t="inlineStr"/>
+      <c r="AB130" s="8" t="inlineStr"/>
+      <c r="AC130" s="8" t="inlineStr">
         <is>
           <t>470.00</t>
         </is>
       </c>
-      <c r="AA130" s="8" t="inlineStr"/>
-      <c r="AB130" s="10" t="n">
+      <c r="AD130" s="8" t="inlineStr"/>
+      <c r="AE130" s="10" t="n">
         <v>460.6666666666667</v>
       </c>
-      <c r="AC130" s="11" t="inlineStr"/>
-      <c r="AD130" s="12" t="inlineStr"/>
+      <c r="AF130" s="11" t="inlineStr"/>
+      <c r="AG130" s="12" t="inlineStr"/>
     </row>
     <row r="131" ht="24" customHeight="1">
       <c r="A131" s="1" t="n"/>
@@ -8343,15 +9015,18 @@
       <c r="W131" s="8" t="inlineStr"/>
       <c r="X131" s="8" t="inlineStr"/>
       <c r="Y131" s="8" t="inlineStr"/>
-      <c r="Z131" s="8" t="inlineStr">
+      <c r="Z131" s="8" t="inlineStr"/>
+      <c r="AA131" s="8" t="inlineStr"/>
+      <c r="AB131" s="8" t="inlineStr"/>
+      <c r="AC131" s="8" t="inlineStr">
         <is>
           <t>557.00</t>
         </is>
       </c>
-      <c r="AA131" s="8" t="inlineStr"/>
-      <c r="AB131" s="10" t="inlineStr"/>
-      <c r="AC131" s="11" t="inlineStr"/>
-      <c r="AD131" s="12" t="inlineStr"/>
+      <c r="AD131" s="8" t="inlineStr"/>
+      <c r="AE131" s="10" t="inlineStr"/>
+      <c r="AF131" s="11" t="inlineStr"/>
+      <c r="AG131" s="12" t="inlineStr"/>
     </row>
     <row r="132" ht="24" customHeight="1">
       <c r="A132" s="1" t="n"/>
@@ -8391,19 +9066,22 @@
       <c r="W132" s="8" t="inlineStr"/>
       <c r="X132" s="8" t="inlineStr"/>
       <c r="Y132" s="8" t="inlineStr"/>
-      <c r="Z132" s="8" t="inlineStr">
+      <c r="Z132" s="8" t="inlineStr"/>
+      <c r="AA132" s="8" t="inlineStr"/>
+      <c r="AB132" s="8" t="inlineStr"/>
+      <c r="AC132" s="8" t="inlineStr">
         <is>
           <t>545.00</t>
         </is>
       </c>
-      <c r="AA132" s="8" t="inlineStr"/>
-      <c r="AB132" s="10" t="n">
+      <c r="AD132" s="8" t="inlineStr"/>
+      <c r="AE132" s="10" t="n">
         <v>505.3333333333333</v>
       </c>
-      <c r="AC132" s="10" t="n">
+      <c r="AF132" s="10" t="n">
         <v>44.66666666666663</v>
       </c>
-      <c r="AD132" s="12" t="n">
+      <c r="AG132" s="12" t="n">
         <v>0.001063839077667397</v>
       </c>
     </row>
@@ -8437,15 +9115,18 @@
       <c r="W133" s="8" t="inlineStr"/>
       <c r="X133" s="8" t="inlineStr"/>
       <c r="Y133" s="8" t="inlineStr"/>
-      <c r="Z133" s="8" t="inlineStr">
+      <c r="Z133" s="8" t="inlineStr"/>
+      <c r="AA133" s="8" t="inlineStr"/>
+      <c r="AB133" s="8" t="inlineStr"/>
+      <c r="AC133" s="8" t="inlineStr">
         <is>
           <t>411.00</t>
         </is>
       </c>
-      <c r="AA133" s="8" t="inlineStr"/>
-      <c r="AB133" s="10" t="inlineStr"/>
-      <c r="AC133" s="11" t="inlineStr"/>
-      <c r="AD133" s="12" t="inlineStr"/>
+      <c r="AD133" s="8" t="inlineStr"/>
+      <c r="AE133" s="10" t="inlineStr"/>
+      <c r="AF133" s="11" t="inlineStr"/>
+      <c r="AG133" s="12" t="inlineStr"/>
     </row>
     <row r="134" ht="24" customHeight="1">
       <c r="A134" s="1" t="n"/>
@@ -8477,15 +9158,18 @@
       <c r="W134" s="8" t="inlineStr"/>
       <c r="X134" s="8" t="inlineStr"/>
       <c r="Y134" s="8" t="inlineStr"/>
-      <c r="Z134" s="8" t="inlineStr">
+      <c r="Z134" s="8" t="inlineStr"/>
+      <c r="AA134" s="8" t="inlineStr"/>
+      <c r="AB134" s="8" t="inlineStr"/>
+      <c r="AC134" s="8" t="inlineStr">
         <is>
           <t>415.00</t>
         </is>
       </c>
-      <c r="AA134" s="8" t="inlineStr"/>
-      <c r="AB134" s="10" t="inlineStr"/>
-      <c r="AC134" s="11" t="inlineStr"/>
-      <c r="AD134" s="12" t="inlineStr"/>
+      <c r="AD134" s="8" t="inlineStr"/>
+      <c r="AE134" s="10" t="inlineStr"/>
+      <c r="AF134" s="11" t="inlineStr"/>
+      <c r="AG134" s="12" t="inlineStr"/>
     </row>
     <row r="135" ht="24" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
@@ -8525,11 +9209,14 @@
       <c r="Y135" s="4" t="inlineStr"/>
       <c r="Z135" s="4" t="inlineStr"/>
       <c r="AA135" s="4" t="inlineStr"/>
-      <c r="AB135" s="5" t="inlineStr"/>
-      <c r="AC135" s="6" t="n">
+      <c r="AB135" s="4" t="inlineStr"/>
+      <c r="AC135" s="4" t="inlineStr"/>
+      <c r="AD135" s="4" t="inlineStr"/>
+      <c r="AE135" s="5" t="inlineStr"/>
+      <c r="AF135" s="6" t="n">
         <v>-2053.75</v>
       </c>
-      <c r="AD135" s="7" t="n">
+      <c r="AG135" s="7" t="n">
         <v>-0.1840310758257316</v>
       </c>
     </row>
@@ -8585,11 +9272,14 @@
       <c r="Y136" s="8" t="inlineStr"/>
       <c r="Z136" s="8" t="inlineStr"/>
       <c r="AA136" s="8" t="inlineStr"/>
-      <c r="AB136" s="10" t="n">
+      <c r="AB136" s="8" t="inlineStr"/>
+      <c r="AC136" s="8" t="inlineStr"/>
+      <c r="AD136" s="8" t="inlineStr"/>
+      <c r="AE136" s="10" t="n">
         <v>5931.25</v>
       </c>
-      <c r="AC136" s="11" t="inlineStr"/>
-      <c r="AD136" s="12" t="inlineStr"/>
+      <c r="AF136" s="11" t="inlineStr"/>
+      <c r="AG136" s="12" t="inlineStr"/>
     </row>
     <row r="137" ht="24" customHeight="1">
       <c r="A137" s="1" t="n"/>
@@ -8635,9 +9325,12 @@
       <c r="Y137" s="8" t="inlineStr"/>
       <c r="Z137" s="8" t="inlineStr"/>
       <c r="AA137" s="8" t="inlineStr"/>
-      <c r="AB137" s="10" t="inlineStr"/>
-      <c r="AC137" s="11" t="inlineStr"/>
-      <c r="AD137" s="12" t="inlineStr"/>
+      <c r="AB137" s="8" t="inlineStr"/>
+      <c r="AC137" s="8" t="inlineStr"/>
+      <c r="AD137" s="8" t="inlineStr"/>
+      <c r="AE137" s="10" t="inlineStr"/>
+      <c r="AF137" s="11" t="inlineStr"/>
+      <c r="AG137" s="12" t="inlineStr"/>
     </row>
     <row r="138" ht="24" customHeight="1">
       <c r="A138" s="1" t="n"/>
@@ -8673,7 +9366,7 @@
           <t>2974.50</t>
         </is>
       </c>
-      <c r="R138" s="15" t="inlineStr">
+      <c r="R138" s="16" t="inlineStr">
         <is>
           <t>7972.50</t>
         </is>
@@ -8685,19 +9378,22 @@
       <c r="W138" s="8" t="inlineStr"/>
       <c r="X138" s="8" t="inlineStr"/>
       <c r="Y138" s="8" t="inlineStr"/>
-      <c r="Z138" s="14" t="inlineStr">
+      <c r="Z138" s="8" t="inlineStr"/>
+      <c r="AA138" s="8" t="inlineStr"/>
+      <c r="AB138" s="8" t="inlineStr"/>
+      <c r="AC138" s="15" t="inlineStr">
         <is>
           <t>RUNNING</t>
         </is>
       </c>
-      <c r="AA138" s="8" t="inlineStr"/>
-      <c r="AB138" s="10" t="n">
+      <c r="AD138" s="8" t="inlineStr"/>
+      <c r="AE138" s="10" t="n">
         <v>6350.5</v>
       </c>
-      <c r="AC138" s="10" t="n">
+      <c r="AF138" s="10" t="n">
         <v>419.25</v>
       </c>
-      <c r="AD138" s="12" t="n">
+      <c r="AG138" s="12" t="n">
         <v>0.03756787756052975</v>
       </c>
     </row>

</xml_diff>